<commit_message>
Full engine run with C1 period-coverage guarantee: 759 clashes (88.4%)
C1 adds coverage scoring for grad-req courses with 6+ sections in
greedy_assign_periods(). Results: 759 vs 752 clashes (+7), theology
clashes 197 vs 199 (-2), grad-req fulfillment 88.1% vs 88.5% (-0.4%).
Tighter Phase D convergence (spread=12 vs 30) but slightly worse optimum.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -6780,7 +6780,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10776,7 +10776,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11516,7 +11516,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11960,7 +11960,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12108,7 +12108,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12404,7 +12404,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13070,7 +13070,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13292,7 +13292,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13366,7 +13366,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14402,7 +14402,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14476,7 +14476,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15290,7 +15290,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15734,7 +15734,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15882,7 +15882,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16252,7 +16252,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16548,7 +16548,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16992,7 +16992,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17066,7 +17066,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17140,7 +17140,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17288,7 +17288,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17732,7 +17732,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18028,7 +18028,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18250,7 +18250,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18398,7 +18398,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18472,7 +18472,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18990,7 +18990,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19286,7 +19286,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19508,7 +19508,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19804,7 +19804,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19952,7 +19952,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20100,7 +20100,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20174,7 +20174,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20470,7 +20470,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20840,7 +20840,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20988,7 +20988,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21284,7 +21284,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21358,7 +21358,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21432,7 +21432,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21506,7 +21506,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21802,7 +21802,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22024,7 +22024,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22394,7 +22394,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22912,7 +22912,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22986,7 +22986,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23208,7 +23208,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23356,7 +23356,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23800,7 +23800,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23874,7 +23874,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23948,7 +23948,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24022,7 +24022,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24170,7 +24170,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24318,7 +24318,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24392,7 +24392,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24614,7 +24614,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24688,7 +24688,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24836,7 +24836,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24910,7 +24910,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr">
@@ -25280,7 +25280,7 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J337" s="2" t="inlineStr">
@@ -25502,7 +25502,7 @@
       </c>
       <c r="I338" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J338" s="2" t="inlineStr">
@@ -25650,7 +25650,7 @@
       </c>
       <c r="I340" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J340" s="2" t="inlineStr">
@@ -25724,7 +25724,7 @@
       </c>
       <c r="I341" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J341" s="2" t="inlineStr">
@@ -25798,7 +25798,7 @@
       </c>
       <c r="I342" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J342" s="2" t="inlineStr">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J343" s="2" t="inlineStr">
@@ -25946,7 +25946,7 @@
       </c>
       <c r="I344" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J344" s="2" t="inlineStr">
@@ -26020,7 +26020,7 @@
       </c>
       <c r="I345" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J345" s="2" t="inlineStr">
@@ -26094,7 +26094,7 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
@@ -26168,7 +26168,7 @@
       </c>
       <c r="I347" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J347" s="2" t="inlineStr">
@@ -26242,7 +26242,7 @@
       </c>
       <c r="I348" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J348" s="2" t="inlineStr">
@@ -28115,10 +28115,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
@@ -28131,13 +28131,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -28147,16 +28147,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>40</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
@@ -28166,16 +28166,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -28191,10 +28191,10 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -28204,16 +28204,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>12</v>
-      </c>
       <c r="D7" s="3" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -28223,16 +28223,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -30829,7 +30829,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -30839,7 +30839,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>310-5</t>
+          <t>310-2</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -30861,7 +30861,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -30871,7 +30871,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>310-5</t>
+          <t>310-2</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -30893,7 +30893,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -31013,7 +31013,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>149/348</t>
+          <t>154/348</t>
         </is>
       </c>
     </row>
@@ -31036,7 +31036,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -31046,7 +31046,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
@@ -31056,7 +31056,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14">
@@ -31066,7 +31066,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15">
@@ -31076,7 +31076,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16">
@@ -31086,7 +31086,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
@@ -31096,7 +31096,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Interim engine outputs from tuned C1 run (in progress)
Job1 section placements and priority audit log from Phase A of the
currently running full engine with tuned C1 weights (-20/+10).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -6928,7 +6928,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10776,7 +10776,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11516,7 +11516,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11960,7 +11960,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12108,7 +12108,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12404,7 +12404,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13070,7 +13070,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13292,7 +13292,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13366,7 +13366,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14402,7 +14402,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14476,7 +14476,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15290,7 +15290,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15734,7 +15734,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15882,7 +15882,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16252,7 +16252,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16548,7 +16548,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16992,7 +16992,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17066,7 +17066,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17140,7 +17140,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17288,7 +17288,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17732,7 +17732,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18028,7 +18028,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18250,7 +18250,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18398,7 +18398,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18472,7 +18472,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18990,7 +18990,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19286,7 +19286,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19508,7 +19508,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19804,7 +19804,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19952,7 +19952,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20100,7 +20100,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20174,7 +20174,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20470,7 +20470,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20840,7 +20840,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20988,7 +20988,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21284,7 +21284,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21358,7 +21358,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21432,7 +21432,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21506,7 +21506,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21802,7 +21802,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22024,7 +22024,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22394,7 +22394,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22912,7 +22912,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22986,7 +22986,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23208,7 +23208,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23356,7 +23356,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23800,7 +23800,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23874,7 +23874,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23948,7 +23948,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24022,7 +24022,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24170,7 +24170,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24318,7 +24318,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24392,7 +24392,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24614,7 +24614,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24688,7 +24688,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24836,7 +24836,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24910,7 +24910,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr">
@@ -25280,7 +25280,7 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J337" s="2" t="inlineStr">
@@ -25502,7 +25502,7 @@
       </c>
       <c r="I338" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J338" s="2" t="inlineStr">
@@ -25650,7 +25650,7 @@
       </c>
       <c r="I340" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J340" s="2" t="inlineStr">
@@ -25724,7 +25724,7 @@
       </c>
       <c r="I341" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J341" s="2" t="inlineStr">
@@ -25798,7 +25798,7 @@
       </c>
       <c r="I342" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J342" s="2" t="inlineStr">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J343" s="2" t="inlineStr">
@@ -25946,7 +25946,7 @@
       </c>
       <c r="I344" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J344" s="2" t="inlineStr">
@@ -26020,7 +26020,7 @@
       </c>
       <c r="I345" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J345" s="2" t="inlineStr">
@@ -26094,7 +26094,7 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
@@ -26168,7 +26168,7 @@
       </c>
       <c r="I347" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J347" s="2" t="inlineStr">
@@ -26242,7 +26242,7 @@
       </c>
       <c r="I348" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J348" s="2" t="inlineStr">
@@ -28115,10 +28115,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -28131,13 +28131,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -28147,16 +28147,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>40</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5">
@@ -28166,16 +28166,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -28191,10 +28191,10 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -28204,16 +28204,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -28223,16 +28223,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -30829,7 +30829,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -30839,7 +30839,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>310-2</t>
+          <t>310-5</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -30861,7 +30861,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -30871,7 +30871,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>310-2</t>
+          <t>310-5</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -30893,7 +30893,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -31013,7 +31013,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>154/348</t>
+          <t>149/348</t>
         </is>
       </c>
     </row>
@@ -31036,7 +31036,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -31046,7 +31046,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13">
@@ -31056,7 +31056,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14">
@@ -31066,7 +31066,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15">
@@ -31076,7 +31076,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
@@ -31086,7 +31086,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -31096,7 +31096,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unlimited seat mode run: 713 clashes (89.1%), 29 sections over cap
Unlimited mode removes all section caps to show natural demand.
713 clashes remain even with unlimited seats — pure period conflicts.
29 sections need splitting (over original cap), 117 low/no demand.
Capacity limits only account for 43 of 756 total clashes.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -660,7 +660,7 @@
         <v>3775</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S2" s="3" t="inlineStr"/>
       <c r="T2" s="3" t="inlineStr">
@@ -738,7 +738,7 @@
         <v>3795</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S3" s="3" t="inlineStr"/>
       <c r="T3" s="3" t="inlineStr">
@@ -816,7 +816,7 @@
         <v>3680</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S4" s="3" t="inlineStr"/>
       <c r="T4" s="3" t="inlineStr"/>
@@ -890,7 +890,7 @@
         <v>3700</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S5" s="3" t="inlineStr"/>
       <c r="T5" s="3" t="inlineStr"/>
@@ -964,7 +964,7 @@
         <v>3660</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S6" s="3" t="inlineStr"/>
       <c r="T6" s="3" t="inlineStr"/>
@@ -1038,7 +1038,7 @@
         <v>3680</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S7" s="3" t="inlineStr"/>
       <c r="T7" s="3" t="inlineStr"/>
@@ -1112,7 +1112,7 @@
         <v>3700</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S8" s="3" t="inlineStr"/>
       <c r="T8" s="3" t="inlineStr"/>
@@ -1186,7 +1186,7 @@
         <v>3720</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S9" s="3" t="inlineStr"/>
       <c r="T9" s="3" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
         <v>3740</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S10" s="3" t="inlineStr"/>
       <c r="T10" s="3" t="inlineStr"/>
@@ -1334,7 +1334,7 @@
         <v>3760</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S11" s="3" t="inlineStr"/>
       <c r="T11" s="3" t="inlineStr"/>
@@ -1408,7 +1408,7 @@
         <v>3780</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S12" s="3" t="inlineStr"/>
       <c r="T12" s="3" t="inlineStr"/>
@@ -1482,7 +1482,7 @@
         <v>3800</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S13" s="3" t="inlineStr"/>
       <c r="T13" s="3" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
         <v>3550</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S14" s="3" t="inlineStr"/>
       <c r="T14" s="3" t="inlineStr"/>
@@ -1630,7 +1630,7 @@
         <v>3550</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S15" s="3" t="inlineStr"/>
       <c r="T15" s="3" t="inlineStr"/>
@@ -1704,7 +1704,7 @@
         <v>3525</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S16" s="3" t="inlineStr"/>
       <c r="T16" s="3" t="inlineStr"/>
@@ -1778,7 +1778,7 @@
         <v>3545</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S17" s="3" t="inlineStr"/>
       <c r="T17" s="3" t="inlineStr"/>
@@ -1852,7 +1852,7 @@
         <v>1725</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S18" s="3" t="inlineStr"/>
       <c r="T18" s="3" t="inlineStr"/>
@@ -1926,7 +1926,7 @@
         <v>1715</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S19" s="3" t="inlineStr"/>
       <c r="T19" s="3" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
         <v>1725</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S20" s="3" t="inlineStr"/>
       <c r="T20" s="3" t="inlineStr"/>
@@ -2074,7 +2074,7 @@
         <v>1735</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S21" s="3" t="inlineStr"/>
       <c r="T21" s="3" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
         <v>1745</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
       <c r="T22" s="3" t="inlineStr"/>
@@ -2222,7 +2222,7 @@
         <v>1695</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S23" s="3" t="inlineStr"/>
       <c r="T23" s="3" t="inlineStr"/>
@@ -2296,7 +2296,7 @@
         <v>1705</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S24" s="3" t="inlineStr"/>
       <c r="T24" s="3" t="inlineStr"/>
@@ -2370,7 +2370,7 @@
         <v>1715</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S25" s="3" t="inlineStr"/>
       <c r="T25" s="3" t="inlineStr"/>
@@ -2444,7 +2444,7 @@
         <v>1725</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S26" s="3" t="inlineStr"/>
       <c r="T26" s="3" t="inlineStr"/>
@@ -2518,7 +2518,7 @@
         <v>1735</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S27" s="3" t="inlineStr"/>
       <c r="T27" s="3" t="inlineStr"/>
@@ -2592,7 +2592,7 @@
         <v>1745</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S28" s="3" t="inlineStr"/>
       <c r="T28" s="3" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
         <v>1755</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S29" s="3" t="inlineStr"/>
       <c r="T29" s="3" t="inlineStr"/>
@@ -2740,7 +2740,7 @@
         <v>1765</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S30" s="3" t="inlineStr"/>
       <c r="T30" s="3" t="inlineStr"/>
@@ -2814,7 +2814,7 @@
         <v>3630</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S31" s="3" t="inlineStr"/>
       <c r="T31" s="3" t="inlineStr"/>
@@ -2888,7 +2888,7 @@
         <v>3480</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S32" s="3" t="inlineStr"/>
       <c r="T32" s="3" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
         <v>3175</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S33" s="3" t="inlineStr"/>
       <c r="T33" s="3" t="inlineStr"/>
@@ -3036,7 +3036,7 @@
         <v>3195</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S34" s="3" t="inlineStr"/>
       <c r="T34" s="3" t="inlineStr"/>
@@ -3110,7 +3110,7 @@
         <v>3445</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S35" s="3" t="inlineStr"/>
       <c r="T35" s="3" t="inlineStr"/>
@@ -3184,7 +3184,7 @@
         <v>3465</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S36" s="3" t="inlineStr"/>
       <c r="T36" s="3" t="inlineStr"/>
@@ -3258,7 +3258,7 @@
         <v>3135</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S37" s="3" t="inlineStr"/>
       <c r="T37" s="3" t="inlineStr"/>
@@ -3332,7 +3332,7 @@
         <v>3155</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S38" s="3" t="inlineStr"/>
       <c r="T38" s="3" t="inlineStr"/>
@@ -3406,7 +3406,7 @@
         <v>3175</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S39" s="3" t="inlineStr"/>
       <c r="T39" s="3" t="inlineStr"/>
@@ -3480,7 +3480,7 @@
         <v>1560</v>
       </c>
       <c r="R40" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S40" s="3" t="inlineStr"/>
       <c r="T40" s="3" t="inlineStr"/>
@@ -3554,7 +3554,7 @@
         <v>1570</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S41" s="3" t="inlineStr"/>
       <c r="T41" s="3" t="inlineStr"/>
@@ -3628,7 +3628,7 @@
         <v>1580</v>
       </c>
       <c r="R42" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S42" s="3" t="inlineStr"/>
       <c r="T42" s="3" t="inlineStr"/>
@@ -3702,7 +3702,7 @@
         <v>3575</v>
       </c>
       <c r="R43" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S43" s="3" t="inlineStr"/>
       <c r="T43" s="3" t="inlineStr"/>
@@ -3776,7 +3776,7 @@
         <v>3595</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S44" s="3" t="inlineStr"/>
       <c r="T44" s="3" t="inlineStr"/>
@@ -3850,7 +3850,7 @@
         <v>3615</v>
       </c>
       <c r="R45" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S45" s="3" t="inlineStr"/>
       <c r="T45" s="3" t="inlineStr"/>
@@ -3924,7 +3924,7 @@
         <v>3110</v>
       </c>
       <c r="R46" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S46" s="3" t="inlineStr"/>
       <c r="T46" s="3" t="inlineStr"/>
@@ -3998,7 +3998,7 @@
         <v>3120</v>
       </c>
       <c r="R47" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S47" s="3" t="inlineStr"/>
       <c r="T47" s="3" t="inlineStr"/>
@@ -4072,7 +4072,7 @@
         <v>3100</v>
       </c>
       <c r="R48" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S48" s="3" t="inlineStr"/>
       <c r="T48" s="3" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
         <v>3120</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S49" s="3" t="inlineStr"/>
       <c r="T49" s="3" t="inlineStr"/>
@@ -4220,7 +4220,7 @@
         <v>3085</v>
       </c>
       <c r="R50" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S50" s="3" t="inlineStr"/>
       <c r="T50" s="3" t="inlineStr"/>
@@ -4294,7 +4294,7 @@
         <v>3105</v>
       </c>
       <c r="R51" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S51" s="3" t="inlineStr"/>
       <c r="T51" s="3" t="inlineStr"/>
@@ -4368,7 +4368,7 @@
         <v>3130</v>
       </c>
       <c r="R52" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S52" s="3" t="inlineStr"/>
       <c r="T52" s="3" t="inlineStr"/>
@@ -4442,7 +4442,7 @@
         <v>3025</v>
       </c>
       <c r="R53" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S53" s="3" t="inlineStr"/>
       <c r="T53" s="3" t="inlineStr"/>
@@ -4516,7 +4516,7 @@
         <v>3045</v>
       </c>
       <c r="R54" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S54" s="3" t="inlineStr"/>
       <c r="T54" s="3" t="inlineStr"/>
@@ -4590,7 +4590,7 @@
         <v>3275</v>
       </c>
       <c r="R55" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S55" s="3" t="inlineStr"/>
       <c r="T55" s="3" t="inlineStr"/>
@@ -4664,7 +4664,7 @@
         <v>3295</v>
       </c>
       <c r="R56" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S56" s="3" t="inlineStr"/>
       <c r="T56" s="3" t="inlineStr"/>
@@ -4738,7 +4738,7 @@
         <v>3315</v>
       </c>
       <c r="R57" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S57" s="3" t="inlineStr"/>
       <c r="T57" s="3" t="inlineStr"/>
@@ -4812,7 +4812,7 @@
         <v>3335</v>
       </c>
       <c r="R58" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S58" s="3" t="inlineStr"/>
       <c r="T58" s="3" t="inlineStr"/>
@@ -4886,7 +4886,7 @@
         <v>3355</v>
       </c>
       <c r="R59" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S59" s="3" t="inlineStr"/>
       <c r="T59" s="3" t="inlineStr"/>
@@ -4960,7 +4960,7 @@
         <v>3375</v>
       </c>
       <c r="R60" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S60" s="3" t="inlineStr"/>
       <c r="T60" s="3" t="inlineStr"/>
@@ -5034,7 +5034,7 @@
         <v>2975</v>
       </c>
       <c r="R61" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S61" s="3" t="inlineStr"/>
       <c r="T61" s="3" t="inlineStr"/>
@@ -5108,7 +5108,7 @@
         <v>2995</v>
       </c>
       <c r="R62" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S62" s="3" t="inlineStr"/>
       <c r="T62" s="3" t="inlineStr"/>
@@ -5182,7 +5182,7 @@
         <v>2950</v>
       </c>
       <c r="R63" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S63" s="3" t="inlineStr"/>
       <c r="T63" s="3" t="inlineStr"/>
@@ -5256,7 +5256,7 @@
         <v>2905</v>
       </c>
       <c r="R64" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S64" s="3" t="inlineStr"/>
       <c r="T64" s="3" t="inlineStr"/>
@@ -5330,7 +5330,7 @@
         <v>2855</v>
       </c>
       <c r="R65" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S65" s="3" t="inlineStr"/>
       <c r="T65" s="3" t="inlineStr"/>
@@ -5404,7 +5404,7 @@
         <v>2875</v>
       </c>
       <c r="R66" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S66" s="3" t="inlineStr"/>
       <c r="T66" s="3" t="inlineStr"/>
@@ -5478,7 +5478,7 @@
         <v>2895</v>
       </c>
       <c r="R67" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S67" s="3" t="inlineStr"/>
       <c r="T67" s="3" t="inlineStr"/>
@@ -5552,7 +5552,7 @@
         <v>2855</v>
       </c>
       <c r="R68" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S68" s="3" t="inlineStr"/>
       <c r="T68" s="3" t="inlineStr"/>
@@ -5626,7 +5626,7 @@
         <v>2875</v>
       </c>
       <c r="R69" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S69" s="3" t="inlineStr"/>
       <c r="T69" s="3" t="inlineStr"/>
@@ -5700,7 +5700,7 @@
         <v>3070</v>
       </c>
       <c r="R70" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S70" s="3" t="inlineStr"/>
       <c r="T70" s="3" t="inlineStr"/>
@@ -5774,7 +5774,7 @@
         <v>2985</v>
       </c>
       <c r="R71" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S71" s="3" t="inlineStr"/>
       <c r="T71" s="3" t="inlineStr"/>
@@ -5848,7 +5848,7 @@
         <v>3005</v>
       </c>
       <c r="R72" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S72" s="3" t="inlineStr"/>
       <c r="T72" s="3" t="inlineStr"/>
@@ -5922,7 +5922,7 @@
         <v>1310</v>
       </c>
       <c r="R73" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S73" s="3" t="inlineStr"/>
       <c r="T73" s="3" t="inlineStr"/>
@@ -5996,7 +5996,7 @@
         <v>1320</v>
       </c>
       <c r="R74" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S74" s="3" t="inlineStr"/>
       <c r="T74" s="3" t="inlineStr"/>
@@ -6070,7 +6070,7 @@
         <v>2635</v>
       </c>
       <c r="R75" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S75" s="3" t="inlineStr"/>
       <c r="T75" s="3" t="inlineStr"/>
@@ -6144,7 +6144,7 @@
         <v>2635</v>
       </c>
       <c r="R76" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S76" s="3" t="inlineStr"/>
       <c r="T76" s="3" t="inlineStr"/>
@@ -6218,7 +6218,7 @@
         <v>2655</v>
       </c>
       <c r="R77" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S77" s="3" t="inlineStr"/>
       <c r="T77" s="3" t="inlineStr"/>
@@ -6292,7 +6292,7 @@
         <v>2630</v>
       </c>
       <c r="R78" s="3" t="n">
-        <v>40</v>
+        <v>9999</v>
       </c>
       <c r="S78" s="3" t="inlineStr"/>
       <c r="T78" s="3" t="inlineStr"/>
@@ -6366,7 +6366,7 @@
         <v>2770</v>
       </c>
       <c r="R79" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S79" s="3" t="inlineStr"/>
       <c r="T79" s="3" t="inlineStr"/>
@@ -6440,7 +6440,7 @@
         <v>2790</v>
       </c>
       <c r="R80" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S80" s="3" t="inlineStr"/>
       <c r="T80" s="3" t="inlineStr"/>
@@ -6514,7 +6514,7 @@
         <v>2560</v>
       </c>
       <c r="R81" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S81" s="3" t="inlineStr"/>
       <c r="T81" s="3" t="inlineStr"/>
@@ -6588,7 +6588,7 @@
         <v>2580</v>
       </c>
       <c r="R82" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S82" s="3" t="inlineStr"/>
       <c r="T82" s="3" t="inlineStr"/>
@@ -6662,7 +6662,7 @@
         <v>2520</v>
       </c>
       <c r="R83" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S83" s="3" t="inlineStr"/>
       <c r="T83" s="3" t="inlineStr"/>
@@ -6736,7 +6736,7 @@
         <v>3235</v>
       </c>
       <c r="R84" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S84" s="3" t="inlineStr"/>
       <c r="T84" s="3" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
         <v>3255</v>
       </c>
       <c r="R85" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S85" s="3" t="inlineStr"/>
       <c r="T85" s="3" t="inlineStr"/>
@@ -6884,7 +6884,7 @@
         <v>3275</v>
       </c>
       <c r="R86" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S86" s="3" t="inlineStr"/>
       <c r="T86" s="3" t="inlineStr"/>
@@ -6958,7 +6958,7 @@
         <v>3295</v>
       </c>
       <c r="R87" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S87" s="3" t="inlineStr"/>
       <c r="T87" s="3" t="inlineStr"/>
@@ -7032,7 +7032,7 @@
         <v>1235</v>
       </c>
       <c r="R88" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S88" s="3" t="inlineStr"/>
       <c r="T88" s="3" t="inlineStr"/>
@@ -7106,7 +7106,7 @@
         <v>1245</v>
       </c>
       <c r="R89" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S89" s="3" t="inlineStr"/>
       <c r="T89" s="3" t="inlineStr"/>
@@ -7180,7 +7180,7 @@
         <v>1255</v>
       </c>
       <c r="R90" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S90" s="3" t="inlineStr"/>
       <c r="T90" s="3" t="inlineStr"/>
@@ -7254,7 +7254,7 @@
         <v>2600</v>
       </c>
       <c r="R91" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S91" s="3" t="inlineStr"/>
       <c r="T91" s="3" t="inlineStr"/>
@@ -7328,7 +7328,7 @@
         <v>2595</v>
       </c>
       <c r="R92" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S92" s="3" t="inlineStr"/>
       <c r="T92" s="3" t="inlineStr"/>
@@ -7402,7 +7402,7 @@
         <v>2615</v>
       </c>
       <c r="R93" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S93" s="3" t="inlineStr"/>
       <c r="T93" s="3" t="inlineStr"/>
@@ -7476,7 +7476,7 @@
         <v>3015</v>
       </c>
       <c r="R94" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S94" s="3" t="inlineStr"/>
       <c r="T94" s="3" t="inlineStr"/>
@@ -7550,7 +7550,7 @@
         <v>3035</v>
       </c>
       <c r="R95" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S95" s="3" t="inlineStr"/>
       <c r="T95" s="3" t="inlineStr"/>
@@ -7624,7 +7624,7 @@
         <v>2790</v>
       </c>
       <c r="R96" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S96" s="3" t="inlineStr"/>
       <c r="T96" s="3" t="inlineStr"/>
@@ -7698,7 +7698,7 @@
         <v>2810</v>
       </c>
       <c r="R97" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S97" s="3" t="inlineStr"/>
       <c r="T97" s="3" t="inlineStr"/>
@@ -7772,7 +7772,7 @@
         <v>2460</v>
       </c>
       <c r="R98" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S98" s="3" t="inlineStr"/>
       <c r="T98" s="3" t="inlineStr"/>
@@ -7846,7 +7846,7 @@
         <v>2995</v>
       </c>
       <c r="R99" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S99" s="3" t="inlineStr"/>
       <c r="T99" s="3" t="inlineStr"/>
@@ -7920,7 +7920,7 @@
         <v>3015</v>
       </c>
       <c r="R100" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S100" s="3" t="inlineStr"/>
       <c r="T100" s="3" t="inlineStr"/>
@@ -7994,7 +7994,7 @@
         <v>3470</v>
       </c>
       <c r="R101" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S101" s="3" t="inlineStr"/>
       <c r="T101" s="3" t="inlineStr"/>
@@ -8068,7 +8068,7 @@
         <v>3490</v>
       </c>
       <c r="R102" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S102" s="3" t="inlineStr"/>
       <c r="T102" s="3" t="inlineStr"/>
@@ -8142,7 +8142,7 @@
         <v>3510</v>
       </c>
       <c r="R103" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S103" s="3" t="inlineStr"/>
       <c r="T103" s="3" t="inlineStr"/>
@@ -8216,7 +8216,7 @@
         <v>3040</v>
       </c>
       <c r="R104" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S104" s="3" t="inlineStr"/>
       <c r="T104" s="3" t="inlineStr"/>
@@ -8290,7 +8290,7 @@
         <v>3455</v>
       </c>
       <c r="R105" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S105" s="3" t="inlineStr"/>
       <c r="T105" s="3" t="inlineStr"/>
@@ -8364,7 +8364,7 @@
         <v>3045</v>
       </c>
       <c r="R106" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S106" s="3" t="inlineStr"/>
       <c r="T106" s="3" t="inlineStr"/>
@@ -8438,7 +8438,7 @@
         <v>3055</v>
       </c>
       <c r="R107" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S107" s="3" t="inlineStr"/>
       <c r="T107" s="3" t="inlineStr"/>
@@ -8512,7 +8512,7 @@
         <v>1270</v>
       </c>
       <c r="R108" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S108" s="3" t="inlineStr"/>
       <c r="T108" s="3" t="inlineStr"/>
@@ -8586,7 +8586,7 @@
         <v>2375</v>
       </c>
       <c r="R109" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S109" s="3" t="inlineStr"/>
       <c r="T109" s="3" t="inlineStr"/>
@@ -8660,7 +8660,7 @@
         <v>2395</v>
       </c>
       <c r="R110" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S110" s="3" t="inlineStr"/>
       <c r="T110" s="3" t="inlineStr"/>
@@ -8734,7 +8734,7 @@
         <v>2430</v>
       </c>
       <c r="R111" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S111" s="3" t="inlineStr"/>
       <c r="T111" s="3" t="inlineStr"/>
@@ -8808,7 +8808,7 @@
         <v>2450</v>
       </c>
       <c r="R112" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S112" s="3" t="inlineStr"/>
       <c r="T112" s="3" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
         <v>2470</v>
       </c>
       <c r="R113" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S113" s="3" t="inlineStr"/>
       <c r="T113" s="3" t="inlineStr"/>
@@ -8956,7 +8956,7 @@
         <v>3010</v>
       </c>
       <c r="R114" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S114" s="3" t="inlineStr"/>
       <c r="T114" s="3" t="inlineStr"/>
@@ -9030,7 +9030,7 @@
         <v>3030</v>
       </c>
       <c r="R115" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S115" s="3" t="inlineStr"/>
       <c r="T115" s="3" t="inlineStr"/>
@@ -9104,7 +9104,7 @@
         <v>1160</v>
       </c>
       <c r="R116" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S116" s="3" t="inlineStr"/>
       <c r="T116" s="3" t="inlineStr"/>
@@ -9178,7 +9178,7 @@
         <v>2545</v>
       </c>
       <c r="R117" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S117" s="3" t="inlineStr"/>
       <c r="T117" s="3" t="inlineStr"/>
@@ -9252,7 +9252,7 @@
         <v>1135</v>
       </c>
       <c r="R118" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S118" s="3" t="inlineStr"/>
       <c r="T118" s="3" t="inlineStr"/>
@@ -9326,7 +9326,7 @@
         <v>1145</v>
       </c>
       <c r="R119" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S119" s="3" t="inlineStr"/>
       <c r="T119" s="3" t="inlineStr"/>
@@ -9400,7 +9400,7 @@
         <v>1155</v>
       </c>
       <c r="R120" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S120" s="3" t="inlineStr"/>
       <c r="T120" s="3" t="inlineStr"/>
@@ -9474,7 +9474,7 @@
         <v>1165</v>
       </c>
       <c r="R121" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S121" s="3" t="inlineStr"/>
       <c r="T121" s="3" t="inlineStr"/>
@@ -9548,7 +9548,7 @@
         <v>1175</v>
       </c>
       <c r="R122" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S122" s="3" t="inlineStr"/>
       <c r="T122" s="3" t="inlineStr"/>
@@ -9622,7 +9622,7 @@
         <v>2980</v>
       </c>
       <c r="R123" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S123" s="3" t="inlineStr"/>
       <c r="T123" s="3" t="inlineStr"/>
@@ -9696,7 +9696,7 @@
         <v>3000</v>
       </c>
       <c r="R124" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S124" s="3" t="inlineStr"/>
       <c r="T124" s="3" t="inlineStr"/>
@@ -9770,7 +9770,7 @@
         <v>2575</v>
       </c>
       <c r="R125" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S125" s="3" t="inlineStr"/>
       <c r="T125" s="3" t="inlineStr"/>
@@ -9844,7 +9844,7 @@
         <v>3220</v>
       </c>
       <c r="R126" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S126" s="3" t="inlineStr"/>
       <c r="T126" s="3" t="inlineStr"/>
@@ -9918,7 +9918,7 @@
         <v>3240</v>
       </c>
       <c r="R127" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S127" s="3" t="inlineStr"/>
       <c r="T127" s="3" t="inlineStr"/>
@@ -9992,7 +9992,7 @@
         <v>1195</v>
       </c>
       <c r="R128" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S128" s="3" t="inlineStr"/>
       <c r="T128" s="3" t="inlineStr"/>
@@ -10066,7 +10066,7 @@
         <v>1210</v>
       </c>
       <c r="R129" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S129" s="3" t="inlineStr"/>
       <c r="T129" s="3" t="inlineStr"/>
@@ -10140,7 +10140,7 @@
         <v>1130</v>
       </c>
       <c r="R130" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S130" s="3" t="inlineStr"/>
       <c r="T130" s="3" t="inlineStr"/>
@@ -10214,7 +10214,7 @@
         <v>1410</v>
       </c>
       <c r="R131" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S131" s="3" t="inlineStr"/>
       <c r="T131" s="3" t="inlineStr"/>
@@ -10288,7 +10288,7 @@
         <v>2165</v>
       </c>
       <c r="R132" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S132" s="3" t="inlineStr"/>
       <c r="T132" s="3" t="inlineStr"/>
@@ -10362,7 +10362,7 @@
         <v>2185</v>
       </c>
       <c r="R133" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S133" s="3" t="inlineStr"/>
       <c r="T133" s="3" t="inlineStr"/>
@@ -10436,7 +10436,7 @@
         <v>2205</v>
       </c>
       <c r="R134" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S134" s="3" t="inlineStr"/>
       <c r="T134" s="3" t="inlineStr"/>
@@ -10510,7 +10510,7 @@
         <v>2165</v>
       </c>
       <c r="R135" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S135" s="3" t="inlineStr"/>
       <c r="T135" s="3" t="inlineStr"/>
@@ -10584,7 +10584,7 @@
         <v>2185</v>
       </c>
       <c r="R136" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S136" s="3" t="inlineStr"/>
       <c r="T136" s="3" t="inlineStr"/>
@@ -10658,7 +10658,7 @@
         <v>2160</v>
       </c>
       <c r="R137" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S137" s="3" t="inlineStr"/>
       <c r="T137" s="3" t="inlineStr"/>
@@ -10732,7 +10732,7 @@
         <v>2800</v>
       </c>
       <c r="R138" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S138" s="3" t="inlineStr"/>
       <c r="T138" s="3" t="inlineStr"/>
@@ -10806,7 +10806,7 @@
         <v>2815</v>
       </c>
       <c r="R139" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S139" s="3" t="inlineStr"/>
       <c r="T139" s="3" t="inlineStr"/>
@@ -10880,7 +10880,7 @@
         <v>2835</v>
       </c>
       <c r="R140" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S140" s="3" t="inlineStr"/>
       <c r="T140" s="3" t="inlineStr"/>
@@ -10954,7 +10954,7 @@
         <v>2855</v>
       </c>
       <c r="R141" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S141" s="3" t="inlineStr"/>
       <c r="T141" s="3" t="inlineStr"/>
@@ -11028,7 +11028,7 @@
         <v>2155</v>
       </c>
       <c r="R142" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S142" s="3" t="inlineStr"/>
       <c r="T142" s="3" t="inlineStr"/>
@@ -11102,7 +11102,7 @@
         <v>2540</v>
       </c>
       <c r="R143" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S143" s="3" t="inlineStr"/>
       <c r="T143" s="3" t="inlineStr"/>
@@ -11176,7 +11176,7 @@
         <v>2560</v>
       </c>
       <c r="R144" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S144" s="3" t="inlineStr"/>
       <c r="T144" s="3" t="inlineStr"/>
@@ -11250,7 +11250,7 @@
         <v>2135</v>
       </c>
       <c r="R145" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S145" s="3" t="inlineStr"/>
       <c r="T145" s="3" t="inlineStr"/>
@@ -11324,7 +11324,7 @@
         <v>2155</v>
       </c>
       <c r="R146" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S146" s="3" t="inlineStr"/>
       <c r="T146" s="3" t="inlineStr"/>
@@ -11398,7 +11398,7 @@
         <v>2135</v>
       </c>
       <c r="R147" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S147" s="3" t="inlineStr"/>
       <c r="T147" s="3" t="inlineStr"/>
@@ -11472,7 +11472,7 @@
         <v>2155</v>
       </c>
       <c r="R148" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S148" s="3" t="inlineStr"/>
       <c r="T148" s="3" t="inlineStr"/>
@@ -11546,7 +11546,7 @@
         <v>2175</v>
       </c>
       <c r="R149" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S149" s="3" t="inlineStr"/>
       <c r="T149" s="3" t="inlineStr"/>
@@ -11620,7 +11620,7 @@
         <v>2195</v>
       </c>
       <c r="R150" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S150" s="3" t="inlineStr"/>
       <c r="T150" s="3" t="inlineStr"/>
@@ -11694,7 +11694,7 @@
         <v>2215</v>
       </c>
       <c r="R151" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S151" s="3" t="inlineStr"/>
       <c r="T151" s="3" t="inlineStr"/>
@@ -11768,7 +11768,7 @@
         <v>2145</v>
       </c>
       <c r="R152" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S152" s="3" t="inlineStr"/>
       <c r="T152" s="3" t="inlineStr"/>
@@ -11842,7 +11842,7 @@
         <v>2165</v>
       </c>
       <c r="R153" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S153" s="3" t="inlineStr"/>
       <c r="T153" s="3" t="inlineStr"/>
@@ -11916,7 +11916,7 @@
         <v>2185</v>
       </c>
       <c r="R154" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S154" s="3" t="inlineStr"/>
       <c r="T154" s="3" t="inlineStr"/>
@@ -11990,7 +11990,7 @@
         <v>2205</v>
       </c>
       <c r="R155" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S155" s="3" t="inlineStr"/>
       <c r="T155" s="3" t="inlineStr"/>
@@ -12064,7 +12064,7 @@
         <v>2175</v>
       </c>
       <c r="R156" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S156" s="3" t="inlineStr"/>
       <c r="T156" s="3" t="inlineStr"/>
@@ -12138,7 +12138,7 @@
         <v>2185</v>
       </c>
       <c r="R157" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S157" s="3" t="inlineStr"/>
       <c r="T157" s="3" t="inlineStr"/>
@@ -12212,7 +12212,7 @@
         <v>2195</v>
       </c>
       <c r="R158" s="3" t="n">
-        <v>15</v>
+        <v>9999</v>
       </c>
       <c r="S158" s="3" t="inlineStr"/>
       <c r="T158" s="3" t="inlineStr"/>
@@ -12286,7 +12286,7 @@
         <v>2985</v>
       </c>
       <c r="R159" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S159" s="3" t="inlineStr"/>
       <c r="T159" s="3" t="inlineStr"/>
@@ -12360,7 +12360,7 @@
         <v>2995</v>
       </c>
       <c r="R160" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S160" s="3" t="inlineStr"/>
       <c r="T160" s="3" t="inlineStr"/>
@@ -12434,7 +12434,7 @@
         <v>3005</v>
       </c>
       <c r="R161" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S161" s="3" t="inlineStr"/>
       <c r="T161" s="3" t="inlineStr"/>
@@ -12508,7 +12508,7 @@
         <v>3015</v>
       </c>
       <c r="R162" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S162" s="3" t="inlineStr"/>
       <c r="T162" s="3" t="inlineStr"/>
@@ -12582,7 +12582,7 @@
         <v>3025</v>
       </c>
       <c r="R163" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S163" s="3" t="inlineStr"/>
       <c r="T163" s="3" t="inlineStr"/>
@@ -12656,7 +12656,7 @@
         <v>3035</v>
       </c>
       <c r="R164" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S164" s="3" t="inlineStr"/>
       <c r="T164" s="3" t="inlineStr"/>
@@ -12730,7 +12730,7 @@
         <v>3045</v>
       </c>
       <c r="R165" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S165" s="3" t="inlineStr"/>
       <c r="T165" s="3" t="inlineStr"/>
@@ -12804,7 +12804,7 @@
         <v>3055</v>
       </c>
       <c r="R166" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S166" s="3" t="inlineStr"/>
       <c r="T166" s="3" t="inlineStr"/>
@@ -12878,7 +12878,7 @@
         <v>2695</v>
       </c>
       <c r="R167" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S167" s="3" t="inlineStr"/>
       <c r="T167" s="3" t="inlineStr"/>
@@ -12952,7 +12952,7 @@
         <v>3200</v>
       </c>
       <c r="R168" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S168" s="3" t="inlineStr"/>
       <c r="T168" s="3" t="inlineStr"/>
@@ -13026,7 +13026,7 @@
         <v>3375</v>
       </c>
       <c r="R169" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S169" s="3" t="inlineStr"/>
       <c r="T169" s="3" t="inlineStr"/>
@@ -13100,7 +13100,7 @@
         <v>3395</v>
       </c>
       <c r="R170" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S170" s="3" t="inlineStr"/>
       <c r="T170" s="3" t="inlineStr"/>
@@ -13174,7 +13174,7 @@
         <v>2950</v>
       </c>
       <c r="R171" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S171" s="3" t="inlineStr"/>
       <c r="T171" s="3" t="inlineStr"/>
@@ -13248,7 +13248,7 @@
         <v>2970</v>
       </c>
       <c r="R172" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S172" s="3" t="inlineStr"/>
       <c r="T172" s="3" t="inlineStr"/>
@@ -13322,7 +13322,7 @@
         <v>2990</v>
       </c>
       <c r="R173" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S173" s="3" t="inlineStr"/>
       <c r="T173" s="3" t="inlineStr"/>
@@ -13396,7 +13396,7 @@
         <v>3010</v>
       </c>
       <c r="R174" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S174" s="3" t="inlineStr"/>
       <c r="T174" s="3" t="inlineStr"/>
@@ -13470,7 +13470,7 @@
         <v>2665</v>
       </c>
       <c r="R175" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S175" s="3" t="inlineStr"/>
       <c r="T175" s="3" t="inlineStr"/>
@@ -13544,7 +13544,7 @@
         <v>2670</v>
       </c>
       <c r="R176" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S176" s="3" t="inlineStr"/>
       <c r="T176" s="3" t="inlineStr"/>
@@ -13618,7 +13618,7 @@
         <v>3375</v>
       </c>
       <c r="R177" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S177" s="3" t="inlineStr"/>
       <c r="T177" s="3" t="inlineStr"/>
@@ -13692,7 +13692,7 @@
         <v>3395</v>
       </c>
       <c r="R178" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S178" s="3" t="inlineStr"/>
       <c r="T178" s="3" t="inlineStr"/>
@@ -13766,7 +13766,7 @@
         <v>2285</v>
       </c>
       <c r="R179" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S179" s="3" t="inlineStr"/>
       <c r="T179" s="3" t="inlineStr"/>
@@ -13840,7 +13840,7 @@
         <v>2305</v>
       </c>
       <c r="R180" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S180" s="3" t="inlineStr"/>
       <c r="T180" s="3" t="inlineStr"/>
@@ -13914,7 +13914,7 @@
         <v>2325</v>
       </c>
       <c r="R181" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S181" s="3" t="inlineStr"/>
       <c r="T181" s="3" t="inlineStr"/>
@@ -13988,7 +13988,7 @@
         <v>2345</v>
       </c>
       <c r="R182" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S182" s="3" t="inlineStr"/>
       <c r="T182" s="3" t="inlineStr"/>
@@ -14062,7 +14062,7 @@
         <v>2115</v>
       </c>
       <c r="R183" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S183" s="3" t="inlineStr"/>
       <c r="T183" s="3" t="inlineStr"/>
@@ -14136,7 +14136,7 @@
         <v>2135</v>
       </c>
       <c r="R184" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S184" s="3" t="inlineStr"/>
       <c r="T184" s="3" t="inlineStr"/>
@@ -14210,7 +14210,7 @@
         <v>2645</v>
       </c>
       <c r="R185" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S185" s="3" t="inlineStr"/>
       <c r="T185" s="3" t="inlineStr"/>
@@ -14284,7 +14284,7 @@
         <v>2665</v>
       </c>
       <c r="R186" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S186" s="3" t="inlineStr"/>
       <c r="T186" s="3" t="inlineStr"/>
@@ -14358,7 +14358,7 @@
         <v>2095</v>
       </c>
       <c r="R187" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S187" s="3" t="inlineStr"/>
       <c r="T187" s="3" t="inlineStr"/>
@@ -14432,7 +14432,7 @@
         <v>2115</v>
       </c>
       <c r="R188" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S188" s="3" t="inlineStr"/>
       <c r="T188" s="3" t="inlineStr"/>
@@ -14506,7 +14506,7 @@
         <v>2135</v>
       </c>
       <c r="R189" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S189" s="3" t="inlineStr"/>
       <c r="T189" s="3" t="inlineStr"/>
@@ -14580,7 +14580,7 @@
         <v>3115</v>
       </c>
       <c r="R190" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S190" s="3" t="inlineStr"/>
       <c r="T190" s="3" t="inlineStr"/>
@@ -14654,7 +14654,7 @@
         <v>3135</v>
       </c>
       <c r="R191" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S191" s="3" t="inlineStr"/>
       <c r="T191" s="3" t="inlineStr"/>
@@ -14728,7 +14728,7 @@
         <v>3155</v>
       </c>
       <c r="R192" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S192" s="3" t="inlineStr"/>
       <c r="T192" s="3" t="inlineStr"/>
@@ -14802,7 +14802,7 @@
         <v>1845</v>
       </c>
       <c r="R193" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S193" s="3" t="inlineStr"/>
       <c r="T193" s="3" t="inlineStr"/>
@@ -14876,7 +14876,7 @@
         <v>1865</v>
       </c>
       <c r="R194" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S194" s="3" t="inlineStr"/>
       <c r="T194" s="3" t="inlineStr"/>
@@ -14950,7 +14950,7 @@
         <v>3380</v>
       </c>
       <c r="R195" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S195" s="3" t="inlineStr"/>
       <c r="T195" s="3" t="inlineStr"/>
@@ -15024,7 +15024,7 @@
         <v>3400</v>
       </c>
       <c r="R196" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S196" s="3" t="inlineStr"/>
       <c r="T196" s="3" t="inlineStr"/>
@@ -15098,7 +15098,7 @@
         <v>3420</v>
       </c>
       <c r="R197" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S197" s="3" t="inlineStr"/>
       <c r="T197" s="3" t="inlineStr"/>
@@ -15172,7 +15172,7 @@
         <v>2345</v>
       </c>
       <c r="R198" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S198" s="3" t="inlineStr"/>
       <c r="T198" s="3" t="inlineStr"/>
@@ -15246,7 +15246,7 @@
         <v>1815</v>
       </c>
       <c r="R199" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S199" s="3" t="inlineStr"/>
       <c r="T199" s="3" t="inlineStr"/>
@@ -15320,7 +15320,7 @@
         <v>1835</v>
       </c>
       <c r="R200" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S200" s="3" t="inlineStr"/>
       <c r="T200" s="3" t="inlineStr"/>
@@ -15394,7 +15394,7 @@
         <v>1855</v>
       </c>
       <c r="R201" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr"/>
@@ -15468,7 +15468,7 @@
         <v>1875</v>
       </c>
       <c r="R202" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S202" s="3" t="inlineStr"/>
       <c r="T202" s="3" t="inlineStr"/>
@@ -15542,7 +15542,7 @@
         <v>2760</v>
       </c>
       <c r="R203" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S203" s="3" t="inlineStr"/>
       <c r="T203" s="3" t="inlineStr"/>
@@ -15616,7 +15616,7 @@
         <v>2780</v>
       </c>
       <c r="R204" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S204" s="3" t="inlineStr"/>
       <c r="T204" s="3" t="inlineStr"/>
@@ -15690,7 +15690,7 @@
         <v>2755</v>
       </c>
       <c r="R205" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S205" s="3" t="inlineStr"/>
       <c r="T205" s="3" t="inlineStr"/>
@@ -15764,7 +15764,7 @@
         <v>2765</v>
       </c>
       <c r="R206" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S206" s="3" t="inlineStr"/>
       <c r="T206" s="3" t="inlineStr"/>
@@ -15838,7 +15838,7 @@
         <v>2775</v>
       </c>
       <c r="R207" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S207" s="3" t="inlineStr"/>
       <c r="T207" s="3" t="inlineStr"/>
@@ -15912,7 +15912,7 @@
         <v>2785</v>
       </c>
       <c r="R208" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S208" s="3" t="inlineStr"/>
       <c r="T208" s="3" t="inlineStr"/>
@@ -15986,7 +15986,7 @@
         <v>2795</v>
       </c>
       <c r="R209" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S209" s="3" t="inlineStr"/>
       <c r="T209" s="3" t="inlineStr"/>
@@ -16060,7 +16060,7 @@
         <v>2805</v>
       </c>
       <c r="R210" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S210" s="3" t="inlineStr"/>
       <c r="T210" s="3" t="inlineStr"/>
@@ -16134,7 +16134,7 @@
         <v>2815</v>
       </c>
       <c r="R211" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S211" s="3" t="inlineStr"/>
       <c r="T211" s="3" t="inlineStr"/>
@@ -16208,7 +16208,7 @@
         <v>2825</v>
       </c>
       <c r="R212" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S212" s="3" t="inlineStr"/>
       <c r="T212" s="3" t="inlineStr"/>
@@ -16282,7 +16282,7 @@
         <v>2835</v>
       </c>
       <c r="R213" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S213" s="3" t="inlineStr"/>
       <c r="T213" s="3" t="inlineStr"/>
@@ -16356,7 +16356,7 @@
         <v>2845</v>
       </c>
       <c r="R214" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S214" s="3" t="inlineStr"/>
       <c r="T214" s="3" t="inlineStr"/>
@@ -16430,7 +16430,7 @@
         <v>1795</v>
       </c>
       <c r="R215" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S215" s="3" t="inlineStr"/>
       <c r="T215" s="3" t="inlineStr"/>
@@ -16504,7 +16504,7 @@
         <v>1815</v>
       </c>
       <c r="R216" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S216" s="3" t="inlineStr"/>
       <c r="T216" s="3" t="inlineStr"/>
@@ -16578,7 +16578,7 @@
         <v>1835</v>
       </c>
       <c r="R217" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S217" s="3" t="inlineStr"/>
       <c r="T217" s="3" t="inlineStr"/>
@@ -16652,7 +16652,7 @@
         <v>3145</v>
       </c>
       <c r="R218" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S218" s="3" t="inlineStr"/>
       <c r="T218" s="3" t="inlineStr"/>
@@ -16726,7 +16726,7 @@
         <v>885</v>
       </c>
       <c r="R219" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S219" s="3" t="inlineStr"/>
       <c r="T219" s="3" t="inlineStr"/>
@@ -16800,7 +16800,7 @@
         <v>2065</v>
       </c>
       <c r="R220" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S220" s="3" t="inlineStr"/>
       <c r="T220" s="3" t="inlineStr"/>
@@ -16874,7 +16874,7 @@
         <v>2085</v>
       </c>
       <c r="R221" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S221" s="3" t="inlineStr"/>
       <c r="T221" s="3" t="inlineStr"/>
@@ -16948,7 +16948,7 @@
         <v>2105</v>
       </c>
       <c r="R222" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S222" s="3" t="inlineStr"/>
       <c r="T222" s="3" t="inlineStr"/>
@@ -17022,7 +17022,7 @@
         <v>2925</v>
       </c>
       <c r="R223" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S223" s="3" t="inlineStr"/>
       <c r="T223" s="3" t="inlineStr"/>
@@ -17096,7 +17096,7 @@
         <v>2945</v>
       </c>
       <c r="R224" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S224" s="3" t="inlineStr"/>
       <c r="T224" s="3" t="inlineStr"/>
@@ -17170,7 +17170,7 @@
         <v>2060</v>
       </c>
       <c r="R225" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S225" s="3" t="inlineStr"/>
       <c r="T225" s="3" t="inlineStr"/>
@@ -17244,7 +17244,7 @@
         <v>2080</v>
       </c>
       <c r="R226" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S226" s="3" t="inlineStr"/>
       <c r="T226" s="3" t="inlineStr"/>
@@ -17318,7 +17318,7 @@
         <v>2100</v>
       </c>
       <c r="R227" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S227" s="3" t="inlineStr"/>
       <c r="T227" s="3" t="inlineStr"/>
@@ -17392,7 +17392,7 @@
         <v>2120</v>
       </c>
       <c r="R228" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S228" s="3" t="inlineStr"/>
       <c r="T228" s="3" t="inlineStr"/>
@@ -17466,7 +17466,7 @@
         <v>2460</v>
       </c>
       <c r="R229" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S229" s="3" t="inlineStr"/>
       <c r="T229" s="3" t="inlineStr"/>
@@ -17540,7 +17540,7 @@
         <v>2480</v>
       </c>
       <c r="R230" s="3" t="n">
-        <v>12</v>
+        <v>9999</v>
       </c>
       <c r="S230" s="3" t="inlineStr"/>
       <c r="T230" s="3" t="inlineStr"/>
@@ -17614,7 +17614,7 @@
         <v>2795</v>
       </c>
       <c r="R231" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S231" s="3" t="inlineStr"/>
       <c r="T231" s="3" t="inlineStr"/>
@@ -17688,7 +17688,7 @@
         <v>2815</v>
       </c>
       <c r="R232" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S232" s="3" t="inlineStr"/>
       <c r="T232" s="3" t="inlineStr"/>
@@ -17762,7 +17762,7 @@
         <v>830</v>
       </c>
       <c r="R233" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S233" s="3" t="inlineStr"/>
       <c r="T233" s="3" t="inlineStr"/>
@@ -17836,7 +17836,7 @@
         <v>840</v>
       </c>
       <c r="R234" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S234" s="3" t="inlineStr"/>
       <c r="T234" s="3" t="inlineStr"/>
@@ -17910,7 +17910,7 @@
         <v>2640</v>
       </c>
       <c r="R235" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S235" s="3" t="inlineStr"/>
       <c r="T235" s="3" t="inlineStr"/>
@@ -17984,7 +17984,7 @@
         <v>2750</v>
       </c>
       <c r="R236" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S236" s="3" t="inlineStr"/>
       <c r="T236" s="3" t="inlineStr"/>
@@ -18058,7 +18058,7 @@
         <v>2770</v>
       </c>
       <c r="R237" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S237" s="3" t="inlineStr"/>
       <c r="T237" s="3" t="inlineStr"/>
@@ -18132,7 +18132,7 @@
         <v>2790</v>
       </c>
       <c r="R238" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S238" s="3" t="inlineStr"/>
       <c r="T238" s="3" t="inlineStr"/>
@@ -18206,7 +18206,7 @@
         <v>2735</v>
       </c>
       <c r="R239" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S239" s="3" t="inlineStr"/>
       <c r="T239" s="3" t="inlineStr"/>
@@ -18280,7 +18280,7 @@
         <v>2755</v>
       </c>
       <c r="R240" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S240" s="3" t="inlineStr"/>
       <c r="T240" s="3" t="inlineStr"/>
@@ -18354,7 +18354,7 @@
         <v>1830</v>
       </c>
       <c r="R241" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S241" s="3" t="inlineStr"/>
       <c r="T241" s="3" t="inlineStr"/>
@@ -18428,7 +18428,7 @@
         <v>2760</v>
       </c>
       <c r="R242" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S242" s="3" t="inlineStr"/>
       <c r="T242" s="3" t="inlineStr"/>
@@ -18502,7 +18502,7 @@
         <v>2590</v>
       </c>
       <c r="R243" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S243" s="3" t="inlineStr"/>
       <c r="T243" s="3" t="inlineStr"/>
@@ -18576,7 +18576,7 @@
         <v>2610</v>
       </c>
       <c r="R244" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S244" s="3" t="inlineStr"/>
       <c r="T244" s="3" t="inlineStr"/>
@@ -18650,7 +18650,7 @@
         <v>1615</v>
       </c>
       <c r="R245" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S245" s="3" t="inlineStr"/>
       <c r="T245" s="3" t="inlineStr"/>
@@ -18724,7 +18724,7 @@
         <v>1635</v>
       </c>
       <c r="R246" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S246" s="3" t="inlineStr"/>
       <c r="T246" s="3" t="inlineStr"/>
@@ -18798,7 +18798,7 @@
         <v>1655</v>
       </c>
       <c r="R247" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S247" s="3" t="inlineStr"/>
       <c r="T247" s="3" t="inlineStr"/>
@@ -18872,7 +18872,7 @@
         <v>1675</v>
       </c>
       <c r="R248" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S248" s="3" t="inlineStr"/>
       <c r="T248" s="3" t="inlineStr"/>
@@ -18946,7 +18946,7 @@
         <v>3055</v>
       </c>
       <c r="R249" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S249" s="3" t="inlineStr"/>
       <c r="T249" s="3" t="inlineStr"/>
@@ -19020,7 +19020,7 @@
         <v>3075</v>
       </c>
       <c r="R250" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S250" s="3" t="inlineStr"/>
       <c r="T250" s="3" t="inlineStr"/>
@@ -19094,7 +19094,7 @@
         <v>1795</v>
       </c>
       <c r="R251" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S251" s="3" t="inlineStr"/>
       <c r="T251" s="3" t="inlineStr"/>
@@ -19168,7 +19168,7 @@
         <v>1815</v>
       </c>
       <c r="R252" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S252" s="3" t="inlineStr"/>
       <c r="T252" s="3" t="inlineStr"/>
@@ -19242,7 +19242,7 @@
         <v>2035</v>
       </c>
       <c r="R253" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S253" s="3" t="inlineStr"/>
       <c r="T253" s="3" t="inlineStr"/>
@@ -19316,7 +19316,7 @@
         <v>1790</v>
       </c>
       <c r="R254" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S254" s="3" t="inlineStr"/>
       <c r="T254" s="3" t="inlineStr"/>
@@ -19390,7 +19390,7 @@
         <v>1810</v>
       </c>
       <c r="R255" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S255" s="3" t="inlineStr"/>
       <c r="T255" s="3" t="inlineStr"/>
@@ -19464,7 +19464,7 @@
         <v>1830</v>
       </c>
       <c r="R256" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S256" s="3" t="inlineStr"/>
       <c r="T256" s="3" t="inlineStr"/>
@@ -19538,7 +19538,7 @@
         <v>2580</v>
       </c>
       <c r="R257" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S257" s="3" t="inlineStr"/>
       <c r="T257" s="3" t="inlineStr"/>
@@ -19612,7 +19612,7 @@
         <v>2600</v>
       </c>
       <c r="R258" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S258" s="3" t="inlineStr"/>
       <c r="T258" s="3" t="inlineStr"/>
@@ -19686,7 +19686,7 @@
         <v>2620</v>
       </c>
       <c r="R259" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S259" s="3" t="inlineStr"/>
       <c r="T259" s="3" t="inlineStr"/>
@@ -19760,7 +19760,7 @@
         <v>2640</v>
       </c>
       <c r="R260" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S260" s="3" t="inlineStr"/>
       <c r="T260" s="3" t="inlineStr"/>
@@ -19834,7 +19834,7 @@
         <v>2290</v>
       </c>
       <c r="R261" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S261" s="3" t="inlineStr"/>
       <c r="T261" s="3" t="inlineStr"/>
@@ -19908,7 +19908,7 @@
         <v>2725</v>
       </c>
       <c r="R262" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S262" s="3" t="inlineStr"/>
       <c r="T262" s="3" t="inlineStr"/>
@@ -19982,7 +19982,7 @@
         <v>2745</v>
       </c>
       <c r="R263" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S263" s="3" t="inlineStr"/>
       <c r="T263" s="3" t="inlineStr"/>
@@ -20056,7 +20056,7 @@
         <v>3100</v>
       </c>
       <c r="R264" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S264" s="3" t="inlineStr"/>
       <c r="T264" s="3" t="inlineStr"/>
@@ -20130,7 +20130,7 @@
         <v>3100</v>
       </c>
       <c r="R265" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S265" s="3" t="inlineStr"/>
       <c r="T265" s="3" t="inlineStr"/>
@@ -20204,7 +20204,7 @@
         <v>3120</v>
       </c>
       <c r="R266" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S266" s="3" t="inlineStr"/>
       <c r="T266" s="3" t="inlineStr"/>
@@ -20278,7 +20278,7 @@
         <v>1675</v>
       </c>
       <c r="R267" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S267" s="3" t="inlineStr"/>
       <c r="T267" s="3" t="inlineStr"/>
@@ -20352,7 +20352,7 @@
         <v>2385</v>
       </c>
       <c r="R268" s="3" t="n">
-        <v>40</v>
+        <v>9999</v>
       </c>
       <c r="S268" s="3" t="inlineStr"/>
       <c r="T268" s="3" t="inlineStr"/>
@@ -20426,7 +20426,7 @@
         <v>1495</v>
       </c>
       <c r="R269" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S269" s="3" t="inlineStr"/>
       <c r="T269" s="3" t="inlineStr"/>
@@ -20500,7 +20500,7 @@
         <v>1515</v>
       </c>
       <c r="R270" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S270" s="3" t="inlineStr"/>
       <c r="T270" s="3" t="inlineStr"/>
@@ -20574,7 +20574,7 @@
         <v>1535</v>
       </c>
       <c r="R271" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S271" s="3" t="inlineStr"/>
       <c r="T271" s="3" t="inlineStr"/>
@@ -20648,7 +20648,7 @@
         <v>1555</v>
       </c>
       <c r="R272" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S272" s="3" t="inlineStr"/>
       <c r="T272" s="3" t="inlineStr"/>
@@ -20722,7 +20722,7 @@
         <v>1575</v>
       </c>
       <c r="R273" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S273" s="3" t="inlineStr"/>
       <c r="T273" s="3" t="inlineStr"/>
@@ -20796,7 +20796,7 @@
         <v>1495</v>
       </c>
       <c r="R274" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S274" s="3" t="inlineStr"/>
       <c r="T274" s="3" t="inlineStr"/>
@@ -20870,7 +20870,7 @@
         <v>2005</v>
       </c>
       <c r="R275" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S275" s="3" t="inlineStr"/>
       <c r="T275" s="3" t="inlineStr"/>
@@ -20944,7 +20944,7 @@
         <v>2025</v>
       </c>
       <c r="R276" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S276" s="3" t="inlineStr"/>
       <c r="T276" s="3" t="inlineStr"/>
@@ -21018,7 +21018,7 @@
         <v>2045</v>
       </c>
       <c r="R277" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S277" s="3" t="inlineStr"/>
       <c r="T277" s="3" t="inlineStr"/>
@@ -21092,7 +21092,7 @@
         <v>2750</v>
       </c>
       <c r="R278" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S278" s="3" t="inlineStr"/>
       <c r="T278" s="3" t="inlineStr"/>
@@ -21166,7 +21166,7 @@
         <v>2770</v>
       </c>
       <c r="R279" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S279" s="3" t="inlineStr"/>
       <c r="T279" s="3" t="inlineStr"/>
@@ -21240,7 +21240,7 @@
         <v>785</v>
       </c>
       <c r="R280" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S280" s="3" t="inlineStr"/>
       <c r="T280" s="3" t="inlineStr"/>
@@ -21314,7 +21314,7 @@
         <v>795</v>
       </c>
       <c r="R281" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S281" s="3" t="inlineStr"/>
       <c r="T281" s="3" t="inlineStr"/>
@@ -21388,7 +21388,7 @@
         <v>805</v>
       </c>
       <c r="R282" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S282" s="3" t="inlineStr"/>
       <c r="T282" s="3" t="inlineStr"/>
@@ -21462,7 +21462,7 @@
         <v>2760</v>
       </c>
       <c r="R283" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S283" s="3" t="inlineStr"/>
       <c r="T283" s="3" t="inlineStr"/>
@@ -21536,7 +21536,7 @@
         <v>2780</v>
       </c>
       <c r="R284" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S284" s="3" t="inlineStr"/>
       <c r="T284" s="3" t="inlineStr"/>
@@ -21610,7 +21610,7 @@
         <v>2550</v>
       </c>
       <c r="R285" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S285" s="3" t="inlineStr"/>
       <c r="T285" s="3" t="inlineStr"/>
@@ -21684,7 +21684,7 @@
         <v>2570</v>
       </c>
       <c r="R286" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S286" s="3" t="inlineStr"/>
       <c r="T286" s="3" t="inlineStr"/>
@@ -21758,7 +21758,7 @@
         <v>2275</v>
       </c>
       <c r="R287" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S287" s="3" t="inlineStr"/>
       <c r="T287" s="3" t="inlineStr"/>
@@ -21832,7 +21832,7 @@
         <v>2295</v>
       </c>
       <c r="R288" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S288" s="3" t="inlineStr"/>
       <c r="T288" s="3" t="inlineStr"/>
@@ -21906,7 +21906,7 @@
         <v>2315</v>
       </c>
       <c r="R289" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S289" s="3" t="inlineStr"/>
       <c r="T289" s="3" t="inlineStr"/>
@@ -21980,7 +21980,7 @@
         <v>2245</v>
       </c>
       <c r="R290" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S290" s="3" t="inlineStr"/>
       <c r="T290" s="3" t="inlineStr"/>
@@ -22054,7 +22054,7 @@
         <v>700</v>
       </c>
       <c r="R291" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S291" s="3" t="inlineStr"/>
       <c r="T291" s="3" t="inlineStr"/>
@@ -22128,7 +22128,7 @@
         <v>710</v>
       </c>
       <c r="R292" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S292" s="3" t="inlineStr"/>
       <c r="T292" s="3" t="inlineStr"/>
@@ -22202,7 +22202,7 @@
         <v>720</v>
       </c>
       <c r="R293" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S293" s="3" t="inlineStr"/>
       <c r="T293" s="3" t="inlineStr"/>
@@ -22276,7 +22276,7 @@
         <v>730</v>
       </c>
       <c r="R294" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S294" s="3" t="inlineStr"/>
       <c r="T294" s="3" t="inlineStr"/>
@@ -22350,7 +22350,7 @@
         <v>740</v>
       </c>
       <c r="R295" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S295" s="3" t="inlineStr"/>
       <c r="T295" s="3" t="inlineStr"/>
@@ -22424,7 +22424,7 @@
         <v>2510</v>
       </c>
       <c r="R296" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S296" s="3" t="inlineStr"/>
       <c r="T296" s="3" t="inlineStr"/>
@@ -22498,7 +22498,7 @@
         <v>3035</v>
       </c>
       <c r="R297" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S297" s="3" t="inlineStr"/>
       <c r="T297" s="3" t="inlineStr"/>
@@ -22572,7 +22572,7 @@
         <v>2360</v>
       </c>
       <c r="R298" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S298" s="3" t="inlineStr"/>
       <c r="T298" s="3" t="inlineStr"/>
@@ -22646,7 +22646,7 @@
         <v>2380</v>
       </c>
       <c r="R299" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S299" s="3" t="inlineStr"/>
       <c r="T299" s="3" t="inlineStr"/>
@@ -22720,7 +22720,7 @@
         <v>2630</v>
       </c>
       <c r="R300" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S300" s="3" t="inlineStr"/>
       <c r="T300" s="3" t="inlineStr"/>
@@ -22794,7 +22794,7 @@
         <v>2650</v>
       </c>
       <c r="R301" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S301" s="3" t="inlineStr"/>
       <c r="T301" s="3" t="inlineStr"/>
@@ -22868,7 +22868,7 @@
         <v>1500</v>
       </c>
       <c r="R302" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S302" s="3" t="inlineStr"/>
       <c r="T302" s="3" t="inlineStr"/>
@@ -22942,7 +22942,7 @@
         <v>1495</v>
       </c>
       <c r="R303" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S303" s="3" t="inlineStr"/>
       <c r="T303" s="3" t="inlineStr"/>
@@ -23016,7 +23016,7 @@
         <v>1515</v>
       </c>
       <c r="R304" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S304" s="3" t="inlineStr"/>
       <c r="T304" s="3" t="inlineStr"/>
@@ -23090,7 +23090,7 @@
         <v>1535</v>
       </c>
       <c r="R305" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S305" s="3" t="inlineStr"/>
       <c r="T305" s="3" t="inlineStr"/>
@@ -23164,7 +23164,7 @@
         <v>670</v>
       </c>
       <c r="R306" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S306" s="3" t="inlineStr"/>
       <c r="T306" s="3" t="inlineStr"/>
@@ -23238,7 +23238,7 @@
         <v>680</v>
       </c>
       <c r="R307" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S307" s="3" t="inlineStr"/>
       <c r="T307" s="3" t="inlineStr"/>
@@ -23312,7 +23312,7 @@
         <v>670</v>
       </c>
       <c r="R308" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S308" s="3" t="inlineStr"/>
       <c r="T308" s="3" t="inlineStr"/>
@@ -23386,7 +23386,7 @@
         <v>680</v>
       </c>
       <c r="R309" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S309" s="3" t="inlineStr"/>
       <c r="T309" s="3" t="inlineStr"/>
@@ -23460,7 +23460,7 @@
         <v>1370</v>
       </c>
       <c r="R310" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S310" s="3" t="inlineStr"/>
       <c r="T310" s="3" t="inlineStr"/>
@@ -23534,7 +23534,7 @@
         <v>1390</v>
       </c>
       <c r="R311" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S311" s="3" t="inlineStr"/>
       <c r="T311" s="3" t="inlineStr"/>
@@ -23608,7 +23608,7 @@
         <v>1410</v>
       </c>
       <c r="R312" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S312" s="3" t="inlineStr"/>
       <c r="T312" s="3" t="inlineStr"/>
@@ -23682,7 +23682,7 @@
         <v>1430</v>
       </c>
       <c r="R313" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S313" s="3" t="inlineStr"/>
       <c r="T313" s="3" t="inlineStr"/>
@@ -23756,7 +23756,7 @@
         <v>1450</v>
       </c>
       <c r="R314" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S314" s="3" t="inlineStr"/>
       <c r="T314" s="3" t="inlineStr"/>
@@ -23830,7 +23830,7 @@
         <v>1470</v>
       </c>
       <c r="R315" s="3" t="n">
-        <v>28</v>
+        <v>9999</v>
       </c>
       <c r="S315" s="3" t="inlineStr"/>
       <c r="T315" s="3" t="inlineStr"/>
@@ -23904,7 +23904,7 @@
         <v>1355</v>
       </c>
       <c r="R316" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S316" s="3" t="inlineStr"/>
       <c r="T316" s="3" t="inlineStr"/>
@@ -23978,7 +23978,7 @@
         <v>1375</v>
       </c>
       <c r="R317" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S317" s="3" t="inlineStr"/>
       <c r="T317" s="3" t="inlineStr"/>
@@ -24052,7 +24052,7 @@
         <v>1395</v>
       </c>
       <c r="R318" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S318" s="3" t="inlineStr"/>
       <c r="T318" s="3" t="inlineStr"/>
@@ -24126,7 +24126,7 @@
         <v>1415</v>
       </c>
       <c r="R319" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S319" s="3" t="inlineStr"/>
       <c r="T319" s="3" t="inlineStr"/>
@@ -24200,7 +24200,7 @@
         <v>1435</v>
       </c>
       <c r="R320" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S320" s="3" t="inlineStr"/>
       <c r="T320" s="3" t="inlineStr"/>
@@ -24274,7 +24274,7 @@
         <v>1355</v>
       </c>
       <c r="R321" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S321" s="3" t="inlineStr"/>
       <c r="T321" s="3" t="inlineStr"/>
@@ -24348,7 +24348,7 @@
         <v>1375</v>
       </c>
       <c r="R322" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S322" s="3" t="inlineStr"/>
       <c r="T322" s="3" t="inlineStr"/>
@@ -24422,7 +24422,7 @@
         <v>1395</v>
       </c>
       <c r="R323" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S323" s="3" t="inlineStr"/>
       <c r="T323" s="3" t="inlineStr"/>
@@ -24496,7 +24496,7 @@
         <v>920</v>
       </c>
       <c r="R324" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S324" s="3" t="inlineStr"/>
       <c r="T324" s="3" t="inlineStr"/>
@@ -24570,7 +24570,7 @@
         <v>1335</v>
       </c>
       <c r="R325" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S325" s="3" t="inlineStr"/>
       <c r="T325" s="3" t="inlineStr"/>
@@ -24644,7 +24644,7 @@
         <v>1355</v>
       </c>
       <c r="R326" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S326" s="3" t="inlineStr"/>
       <c r="T326" s="3" t="inlineStr"/>
@@ -24718,7 +24718,7 @@
         <v>1375</v>
       </c>
       <c r="R327" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S327" s="3" t="inlineStr"/>
       <c r="T327" s="3" t="inlineStr"/>
@@ -24792,7 +24792,7 @@
         <v>1395</v>
       </c>
       <c r="R328" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S328" s="3" t="inlineStr"/>
       <c r="T328" s="3" t="inlineStr"/>
@@ -24866,7 +24866,7 @@
         <v>1415</v>
       </c>
       <c r="R329" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S329" s="3" t="inlineStr"/>
       <c r="T329" s="3" t="inlineStr"/>
@@ -24940,7 +24940,7 @@
         <v>965</v>
       </c>
       <c r="R330" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S330" s="3" t="inlineStr"/>
       <c r="T330" s="3" t="inlineStr"/>
@@ -25014,7 +25014,7 @@
         <v>975</v>
       </c>
       <c r="R331" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S331" s="3" t="inlineStr"/>
       <c r="T331" s="3" t="inlineStr"/>
@@ -25088,7 +25088,7 @@
         <v>985</v>
       </c>
       <c r="R332" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S332" s="3" t="inlineStr"/>
       <c r="T332" s="3" t="inlineStr"/>
@@ -25162,7 +25162,7 @@
         <v>905</v>
       </c>
       <c r="R333" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S333" s="3" t="inlineStr"/>
       <c r="T333" s="3" t="inlineStr"/>
@@ -25236,7 +25236,7 @@
         <v>915</v>
       </c>
       <c r="R334" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S334" s="3" t="inlineStr"/>
       <c r="T334" s="3" t="inlineStr"/>
@@ -25310,7 +25310,7 @@
         <v>925</v>
       </c>
       <c r="R335" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S335" s="3" t="inlineStr"/>
       <c r="T335" s="3" t="inlineStr"/>
@@ -25384,7 +25384,7 @@
         <v>1385</v>
       </c>
       <c r="R336" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S336" s="3" t="inlineStr"/>
       <c r="T336" s="3" t="inlineStr"/>
@@ -25458,7 +25458,7 @@
         <v>1405</v>
       </c>
       <c r="R337" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S337" s="3" t="inlineStr"/>
       <c r="T337" s="3" t="inlineStr"/>
@@ -25532,7 +25532,7 @@
         <v>905</v>
       </c>
       <c r="R338" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S338" s="3" t="inlineStr"/>
       <c r="T338" s="3" t="inlineStr"/>
@@ -25606,7 +25606,7 @@
         <v>650</v>
       </c>
       <c r="R339" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S339" s="3" t="inlineStr"/>
       <c r="T339" s="3" t="inlineStr"/>
@@ -25680,7 +25680,7 @@
         <v>660</v>
       </c>
       <c r="R340" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S340" s="3" t="inlineStr"/>
       <c r="T340" s="3" t="inlineStr"/>
@@ -25754,7 +25754,7 @@
         <v>670</v>
       </c>
       <c r="R341" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S341" s="3" t="inlineStr"/>
       <c r="T341" s="3" t="inlineStr"/>
@@ -25828,7 +25828,7 @@
         <v>600</v>
       </c>
       <c r="R342" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S342" s="3" t="inlineStr"/>
       <c r="T342" s="3" t="inlineStr"/>
@@ -25902,7 +25902,7 @@
         <v>610</v>
       </c>
       <c r="R343" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S343" s="3" t="inlineStr"/>
       <c r="T343" s="3" t="inlineStr"/>
@@ -25976,7 +25976,7 @@
         <v>620</v>
       </c>
       <c r="R344" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S344" s="3" t="inlineStr"/>
       <c r="T344" s="3" t="inlineStr"/>
@@ -26050,7 +26050,7 @@
         <v>630</v>
       </c>
       <c r="R345" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S345" s="3" t="inlineStr"/>
       <c r="T345" s="3" t="inlineStr"/>
@@ -26124,7 +26124,7 @@
         <v>640</v>
       </c>
       <c r="R346" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S346" s="3" t="inlineStr"/>
       <c r="T346" s="3" t="inlineStr"/>
@@ -26198,7 +26198,7 @@
         <v>625</v>
       </c>
       <c r="R347" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S347" s="3" t="inlineStr"/>
       <c r="T347" s="3" t="inlineStr"/>
@@ -26272,7 +26272,7 @@
         <v>635</v>
       </c>
       <c r="R348" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S348" s="3" t="inlineStr"/>
       <c r="T348" s="3" t="inlineStr"/>
@@ -26346,7 +26346,7 @@
         <v>645</v>
       </c>
       <c r="R349" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S349" s="3" t="inlineStr"/>
       <c r="T349" s="3" t="inlineStr"/>
@@ -26416,7 +26416,7 @@
       </c>
       <c r="Q350" s="3" t="inlineStr"/>
       <c r="R350" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S350" s="3" t="inlineStr">
         <is>
@@ -26490,7 +26490,7 @@
       </c>
       <c r="Q351" s="3" t="inlineStr"/>
       <c r="R351" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S351" s="3" t="inlineStr">
         <is>
@@ -26564,7 +26564,7 @@
       </c>
       <c r="Q352" s="3" t="inlineStr"/>
       <c r="R352" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S352" s="3" t="inlineStr">
         <is>
@@ -26638,7 +26638,7 @@
       </c>
       <c r="Q353" s="3" t="inlineStr"/>
       <c r="R353" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S353" s="3" t="inlineStr">
         <is>
@@ -26712,7 +26712,7 @@
       </c>
       <c r="Q354" s="3" t="inlineStr"/>
       <c r="R354" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S354" s="3" t="inlineStr">
         <is>
@@ -26786,7 +26786,7 @@
       </c>
       <c r="Q355" s="3" t="inlineStr"/>
       <c r="R355" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S355" s="3" t="inlineStr">
         <is>
@@ -26860,7 +26860,7 @@
       </c>
       <c r="Q356" s="3" t="inlineStr"/>
       <c r="R356" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S356" s="3" t="inlineStr">
         <is>
@@ -26934,7 +26934,7 @@
       </c>
       <c r="Q357" s="3" t="inlineStr"/>
       <c r="R357" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S357" s="3" t="inlineStr">
         <is>
@@ -27008,7 +27008,7 @@
       </c>
       <c r="Q358" s="3" t="inlineStr"/>
       <c r="R358" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S358" s="3" t="inlineStr">
         <is>
@@ -27082,7 +27082,7 @@
       </c>
       <c r="Q359" s="3" t="inlineStr"/>
       <c r="R359" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S359" s="3" t="inlineStr">
         <is>
@@ -27156,7 +27156,7 @@
       </c>
       <c r="Q360" s="3" t="inlineStr"/>
       <c r="R360" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S360" s="3" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
       </c>
       <c r="Q361" s="3" t="inlineStr"/>
       <c r="R361" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S361" s="3" t="inlineStr">
         <is>
@@ -27304,7 +27304,7 @@
       </c>
       <c r="Q362" s="3" t="inlineStr"/>
       <c r="R362" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S362" s="3" t="inlineStr">
         <is>
@@ -27378,7 +27378,7 @@
       </c>
       <c r="Q363" s="3" t="inlineStr"/>
       <c r="R363" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S363" s="3" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
       </c>
       <c r="Q364" s="3" t="inlineStr"/>
       <c r="R364" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S364" s="3" t="inlineStr">
         <is>
@@ -27526,7 +27526,7 @@
       </c>
       <c r="Q365" s="3" t="inlineStr"/>
       <c r="R365" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S365" s="3" t="inlineStr">
         <is>
@@ -27600,7 +27600,7 @@
       </c>
       <c r="Q366" s="3" t="inlineStr"/>
       <c r="R366" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S366" s="3" t="inlineStr">
         <is>
@@ -27674,7 +27674,7 @@
       </c>
       <c r="Q367" s="3" t="inlineStr"/>
       <c r="R367" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S367" s="3" t="inlineStr">
         <is>
@@ -27748,7 +27748,7 @@
       </c>
       <c r="Q368" s="3" t="inlineStr"/>
       <c r="R368" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S368" s="3" t="inlineStr">
         <is>
@@ -27822,7 +27822,7 @@
       </c>
       <c r="Q369" s="3" t="inlineStr"/>
       <c r="R369" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S369" s="3" t="inlineStr">
         <is>
@@ -27896,7 +27896,7 @@
       </c>
       <c r="Q370" s="3" t="inlineStr"/>
       <c r="R370" s="3" t="n">
-        <v>20</v>
+        <v>9999</v>
       </c>
       <c r="S370" s="3" t="inlineStr">
         <is>
@@ -27970,7 +27970,7 @@
       </c>
       <c r="Q371" s="3" t="inlineStr"/>
       <c r="R371" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S371" s="3" t="inlineStr">
         <is>
@@ -28044,7 +28044,7 @@
       </c>
       <c r="Q372" s="3" t="inlineStr"/>
       <c r="R372" s="3" t="n">
-        <v>25</v>
+        <v>9999</v>
       </c>
       <c r="S372" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update engine output files from prior run
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -660,7 +660,7 @@
         <v>3775</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S2" s="3" t="inlineStr"/>
       <c r="T2" s="3" t="inlineStr">
@@ -738,7 +738,7 @@
         <v>3795</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S3" s="3" t="inlineStr"/>
       <c r="T3" s="3" t="inlineStr">
@@ -816,7 +816,7 @@
         <v>3680</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S4" s="3" t="inlineStr"/>
       <c r="T4" s="3" t="inlineStr"/>
@@ -890,7 +890,7 @@
         <v>3700</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S5" s="3" t="inlineStr"/>
       <c r="T5" s="3" t="inlineStr"/>
@@ -964,7 +964,7 @@
         <v>3660</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S6" s="3" t="inlineStr"/>
       <c r="T6" s="3" t="inlineStr"/>
@@ -1038,7 +1038,7 @@
         <v>3680</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S7" s="3" t="inlineStr"/>
       <c r="T7" s="3" t="inlineStr"/>
@@ -1112,7 +1112,7 @@
         <v>3700</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S8" s="3" t="inlineStr"/>
       <c r="T8" s="3" t="inlineStr"/>
@@ -1186,7 +1186,7 @@
         <v>3720</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S9" s="3" t="inlineStr"/>
       <c r="T9" s="3" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
         <v>3740</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S10" s="3" t="inlineStr"/>
       <c r="T10" s="3" t="inlineStr"/>
@@ -1334,7 +1334,7 @@
         <v>3760</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S11" s="3" t="inlineStr"/>
       <c r="T11" s="3" t="inlineStr"/>
@@ -1408,7 +1408,7 @@
         <v>3780</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S12" s="3" t="inlineStr"/>
       <c r="T12" s="3" t="inlineStr"/>
@@ -1482,7 +1482,7 @@
         <v>3800</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S13" s="3" t="inlineStr"/>
       <c r="T13" s="3" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
         <v>3550</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S14" s="3" t="inlineStr"/>
       <c r="T14" s="3" t="inlineStr"/>
@@ -1630,7 +1630,7 @@
         <v>3550</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S15" s="3" t="inlineStr"/>
       <c r="T15" s="3" t="inlineStr"/>
@@ -1704,7 +1704,7 @@
         <v>3525</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S16" s="3" t="inlineStr"/>
       <c r="T16" s="3" t="inlineStr"/>
@@ -1778,7 +1778,7 @@
         <v>3545</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S17" s="3" t="inlineStr"/>
       <c r="T17" s="3" t="inlineStr"/>
@@ -1852,7 +1852,7 @@
         <v>1725</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S18" s="3" t="inlineStr"/>
       <c r="T18" s="3" t="inlineStr"/>
@@ -1926,7 +1926,7 @@
         <v>1715</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S19" s="3" t="inlineStr"/>
       <c r="T19" s="3" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
         <v>1725</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S20" s="3" t="inlineStr"/>
       <c r="T20" s="3" t="inlineStr"/>
@@ -2074,7 +2074,7 @@
         <v>1735</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S21" s="3" t="inlineStr"/>
       <c r="T21" s="3" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
         <v>1745</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
       <c r="T22" s="3" t="inlineStr"/>
@@ -2222,7 +2222,7 @@
         <v>1695</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S23" s="3" t="inlineStr"/>
       <c r="T23" s="3" t="inlineStr"/>
@@ -2296,7 +2296,7 @@
         <v>1705</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S24" s="3" t="inlineStr"/>
       <c r="T24" s="3" t="inlineStr"/>
@@ -2370,7 +2370,7 @@
         <v>1715</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S25" s="3" t="inlineStr"/>
       <c r="T25" s="3" t="inlineStr"/>
@@ -2444,7 +2444,7 @@
         <v>1725</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S26" s="3" t="inlineStr"/>
       <c r="T26" s="3" t="inlineStr"/>
@@ -2518,7 +2518,7 @@
         <v>1735</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S27" s="3" t="inlineStr"/>
       <c r="T27" s="3" t="inlineStr"/>
@@ -2592,7 +2592,7 @@
         <v>1745</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S28" s="3" t="inlineStr"/>
       <c r="T28" s="3" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
         <v>1755</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S29" s="3" t="inlineStr"/>
       <c r="T29" s="3" t="inlineStr"/>
@@ -2740,7 +2740,7 @@
         <v>1765</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S30" s="3" t="inlineStr"/>
       <c r="T30" s="3" t="inlineStr"/>
@@ -2814,7 +2814,7 @@
         <v>3630</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S31" s="3" t="inlineStr"/>
       <c r="T31" s="3" t="inlineStr"/>
@@ -2888,7 +2888,7 @@
         <v>3480</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S32" s="3" t="inlineStr"/>
       <c r="T32" s="3" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
         <v>3175</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S33" s="3" t="inlineStr"/>
       <c r="T33" s="3" t="inlineStr"/>
@@ -3036,7 +3036,7 @@
         <v>3195</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S34" s="3" t="inlineStr"/>
       <c r="T34" s="3" t="inlineStr"/>
@@ -3110,7 +3110,7 @@
         <v>3445</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S35" s="3" t="inlineStr"/>
       <c r="T35" s="3" t="inlineStr"/>
@@ -3184,7 +3184,7 @@
         <v>3465</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S36" s="3" t="inlineStr"/>
       <c r="T36" s="3" t="inlineStr"/>
@@ -3258,7 +3258,7 @@
         <v>3135</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S37" s="3" t="inlineStr"/>
       <c r="T37" s="3" t="inlineStr"/>
@@ -3332,7 +3332,7 @@
         <v>3155</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S38" s="3" t="inlineStr"/>
       <c r="T38" s="3" t="inlineStr"/>
@@ -3406,7 +3406,7 @@
         <v>3175</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S39" s="3" t="inlineStr"/>
       <c r="T39" s="3" t="inlineStr"/>
@@ -3480,7 +3480,7 @@
         <v>1560</v>
       </c>
       <c r="R40" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S40" s="3" t="inlineStr"/>
       <c r="T40" s="3" t="inlineStr"/>
@@ -3554,7 +3554,7 @@
         <v>1570</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S41" s="3" t="inlineStr"/>
       <c r="T41" s="3" t="inlineStr"/>
@@ -3628,7 +3628,7 @@
         <v>1580</v>
       </c>
       <c r="R42" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S42" s="3" t="inlineStr"/>
       <c r="T42" s="3" t="inlineStr"/>
@@ -3702,7 +3702,7 @@
         <v>3575</v>
       </c>
       <c r="R43" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S43" s="3" t="inlineStr"/>
       <c r="T43" s="3" t="inlineStr"/>
@@ -3776,7 +3776,7 @@
         <v>3595</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S44" s="3" t="inlineStr"/>
       <c r="T44" s="3" t="inlineStr"/>
@@ -3850,7 +3850,7 @@
         <v>3615</v>
       </c>
       <c r="R45" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S45" s="3" t="inlineStr"/>
       <c r="T45" s="3" t="inlineStr"/>
@@ -3924,7 +3924,7 @@
         <v>3110</v>
       </c>
       <c r="R46" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S46" s="3" t="inlineStr"/>
       <c r="T46" s="3" t="inlineStr"/>
@@ -3998,7 +3998,7 @@
         <v>3120</v>
       </c>
       <c r="R47" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S47" s="3" t="inlineStr"/>
       <c r="T47" s="3" t="inlineStr"/>
@@ -4072,7 +4072,7 @@
         <v>3100</v>
       </c>
       <c r="R48" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S48" s="3" t="inlineStr"/>
       <c r="T48" s="3" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
         <v>3120</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S49" s="3" t="inlineStr"/>
       <c r="T49" s="3" t="inlineStr"/>
@@ -4220,7 +4220,7 @@
         <v>3085</v>
       </c>
       <c r="R50" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S50" s="3" t="inlineStr"/>
       <c r="T50" s="3" t="inlineStr"/>
@@ -4294,7 +4294,7 @@
         <v>3105</v>
       </c>
       <c r="R51" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S51" s="3" t="inlineStr"/>
       <c r="T51" s="3" t="inlineStr"/>
@@ -4368,7 +4368,7 @@
         <v>3130</v>
       </c>
       <c r="R52" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S52" s="3" t="inlineStr"/>
       <c r="T52" s="3" t="inlineStr"/>
@@ -4442,7 +4442,7 @@
         <v>3025</v>
       </c>
       <c r="R53" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S53" s="3" t="inlineStr"/>
       <c r="T53" s="3" t="inlineStr"/>
@@ -4516,7 +4516,7 @@
         <v>3045</v>
       </c>
       <c r="R54" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S54" s="3" t="inlineStr"/>
       <c r="T54" s="3" t="inlineStr"/>
@@ -4590,7 +4590,7 @@
         <v>3275</v>
       </c>
       <c r="R55" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S55" s="3" t="inlineStr"/>
       <c r="T55" s="3" t="inlineStr"/>
@@ -4664,7 +4664,7 @@
         <v>3295</v>
       </c>
       <c r="R56" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S56" s="3" t="inlineStr"/>
       <c r="T56" s="3" t="inlineStr"/>
@@ -4738,7 +4738,7 @@
         <v>3315</v>
       </c>
       <c r="R57" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S57" s="3" t="inlineStr"/>
       <c r="T57" s="3" t="inlineStr"/>
@@ -4812,7 +4812,7 @@
         <v>3335</v>
       </c>
       <c r="R58" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S58" s="3" t="inlineStr"/>
       <c r="T58" s="3" t="inlineStr"/>
@@ -4886,7 +4886,7 @@
         <v>3355</v>
       </c>
       <c r="R59" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S59" s="3" t="inlineStr"/>
       <c r="T59" s="3" t="inlineStr"/>
@@ -4960,7 +4960,7 @@
         <v>3375</v>
       </c>
       <c r="R60" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S60" s="3" t="inlineStr"/>
       <c r="T60" s="3" t="inlineStr"/>
@@ -5034,7 +5034,7 @@
         <v>2975</v>
       </c>
       <c r="R61" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S61" s="3" t="inlineStr"/>
       <c r="T61" s="3" t="inlineStr"/>
@@ -5108,7 +5108,7 @@
         <v>2995</v>
       </c>
       <c r="R62" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S62" s="3" t="inlineStr"/>
       <c r="T62" s="3" t="inlineStr"/>
@@ -5182,7 +5182,7 @@
         <v>2950</v>
       </c>
       <c r="R63" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S63" s="3" t="inlineStr"/>
       <c r="T63" s="3" t="inlineStr"/>
@@ -5256,7 +5256,7 @@
         <v>2905</v>
       </c>
       <c r="R64" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S64" s="3" t="inlineStr"/>
       <c r="T64" s="3" t="inlineStr"/>
@@ -5330,7 +5330,7 @@
         <v>2855</v>
       </c>
       <c r="R65" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S65" s="3" t="inlineStr"/>
       <c r="T65" s="3" t="inlineStr"/>
@@ -5404,7 +5404,7 @@
         <v>2875</v>
       </c>
       <c r="R66" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S66" s="3" t="inlineStr"/>
       <c r="T66" s="3" t="inlineStr"/>
@@ -5478,7 +5478,7 @@
         <v>2895</v>
       </c>
       <c r="R67" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S67" s="3" t="inlineStr"/>
       <c r="T67" s="3" t="inlineStr"/>
@@ -5552,7 +5552,7 @@
         <v>2855</v>
       </c>
       <c r="R68" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S68" s="3" t="inlineStr"/>
       <c r="T68" s="3" t="inlineStr"/>
@@ -5626,7 +5626,7 @@
         <v>2875</v>
       </c>
       <c r="R69" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S69" s="3" t="inlineStr"/>
       <c r="T69" s="3" t="inlineStr"/>
@@ -5700,7 +5700,7 @@
         <v>3070</v>
       </c>
       <c r="R70" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S70" s="3" t="inlineStr"/>
       <c r="T70" s="3" t="inlineStr"/>
@@ -5774,7 +5774,7 @@
         <v>2985</v>
       </c>
       <c r="R71" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S71" s="3" t="inlineStr"/>
       <c r="T71" s="3" t="inlineStr"/>
@@ -5848,7 +5848,7 @@
         <v>3005</v>
       </c>
       <c r="R72" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S72" s="3" t="inlineStr"/>
       <c r="T72" s="3" t="inlineStr"/>
@@ -5922,7 +5922,7 @@
         <v>1310</v>
       </c>
       <c r="R73" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S73" s="3" t="inlineStr"/>
       <c r="T73" s="3" t="inlineStr"/>
@@ -5996,7 +5996,7 @@
         <v>1320</v>
       </c>
       <c r="R74" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S74" s="3" t="inlineStr"/>
       <c r="T74" s="3" t="inlineStr"/>
@@ -6070,7 +6070,7 @@
         <v>2635</v>
       </c>
       <c r="R75" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S75" s="3" t="inlineStr"/>
       <c r="T75" s="3" t="inlineStr"/>
@@ -6144,7 +6144,7 @@
         <v>2635</v>
       </c>
       <c r="R76" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S76" s="3" t="inlineStr"/>
       <c r="T76" s="3" t="inlineStr"/>
@@ -6218,7 +6218,7 @@
         <v>2655</v>
       </c>
       <c r="R77" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S77" s="3" t="inlineStr"/>
       <c r="T77" s="3" t="inlineStr"/>
@@ -6292,7 +6292,7 @@
         <v>2630</v>
       </c>
       <c r="R78" s="3" t="n">
-        <v>9999</v>
+        <v>40</v>
       </c>
       <c r="S78" s="3" t="inlineStr"/>
       <c r="T78" s="3" t="inlineStr"/>
@@ -6366,7 +6366,7 @@
         <v>2770</v>
       </c>
       <c r="R79" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S79" s="3" t="inlineStr"/>
       <c r="T79" s="3" t="inlineStr"/>
@@ -6440,7 +6440,7 @@
         <v>2790</v>
       </c>
       <c r="R80" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S80" s="3" t="inlineStr"/>
       <c r="T80" s="3" t="inlineStr"/>
@@ -6514,7 +6514,7 @@
         <v>2560</v>
       </c>
       <c r="R81" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S81" s="3" t="inlineStr"/>
       <c r="T81" s="3" t="inlineStr"/>
@@ -6588,7 +6588,7 @@
         <v>2580</v>
       </c>
       <c r="R82" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S82" s="3" t="inlineStr"/>
       <c r="T82" s="3" t="inlineStr"/>
@@ -6662,7 +6662,7 @@
         <v>2520</v>
       </c>
       <c r="R83" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S83" s="3" t="inlineStr"/>
       <c r="T83" s="3" t="inlineStr"/>
@@ -6736,7 +6736,7 @@
         <v>3235</v>
       </c>
       <c r="R84" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S84" s="3" t="inlineStr"/>
       <c r="T84" s="3" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
         <v>3255</v>
       </c>
       <c r="R85" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S85" s="3" t="inlineStr"/>
       <c r="T85" s="3" t="inlineStr"/>
@@ -6884,7 +6884,7 @@
         <v>3275</v>
       </c>
       <c r="R86" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S86" s="3" t="inlineStr"/>
       <c r="T86" s="3" t="inlineStr"/>
@@ -6958,7 +6958,7 @@
         <v>3295</v>
       </c>
       <c r="R87" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S87" s="3" t="inlineStr"/>
       <c r="T87" s="3" t="inlineStr"/>
@@ -7032,7 +7032,7 @@
         <v>1235</v>
       </c>
       <c r="R88" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S88" s="3" t="inlineStr"/>
       <c r="T88" s="3" t="inlineStr"/>
@@ -7106,7 +7106,7 @@
         <v>1245</v>
       </c>
       <c r="R89" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S89" s="3" t="inlineStr"/>
       <c r="T89" s="3" t="inlineStr"/>
@@ -7180,7 +7180,7 @@
         <v>1255</v>
       </c>
       <c r="R90" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S90" s="3" t="inlineStr"/>
       <c r="T90" s="3" t="inlineStr"/>
@@ -7254,7 +7254,7 @@
         <v>2600</v>
       </c>
       <c r="R91" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S91" s="3" t="inlineStr"/>
       <c r="T91" s="3" t="inlineStr"/>
@@ -7328,7 +7328,7 @@
         <v>2595</v>
       </c>
       <c r="R92" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S92" s="3" t="inlineStr"/>
       <c r="T92" s="3" t="inlineStr"/>
@@ -7402,7 +7402,7 @@
         <v>2615</v>
       </c>
       <c r="R93" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S93" s="3" t="inlineStr"/>
       <c r="T93" s="3" t="inlineStr"/>
@@ -7476,7 +7476,7 @@
         <v>3015</v>
       </c>
       <c r="R94" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S94" s="3" t="inlineStr"/>
       <c r="T94" s="3" t="inlineStr"/>
@@ -7550,7 +7550,7 @@
         <v>3035</v>
       </c>
       <c r="R95" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S95" s="3" t="inlineStr"/>
       <c r="T95" s="3" t="inlineStr"/>
@@ -7624,7 +7624,7 @@
         <v>2790</v>
       </c>
       <c r="R96" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S96" s="3" t="inlineStr"/>
       <c r="T96" s="3" t="inlineStr"/>
@@ -7698,7 +7698,7 @@
         <v>2810</v>
       </c>
       <c r="R97" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S97" s="3" t="inlineStr"/>
       <c r="T97" s="3" t="inlineStr"/>
@@ -7772,7 +7772,7 @@
         <v>2460</v>
       </c>
       <c r="R98" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S98" s="3" t="inlineStr"/>
       <c r="T98" s="3" t="inlineStr"/>
@@ -7846,7 +7846,7 @@
         <v>2995</v>
       </c>
       <c r="R99" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S99" s="3" t="inlineStr"/>
       <c r="T99" s="3" t="inlineStr"/>
@@ -7920,7 +7920,7 @@
         <v>3015</v>
       </c>
       <c r="R100" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S100" s="3" t="inlineStr"/>
       <c r="T100" s="3" t="inlineStr"/>
@@ -7994,7 +7994,7 @@
         <v>3470</v>
       </c>
       <c r="R101" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S101" s="3" t="inlineStr"/>
       <c r="T101" s="3" t="inlineStr"/>
@@ -8068,7 +8068,7 @@
         <v>3490</v>
       </c>
       <c r="R102" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S102" s="3" t="inlineStr"/>
       <c r="T102" s="3" t="inlineStr"/>
@@ -8142,7 +8142,7 @@
         <v>3510</v>
       </c>
       <c r="R103" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S103" s="3" t="inlineStr"/>
       <c r="T103" s="3" t="inlineStr"/>
@@ -8216,7 +8216,7 @@
         <v>3040</v>
       </c>
       <c r="R104" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S104" s="3" t="inlineStr"/>
       <c r="T104" s="3" t="inlineStr"/>
@@ -8290,7 +8290,7 @@
         <v>3455</v>
       </c>
       <c r="R105" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S105" s="3" t="inlineStr"/>
       <c r="T105" s="3" t="inlineStr"/>
@@ -8364,7 +8364,7 @@
         <v>3045</v>
       </c>
       <c r="R106" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S106" s="3" t="inlineStr"/>
       <c r="T106" s="3" t="inlineStr"/>
@@ -8438,7 +8438,7 @@
         <v>3055</v>
       </c>
       <c r="R107" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S107" s="3" t="inlineStr"/>
       <c r="T107" s="3" t="inlineStr"/>
@@ -8512,7 +8512,7 @@
         <v>1270</v>
       </c>
       <c r="R108" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S108" s="3" t="inlineStr"/>
       <c r="T108" s="3" t="inlineStr"/>
@@ -8586,7 +8586,7 @@
         <v>2375</v>
       </c>
       <c r="R109" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S109" s="3" t="inlineStr"/>
       <c r="T109" s="3" t="inlineStr"/>
@@ -8660,7 +8660,7 @@
         <v>2395</v>
       </c>
       <c r="R110" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S110" s="3" t="inlineStr"/>
       <c r="T110" s="3" t="inlineStr"/>
@@ -8734,7 +8734,7 @@
         <v>2430</v>
       </c>
       <c r="R111" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S111" s="3" t="inlineStr"/>
       <c r="T111" s="3" t="inlineStr"/>
@@ -8808,7 +8808,7 @@
         <v>2450</v>
       </c>
       <c r="R112" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S112" s="3" t="inlineStr"/>
       <c r="T112" s="3" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
         <v>2470</v>
       </c>
       <c r="R113" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S113" s="3" t="inlineStr"/>
       <c r="T113" s="3" t="inlineStr"/>
@@ -8956,7 +8956,7 @@
         <v>3010</v>
       </c>
       <c r="R114" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S114" s="3" t="inlineStr"/>
       <c r="T114" s="3" t="inlineStr"/>
@@ -9030,7 +9030,7 @@
         <v>3030</v>
       </c>
       <c r="R115" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S115" s="3" t="inlineStr"/>
       <c r="T115" s="3" t="inlineStr"/>
@@ -9104,7 +9104,7 @@
         <v>1160</v>
       </c>
       <c r="R116" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S116" s="3" t="inlineStr"/>
       <c r="T116" s="3" t="inlineStr"/>
@@ -9178,7 +9178,7 @@
         <v>2545</v>
       </c>
       <c r="R117" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S117" s="3" t="inlineStr"/>
       <c r="T117" s="3" t="inlineStr"/>
@@ -9252,7 +9252,7 @@
         <v>1135</v>
       </c>
       <c r="R118" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S118" s="3" t="inlineStr"/>
       <c r="T118" s="3" t="inlineStr"/>
@@ -9326,7 +9326,7 @@
         <v>1145</v>
       </c>
       <c r="R119" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S119" s="3" t="inlineStr"/>
       <c r="T119" s="3" t="inlineStr"/>
@@ -9400,7 +9400,7 @@
         <v>1155</v>
       </c>
       <c r="R120" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S120" s="3" t="inlineStr"/>
       <c r="T120" s="3" t="inlineStr"/>
@@ -9474,7 +9474,7 @@
         <v>1165</v>
       </c>
       <c r="R121" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S121" s="3" t="inlineStr"/>
       <c r="T121" s="3" t="inlineStr"/>
@@ -9548,7 +9548,7 @@
         <v>1175</v>
       </c>
       <c r="R122" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S122" s="3" t="inlineStr"/>
       <c r="T122" s="3" t="inlineStr"/>
@@ -9622,7 +9622,7 @@
         <v>2980</v>
       </c>
       <c r="R123" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S123" s="3" t="inlineStr"/>
       <c r="T123" s="3" t="inlineStr"/>
@@ -9696,7 +9696,7 @@
         <v>3000</v>
       </c>
       <c r="R124" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S124" s="3" t="inlineStr"/>
       <c r="T124" s="3" t="inlineStr"/>
@@ -9770,7 +9770,7 @@
         <v>2575</v>
       </c>
       <c r="R125" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S125" s="3" t="inlineStr"/>
       <c r="T125" s="3" t="inlineStr"/>
@@ -9844,7 +9844,7 @@
         <v>3220</v>
       </c>
       <c r="R126" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S126" s="3" t="inlineStr"/>
       <c r="T126" s="3" t="inlineStr"/>
@@ -9918,7 +9918,7 @@
         <v>3240</v>
       </c>
       <c r="R127" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S127" s="3" t="inlineStr"/>
       <c r="T127" s="3" t="inlineStr"/>
@@ -9992,7 +9992,7 @@
         <v>1195</v>
       </c>
       <c r="R128" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S128" s="3" t="inlineStr"/>
       <c r="T128" s="3" t="inlineStr"/>
@@ -10066,7 +10066,7 @@
         <v>1210</v>
       </c>
       <c r="R129" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S129" s="3" t="inlineStr"/>
       <c r="T129" s="3" t="inlineStr"/>
@@ -10140,7 +10140,7 @@
         <v>1130</v>
       </c>
       <c r="R130" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S130" s="3" t="inlineStr"/>
       <c r="T130" s="3" t="inlineStr"/>
@@ -10214,7 +10214,7 @@
         <v>1410</v>
       </c>
       <c r="R131" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S131" s="3" t="inlineStr"/>
       <c r="T131" s="3" t="inlineStr"/>
@@ -10288,7 +10288,7 @@
         <v>2165</v>
       </c>
       <c r="R132" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S132" s="3" t="inlineStr"/>
       <c r="T132" s="3" t="inlineStr"/>
@@ -10362,7 +10362,7 @@
         <v>2185</v>
       </c>
       <c r="R133" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S133" s="3" t="inlineStr"/>
       <c r="T133" s="3" t="inlineStr"/>
@@ -10436,7 +10436,7 @@
         <v>2205</v>
       </c>
       <c r="R134" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S134" s="3" t="inlineStr"/>
       <c r="T134" s="3" t="inlineStr"/>
@@ -10510,7 +10510,7 @@
         <v>2165</v>
       </c>
       <c r="R135" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S135" s="3" t="inlineStr"/>
       <c r="T135" s="3" t="inlineStr"/>
@@ -10584,7 +10584,7 @@
         <v>2185</v>
       </c>
       <c r="R136" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S136" s="3" t="inlineStr"/>
       <c r="T136" s="3" t="inlineStr"/>
@@ -10658,7 +10658,7 @@
         <v>2160</v>
       </c>
       <c r="R137" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S137" s="3" t="inlineStr"/>
       <c r="T137" s="3" t="inlineStr"/>
@@ -10732,7 +10732,7 @@
         <v>2800</v>
       </c>
       <c r="R138" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S138" s="3" t="inlineStr"/>
       <c r="T138" s="3" t="inlineStr"/>
@@ -10806,7 +10806,7 @@
         <v>2815</v>
       </c>
       <c r="R139" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S139" s="3" t="inlineStr"/>
       <c r="T139" s="3" t="inlineStr"/>
@@ -10880,7 +10880,7 @@
         <v>2835</v>
       </c>
       <c r="R140" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S140" s="3" t="inlineStr"/>
       <c r="T140" s="3" t="inlineStr"/>
@@ -10954,7 +10954,7 @@
         <v>2855</v>
       </c>
       <c r="R141" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S141" s="3" t="inlineStr"/>
       <c r="T141" s="3" t="inlineStr"/>
@@ -11028,7 +11028,7 @@
         <v>2155</v>
       </c>
       <c r="R142" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S142" s="3" t="inlineStr"/>
       <c r="T142" s="3" t="inlineStr"/>
@@ -11102,7 +11102,7 @@
         <v>2540</v>
       </c>
       <c r="R143" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S143" s="3" t="inlineStr"/>
       <c r="T143" s="3" t="inlineStr"/>
@@ -11176,7 +11176,7 @@
         <v>2560</v>
       </c>
       <c r="R144" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S144" s="3" t="inlineStr"/>
       <c r="T144" s="3" t="inlineStr"/>
@@ -11250,7 +11250,7 @@
         <v>2135</v>
       </c>
       <c r="R145" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S145" s="3" t="inlineStr"/>
       <c r="T145" s="3" t="inlineStr"/>
@@ -11324,7 +11324,7 @@
         <v>2155</v>
       </c>
       <c r="R146" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S146" s="3" t="inlineStr"/>
       <c r="T146" s="3" t="inlineStr"/>
@@ -11398,7 +11398,7 @@
         <v>2135</v>
       </c>
       <c r="R147" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S147" s="3" t="inlineStr"/>
       <c r="T147" s="3" t="inlineStr"/>
@@ -11472,7 +11472,7 @@
         <v>2155</v>
       </c>
       <c r="R148" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S148" s="3" t="inlineStr"/>
       <c r="T148" s="3" t="inlineStr"/>
@@ -11546,7 +11546,7 @@
         <v>2175</v>
       </c>
       <c r="R149" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S149" s="3" t="inlineStr"/>
       <c r="T149" s="3" t="inlineStr"/>
@@ -11620,7 +11620,7 @@
         <v>2195</v>
       </c>
       <c r="R150" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S150" s="3" t="inlineStr"/>
       <c r="T150" s="3" t="inlineStr"/>
@@ -11694,7 +11694,7 @@
         <v>2215</v>
       </c>
       <c r="R151" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S151" s="3" t="inlineStr"/>
       <c r="T151" s="3" t="inlineStr"/>
@@ -11768,7 +11768,7 @@
         <v>2145</v>
       </c>
       <c r="R152" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S152" s="3" t="inlineStr"/>
       <c r="T152" s="3" t="inlineStr"/>
@@ -11842,7 +11842,7 @@
         <v>2165</v>
       </c>
       <c r="R153" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S153" s="3" t="inlineStr"/>
       <c r="T153" s="3" t="inlineStr"/>
@@ -11916,7 +11916,7 @@
         <v>2185</v>
       </c>
       <c r="R154" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S154" s="3" t="inlineStr"/>
       <c r="T154" s="3" t="inlineStr"/>
@@ -11990,7 +11990,7 @@
         <v>2205</v>
       </c>
       <c r="R155" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S155" s="3" t="inlineStr"/>
       <c r="T155" s="3" t="inlineStr"/>
@@ -12064,7 +12064,7 @@
         <v>2175</v>
       </c>
       <c r="R156" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S156" s="3" t="inlineStr"/>
       <c r="T156" s="3" t="inlineStr"/>
@@ -12138,7 +12138,7 @@
         <v>2185</v>
       </c>
       <c r="R157" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S157" s="3" t="inlineStr"/>
       <c r="T157" s="3" t="inlineStr"/>
@@ -12212,7 +12212,7 @@
         <v>2195</v>
       </c>
       <c r="R158" s="3" t="n">
-        <v>9999</v>
+        <v>15</v>
       </c>
       <c r="S158" s="3" t="inlineStr"/>
       <c r="T158" s="3" t="inlineStr"/>
@@ -12286,7 +12286,7 @@
         <v>2985</v>
       </c>
       <c r="R159" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S159" s="3" t="inlineStr"/>
       <c r="T159" s="3" t="inlineStr"/>
@@ -12360,7 +12360,7 @@
         <v>2995</v>
       </c>
       <c r="R160" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S160" s="3" t="inlineStr"/>
       <c r="T160" s="3" t="inlineStr"/>
@@ -12434,7 +12434,7 @@
         <v>3005</v>
       </c>
       <c r="R161" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S161" s="3" t="inlineStr"/>
       <c r="T161" s="3" t="inlineStr"/>
@@ -12508,7 +12508,7 @@
         <v>3015</v>
       </c>
       <c r="R162" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S162" s="3" t="inlineStr"/>
       <c r="T162" s="3" t="inlineStr"/>
@@ -12582,7 +12582,7 @@
         <v>3025</v>
       </c>
       <c r="R163" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S163" s="3" t="inlineStr"/>
       <c r="T163" s="3" t="inlineStr"/>
@@ -12656,7 +12656,7 @@
         <v>3035</v>
       </c>
       <c r="R164" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S164" s="3" t="inlineStr"/>
       <c r="T164" s="3" t="inlineStr"/>
@@ -12730,7 +12730,7 @@
         <v>3045</v>
       </c>
       <c r="R165" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S165" s="3" t="inlineStr"/>
       <c r="T165" s="3" t="inlineStr"/>
@@ -12804,7 +12804,7 @@
         <v>3055</v>
       </c>
       <c r="R166" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S166" s="3" t="inlineStr"/>
       <c r="T166" s="3" t="inlineStr"/>
@@ -12878,7 +12878,7 @@
         <v>2695</v>
       </c>
       <c r="R167" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S167" s="3" t="inlineStr"/>
       <c r="T167" s="3" t="inlineStr"/>
@@ -12952,7 +12952,7 @@
         <v>3200</v>
       </c>
       <c r="R168" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S168" s="3" t="inlineStr"/>
       <c r="T168" s="3" t="inlineStr"/>
@@ -13026,7 +13026,7 @@
         <v>3375</v>
       </c>
       <c r="R169" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S169" s="3" t="inlineStr"/>
       <c r="T169" s="3" t="inlineStr"/>
@@ -13100,7 +13100,7 @@
         <v>3395</v>
       </c>
       <c r="R170" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S170" s="3" t="inlineStr"/>
       <c r="T170" s="3" t="inlineStr"/>
@@ -13174,7 +13174,7 @@
         <v>2950</v>
       </c>
       <c r="R171" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S171" s="3" t="inlineStr"/>
       <c r="T171" s="3" t="inlineStr"/>
@@ -13248,7 +13248,7 @@
         <v>2970</v>
       </c>
       <c r="R172" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S172" s="3" t="inlineStr"/>
       <c r="T172" s="3" t="inlineStr"/>
@@ -13322,7 +13322,7 @@
         <v>2990</v>
       </c>
       <c r="R173" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S173" s="3" t="inlineStr"/>
       <c r="T173" s="3" t="inlineStr"/>
@@ -13396,7 +13396,7 @@
         <v>3010</v>
       </c>
       <c r="R174" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S174" s="3" t="inlineStr"/>
       <c r="T174" s="3" t="inlineStr"/>
@@ -13470,7 +13470,7 @@
         <v>2665</v>
       </c>
       <c r="R175" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S175" s="3" t="inlineStr"/>
       <c r="T175" s="3" t="inlineStr"/>
@@ -13544,7 +13544,7 @@
         <v>2670</v>
       </c>
       <c r="R176" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S176" s="3" t="inlineStr"/>
       <c r="T176" s="3" t="inlineStr"/>
@@ -13618,7 +13618,7 @@
         <v>3375</v>
       </c>
       <c r="R177" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S177" s="3" t="inlineStr"/>
       <c r="T177" s="3" t="inlineStr"/>
@@ -13692,7 +13692,7 @@
         <v>3395</v>
       </c>
       <c r="R178" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S178" s="3" t="inlineStr"/>
       <c r="T178" s="3" t="inlineStr"/>
@@ -13766,7 +13766,7 @@
         <v>2285</v>
       </c>
       <c r="R179" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S179" s="3" t="inlineStr"/>
       <c r="T179" s="3" t="inlineStr"/>
@@ -13840,7 +13840,7 @@
         <v>2305</v>
       </c>
       <c r="R180" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S180" s="3" t="inlineStr"/>
       <c r="T180" s="3" t="inlineStr"/>
@@ -13914,7 +13914,7 @@
         <v>2325</v>
       </c>
       <c r="R181" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S181" s="3" t="inlineStr"/>
       <c r="T181" s="3" t="inlineStr"/>
@@ -13988,7 +13988,7 @@
         <v>2345</v>
       </c>
       <c r="R182" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S182" s="3" t="inlineStr"/>
       <c r="T182" s="3" t="inlineStr"/>
@@ -14062,7 +14062,7 @@
         <v>2115</v>
       </c>
       <c r="R183" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S183" s="3" t="inlineStr"/>
       <c r="T183" s="3" t="inlineStr"/>
@@ -14136,7 +14136,7 @@
         <v>2135</v>
       </c>
       <c r="R184" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S184" s="3" t="inlineStr"/>
       <c r="T184" s="3" t="inlineStr"/>
@@ -14210,7 +14210,7 @@
         <v>2645</v>
       </c>
       <c r="R185" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S185" s="3" t="inlineStr"/>
       <c r="T185" s="3" t="inlineStr"/>
@@ -14284,7 +14284,7 @@
         <v>2665</v>
       </c>
       <c r="R186" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S186" s="3" t="inlineStr"/>
       <c r="T186" s="3" t="inlineStr"/>
@@ -14358,7 +14358,7 @@
         <v>2095</v>
       </c>
       <c r="R187" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S187" s="3" t="inlineStr"/>
       <c r="T187" s="3" t="inlineStr"/>
@@ -14432,7 +14432,7 @@
         <v>2115</v>
       </c>
       <c r="R188" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S188" s="3" t="inlineStr"/>
       <c r="T188" s="3" t="inlineStr"/>
@@ -14506,7 +14506,7 @@
         <v>2135</v>
       </c>
       <c r="R189" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S189" s="3" t="inlineStr"/>
       <c r="T189" s="3" t="inlineStr"/>
@@ -14580,7 +14580,7 @@
         <v>3115</v>
       </c>
       <c r="R190" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S190" s="3" t="inlineStr"/>
       <c r="T190" s="3" t="inlineStr"/>
@@ -14654,7 +14654,7 @@
         <v>3135</v>
       </c>
       <c r="R191" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S191" s="3" t="inlineStr"/>
       <c r="T191" s="3" t="inlineStr"/>
@@ -14728,7 +14728,7 @@
         <v>3155</v>
       </c>
       <c r="R192" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S192" s="3" t="inlineStr"/>
       <c r="T192" s="3" t="inlineStr"/>
@@ -14802,7 +14802,7 @@
         <v>1845</v>
       </c>
       <c r="R193" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S193" s="3" t="inlineStr"/>
       <c r="T193" s="3" t="inlineStr"/>
@@ -14876,7 +14876,7 @@
         <v>1865</v>
       </c>
       <c r="R194" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S194" s="3" t="inlineStr"/>
       <c r="T194" s="3" t="inlineStr"/>
@@ -14950,7 +14950,7 @@
         <v>3380</v>
       </c>
       <c r="R195" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S195" s="3" t="inlineStr"/>
       <c r="T195" s="3" t="inlineStr"/>
@@ -15024,7 +15024,7 @@
         <v>3400</v>
       </c>
       <c r="R196" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S196" s="3" t="inlineStr"/>
       <c r="T196" s="3" t="inlineStr"/>
@@ -15098,7 +15098,7 @@
         <v>3420</v>
       </c>
       <c r="R197" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S197" s="3" t="inlineStr"/>
       <c r="T197" s="3" t="inlineStr"/>
@@ -15172,7 +15172,7 @@
         <v>2345</v>
       </c>
       <c r="R198" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S198" s="3" t="inlineStr"/>
       <c r="T198" s="3" t="inlineStr"/>
@@ -15246,7 +15246,7 @@
         <v>1815</v>
       </c>
       <c r="R199" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S199" s="3" t="inlineStr"/>
       <c r="T199" s="3" t="inlineStr"/>
@@ -15320,7 +15320,7 @@
         <v>1835</v>
       </c>
       <c r="R200" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S200" s="3" t="inlineStr"/>
       <c r="T200" s="3" t="inlineStr"/>
@@ -15394,7 +15394,7 @@
         <v>1855</v>
       </c>
       <c r="R201" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr"/>
@@ -15468,7 +15468,7 @@
         <v>1875</v>
       </c>
       <c r="R202" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S202" s="3" t="inlineStr"/>
       <c r="T202" s="3" t="inlineStr"/>
@@ -15542,7 +15542,7 @@
         <v>2760</v>
       </c>
       <c r="R203" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S203" s="3" t="inlineStr"/>
       <c r="T203" s="3" t="inlineStr"/>
@@ -15616,7 +15616,7 @@
         <v>2780</v>
       </c>
       <c r="R204" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S204" s="3" t="inlineStr"/>
       <c r="T204" s="3" t="inlineStr"/>
@@ -15690,7 +15690,7 @@
         <v>2755</v>
       </c>
       <c r="R205" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S205" s="3" t="inlineStr"/>
       <c r="T205" s="3" t="inlineStr"/>
@@ -15764,7 +15764,7 @@
         <v>2765</v>
       </c>
       <c r="R206" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S206" s="3" t="inlineStr"/>
       <c r="T206" s="3" t="inlineStr"/>
@@ -15838,7 +15838,7 @@
         <v>2775</v>
       </c>
       <c r="R207" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S207" s="3" t="inlineStr"/>
       <c r="T207" s="3" t="inlineStr"/>
@@ -15912,7 +15912,7 @@
         <v>2785</v>
       </c>
       <c r="R208" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S208" s="3" t="inlineStr"/>
       <c r="T208" s="3" t="inlineStr"/>
@@ -15986,7 +15986,7 @@
         <v>2795</v>
       </c>
       <c r="R209" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S209" s="3" t="inlineStr"/>
       <c r="T209" s="3" t="inlineStr"/>
@@ -16060,7 +16060,7 @@
         <v>2805</v>
       </c>
       <c r="R210" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S210" s="3" t="inlineStr"/>
       <c r="T210" s="3" t="inlineStr"/>
@@ -16134,7 +16134,7 @@
         <v>2815</v>
       </c>
       <c r="R211" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S211" s="3" t="inlineStr"/>
       <c r="T211" s="3" t="inlineStr"/>
@@ -16208,7 +16208,7 @@
         <v>2825</v>
       </c>
       <c r="R212" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S212" s="3" t="inlineStr"/>
       <c r="T212" s="3" t="inlineStr"/>
@@ -16282,7 +16282,7 @@
         <v>2835</v>
       </c>
       <c r="R213" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S213" s="3" t="inlineStr"/>
       <c r="T213" s="3" t="inlineStr"/>
@@ -16356,7 +16356,7 @@
         <v>2845</v>
       </c>
       <c r="R214" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S214" s="3" t="inlineStr"/>
       <c r="T214" s="3" t="inlineStr"/>
@@ -16430,7 +16430,7 @@
         <v>1795</v>
       </c>
       <c r="R215" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S215" s="3" t="inlineStr"/>
       <c r="T215" s="3" t="inlineStr"/>
@@ -16504,7 +16504,7 @@
         <v>1815</v>
       </c>
       <c r="R216" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S216" s="3" t="inlineStr"/>
       <c r="T216" s="3" t="inlineStr"/>
@@ -16578,7 +16578,7 @@
         <v>1835</v>
       </c>
       <c r="R217" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S217" s="3" t="inlineStr"/>
       <c r="T217" s="3" t="inlineStr"/>
@@ -16652,7 +16652,7 @@
         <v>3145</v>
       </c>
       <c r="R218" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S218" s="3" t="inlineStr"/>
       <c r="T218" s="3" t="inlineStr"/>
@@ -16726,7 +16726,7 @@
         <v>885</v>
       </c>
       <c r="R219" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S219" s="3" t="inlineStr"/>
       <c r="T219" s="3" t="inlineStr"/>
@@ -16800,7 +16800,7 @@
         <v>2065</v>
       </c>
       <c r="R220" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S220" s="3" t="inlineStr"/>
       <c r="T220" s="3" t="inlineStr"/>
@@ -16874,7 +16874,7 @@
         <v>2085</v>
       </c>
       <c r="R221" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S221" s="3" t="inlineStr"/>
       <c r="T221" s="3" t="inlineStr"/>
@@ -16948,7 +16948,7 @@
         <v>2105</v>
       </c>
       <c r="R222" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S222" s="3" t="inlineStr"/>
       <c r="T222" s="3" t="inlineStr"/>
@@ -17022,7 +17022,7 @@
         <v>2925</v>
       </c>
       <c r="R223" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S223" s="3" t="inlineStr"/>
       <c r="T223" s="3" t="inlineStr"/>
@@ -17096,7 +17096,7 @@
         <v>2945</v>
       </c>
       <c r="R224" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S224" s="3" t="inlineStr"/>
       <c r="T224" s="3" t="inlineStr"/>
@@ -17170,7 +17170,7 @@
         <v>2060</v>
       </c>
       <c r="R225" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S225" s="3" t="inlineStr"/>
       <c r="T225" s="3" t="inlineStr"/>
@@ -17244,7 +17244,7 @@
         <v>2080</v>
       </c>
       <c r="R226" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S226" s="3" t="inlineStr"/>
       <c r="T226" s="3" t="inlineStr"/>
@@ -17318,7 +17318,7 @@
         <v>2100</v>
       </c>
       <c r="R227" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S227" s="3" t="inlineStr"/>
       <c r="T227" s="3" t="inlineStr"/>
@@ -17392,7 +17392,7 @@
         <v>2120</v>
       </c>
       <c r="R228" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S228" s="3" t="inlineStr"/>
       <c r="T228" s="3" t="inlineStr"/>
@@ -17466,7 +17466,7 @@
         <v>2460</v>
       </c>
       <c r="R229" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S229" s="3" t="inlineStr"/>
       <c r="T229" s="3" t="inlineStr"/>
@@ -17540,7 +17540,7 @@
         <v>2480</v>
       </c>
       <c r="R230" s="3" t="n">
-        <v>9999</v>
+        <v>12</v>
       </c>
       <c r="S230" s="3" t="inlineStr"/>
       <c r="T230" s="3" t="inlineStr"/>
@@ -17614,7 +17614,7 @@
         <v>2795</v>
       </c>
       <c r="R231" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S231" s="3" t="inlineStr"/>
       <c r="T231" s="3" t="inlineStr"/>
@@ -17688,7 +17688,7 @@
         <v>2815</v>
       </c>
       <c r="R232" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S232" s="3" t="inlineStr"/>
       <c r="T232" s="3" t="inlineStr"/>
@@ -17762,7 +17762,7 @@
         <v>830</v>
       </c>
       <c r="R233" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S233" s="3" t="inlineStr"/>
       <c r="T233" s="3" t="inlineStr"/>
@@ -17836,7 +17836,7 @@
         <v>840</v>
       </c>
       <c r="R234" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S234" s="3" t="inlineStr"/>
       <c r="T234" s="3" t="inlineStr"/>
@@ -17910,7 +17910,7 @@
         <v>2640</v>
       </c>
       <c r="R235" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S235" s="3" t="inlineStr"/>
       <c r="T235" s="3" t="inlineStr"/>
@@ -17984,7 +17984,7 @@
         <v>2750</v>
       </c>
       <c r="R236" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S236" s="3" t="inlineStr"/>
       <c r="T236" s="3" t="inlineStr"/>
@@ -18058,7 +18058,7 @@
         <v>2770</v>
       </c>
       <c r="R237" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S237" s="3" t="inlineStr"/>
       <c r="T237" s="3" t="inlineStr"/>
@@ -18132,7 +18132,7 @@
         <v>2790</v>
       </c>
       <c r="R238" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S238" s="3" t="inlineStr"/>
       <c r="T238" s="3" t="inlineStr"/>
@@ -18206,7 +18206,7 @@
         <v>2735</v>
       </c>
       <c r="R239" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S239" s="3" t="inlineStr"/>
       <c r="T239" s="3" t="inlineStr"/>
@@ -18280,7 +18280,7 @@
         <v>2755</v>
       </c>
       <c r="R240" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S240" s="3" t="inlineStr"/>
       <c r="T240" s="3" t="inlineStr"/>
@@ -18354,7 +18354,7 @@
         <v>1830</v>
       </c>
       <c r="R241" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S241" s="3" t="inlineStr"/>
       <c r="T241" s="3" t="inlineStr"/>
@@ -18428,7 +18428,7 @@
         <v>2760</v>
       </c>
       <c r="R242" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S242" s="3" t="inlineStr"/>
       <c r="T242" s="3" t="inlineStr"/>
@@ -18502,7 +18502,7 @@
         <v>2590</v>
       </c>
       <c r="R243" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S243" s="3" t="inlineStr"/>
       <c r="T243" s="3" t="inlineStr"/>
@@ -18576,7 +18576,7 @@
         <v>2610</v>
       </c>
       <c r="R244" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S244" s="3" t="inlineStr"/>
       <c r="T244" s="3" t="inlineStr"/>
@@ -18650,7 +18650,7 @@
         <v>1615</v>
       </c>
       <c r="R245" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S245" s="3" t="inlineStr"/>
       <c r="T245" s="3" t="inlineStr"/>
@@ -18724,7 +18724,7 @@
         <v>1635</v>
       </c>
       <c r="R246" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S246" s="3" t="inlineStr"/>
       <c r="T246" s="3" t="inlineStr"/>
@@ -18798,7 +18798,7 @@
         <v>1655</v>
       </c>
       <c r="R247" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S247" s="3" t="inlineStr"/>
       <c r="T247" s="3" t="inlineStr"/>
@@ -18872,7 +18872,7 @@
         <v>1675</v>
       </c>
       <c r="R248" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S248" s="3" t="inlineStr"/>
       <c r="T248" s="3" t="inlineStr"/>
@@ -18946,7 +18946,7 @@
         <v>3055</v>
       </c>
       <c r="R249" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S249" s="3" t="inlineStr"/>
       <c r="T249" s="3" t="inlineStr"/>
@@ -19020,7 +19020,7 @@
         <v>3075</v>
       </c>
       <c r="R250" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S250" s="3" t="inlineStr"/>
       <c r="T250" s="3" t="inlineStr"/>
@@ -19094,7 +19094,7 @@
         <v>1795</v>
       </c>
       <c r="R251" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S251" s="3" t="inlineStr"/>
       <c r="T251" s="3" t="inlineStr"/>
@@ -19168,7 +19168,7 @@
         <v>1815</v>
       </c>
       <c r="R252" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S252" s="3" t="inlineStr"/>
       <c r="T252" s="3" t="inlineStr"/>
@@ -19242,7 +19242,7 @@
         <v>2035</v>
       </c>
       <c r="R253" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S253" s="3" t="inlineStr"/>
       <c r="T253" s="3" t="inlineStr"/>
@@ -19316,7 +19316,7 @@
         <v>1790</v>
       </c>
       <c r="R254" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S254" s="3" t="inlineStr"/>
       <c r="T254" s="3" t="inlineStr"/>
@@ -19390,7 +19390,7 @@
         <v>1810</v>
       </c>
       <c r="R255" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S255" s="3" t="inlineStr"/>
       <c r="T255" s="3" t="inlineStr"/>
@@ -19464,7 +19464,7 @@
         <v>1830</v>
       </c>
       <c r="R256" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S256" s="3" t="inlineStr"/>
       <c r="T256" s="3" t="inlineStr"/>
@@ -19538,7 +19538,7 @@
         <v>2580</v>
       </c>
       <c r="R257" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S257" s="3" t="inlineStr"/>
       <c r="T257" s="3" t="inlineStr"/>
@@ -19612,7 +19612,7 @@
         <v>2600</v>
       </c>
       <c r="R258" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S258" s="3" t="inlineStr"/>
       <c r="T258" s="3" t="inlineStr"/>
@@ -19686,7 +19686,7 @@
         <v>2620</v>
       </c>
       <c r="R259" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S259" s="3" t="inlineStr"/>
       <c r="T259" s="3" t="inlineStr"/>
@@ -19760,7 +19760,7 @@
         <v>2640</v>
       </c>
       <c r="R260" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S260" s="3" t="inlineStr"/>
       <c r="T260" s="3" t="inlineStr"/>
@@ -19834,7 +19834,7 @@
         <v>2290</v>
       </c>
       <c r="R261" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S261" s="3" t="inlineStr"/>
       <c r="T261" s="3" t="inlineStr"/>
@@ -19908,7 +19908,7 @@
         <v>2725</v>
       </c>
       <c r="R262" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S262" s="3" t="inlineStr"/>
       <c r="T262" s="3" t="inlineStr"/>
@@ -19982,7 +19982,7 @@
         <v>2745</v>
       </c>
       <c r="R263" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S263" s="3" t="inlineStr"/>
       <c r="T263" s="3" t="inlineStr"/>
@@ -20056,7 +20056,7 @@
         <v>3100</v>
       </c>
       <c r="R264" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S264" s="3" t="inlineStr"/>
       <c r="T264" s="3" t="inlineStr"/>
@@ -20130,7 +20130,7 @@
         <v>3100</v>
       </c>
       <c r="R265" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S265" s="3" t="inlineStr"/>
       <c r="T265" s="3" t="inlineStr"/>
@@ -20204,7 +20204,7 @@
         <v>3120</v>
       </c>
       <c r="R266" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S266" s="3" t="inlineStr"/>
       <c r="T266" s="3" t="inlineStr"/>
@@ -20278,7 +20278,7 @@
         <v>1675</v>
       </c>
       <c r="R267" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S267" s="3" t="inlineStr"/>
       <c r="T267" s="3" t="inlineStr"/>
@@ -20352,7 +20352,7 @@
         <v>2385</v>
       </c>
       <c r="R268" s="3" t="n">
-        <v>9999</v>
+        <v>40</v>
       </c>
       <c r="S268" s="3" t="inlineStr"/>
       <c r="T268" s="3" t="inlineStr"/>
@@ -20426,7 +20426,7 @@
         <v>1495</v>
       </c>
       <c r="R269" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S269" s="3" t="inlineStr"/>
       <c r="T269" s="3" t="inlineStr"/>
@@ -20500,7 +20500,7 @@
         <v>1515</v>
       </c>
       <c r="R270" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S270" s="3" t="inlineStr"/>
       <c r="T270" s="3" t="inlineStr"/>
@@ -20574,7 +20574,7 @@
         <v>1535</v>
       </c>
       <c r="R271" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S271" s="3" t="inlineStr"/>
       <c r="T271" s="3" t="inlineStr"/>
@@ -20648,7 +20648,7 @@
         <v>1555</v>
       </c>
       <c r="R272" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S272" s="3" t="inlineStr"/>
       <c r="T272" s="3" t="inlineStr"/>
@@ -20722,7 +20722,7 @@
         <v>1575</v>
       </c>
       <c r="R273" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S273" s="3" t="inlineStr"/>
       <c r="T273" s="3" t="inlineStr"/>
@@ -20796,7 +20796,7 @@
         <v>1495</v>
       </c>
       <c r="R274" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S274" s="3" t="inlineStr"/>
       <c r="T274" s="3" t="inlineStr"/>
@@ -20870,7 +20870,7 @@
         <v>2005</v>
       </c>
       <c r="R275" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S275" s="3" t="inlineStr"/>
       <c r="T275" s="3" t="inlineStr"/>
@@ -20944,7 +20944,7 @@
         <v>2025</v>
       </c>
       <c r="R276" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S276" s="3" t="inlineStr"/>
       <c r="T276" s="3" t="inlineStr"/>
@@ -21018,7 +21018,7 @@
         <v>2045</v>
       </c>
       <c r="R277" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S277" s="3" t="inlineStr"/>
       <c r="T277" s="3" t="inlineStr"/>
@@ -21092,7 +21092,7 @@
         <v>2750</v>
       </c>
       <c r="R278" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S278" s="3" t="inlineStr"/>
       <c r="T278" s="3" t="inlineStr"/>
@@ -21166,7 +21166,7 @@
         <v>2770</v>
       </c>
       <c r="R279" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S279" s="3" t="inlineStr"/>
       <c r="T279" s="3" t="inlineStr"/>
@@ -21240,7 +21240,7 @@
         <v>785</v>
       </c>
       <c r="R280" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S280" s="3" t="inlineStr"/>
       <c r="T280" s="3" t="inlineStr"/>
@@ -21314,7 +21314,7 @@
         <v>795</v>
       </c>
       <c r="R281" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S281" s="3" t="inlineStr"/>
       <c r="T281" s="3" t="inlineStr"/>
@@ -21388,7 +21388,7 @@
         <v>805</v>
       </c>
       <c r="R282" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S282" s="3" t="inlineStr"/>
       <c r="T282" s="3" t="inlineStr"/>
@@ -21462,7 +21462,7 @@
         <v>2760</v>
       </c>
       <c r="R283" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S283" s="3" t="inlineStr"/>
       <c r="T283" s="3" t="inlineStr"/>
@@ -21536,7 +21536,7 @@
         <v>2780</v>
       </c>
       <c r="R284" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S284" s="3" t="inlineStr"/>
       <c r="T284" s="3" t="inlineStr"/>
@@ -21610,7 +21610,7 @@
         <v>2550</v>
       </c>
       <c r="R285" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S285" s="3" t="inlineStr"/>
       <c r="T285" s="3" t="inlineStr"/>
@@ -21684,7 +21684,7 @@
         <v>2570</v>
       </c>
       <c r="R286" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S286" s="3" t="inlineStr"/>
       <c r="T286" s="3" t="inlineStr"/>
@@ -21758,7 +21758,7 @@
         <v>2275</v>
       </c>
       <c r="R287" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S287" s="3" t="inlineStr"/>
       <c r="T287" s="3" t="inlineStr"/>
@@ -21832,7 +21832,7 @@
         <v>2295</v>
       </c>
       <c r="R288" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S288" s="3" t="inlineStr"/>
       <c r="T288" s="3" t="inlineStr"/>
@@ -21906,7 +21906,7 @@
         <v>2315</v>
       </c>
       <c r="R289" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S289" s="3" t="inlineStr"/>
       <c r="T289" s="3" t="inlineStr"/>
@@ -21980,7 +21980,7 @@
         <v>2245</v>
       </c>
       <c r="R290" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S290" s="3" t="inlineStr"/>
       <c r="T290" s="3" t="inlineStr"/>
@@ -22054,7 +22054,7 @@
         <v>700</v>
       </c>
       <c r="R291" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S291" s="3" t="inlineStr"/>
       <c r="T291" s="3" t="inlineStr"/>
@@ -22128,7 +22128,7 @@
         <v>710</v>
       </c>
       <c r="R292" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S292" s="3" t="inlineStr"/>
       <c r="T292" s="3" t="inlineStr"/>
@@ -22202,7 +22202,7 @@
         <v>720</v>
       </c>
       <c r="R293" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S293" s="3" t="inlineStr"/>
       <c r="T293" s="3" t="inlineStr"/>
@@ -22276,7 +22276,7 @@
         <v>730</v>
       </c>
       <c r="R294" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S294" s="3" t="inlineStr"/>
       <c r="T294" s="3" t="inlineStr"/>
@@ -22350,7 +22350,7 @@
         <v>740</v>
       </c>
       <c r="R295" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S295" s="3" t="inlineStr"/>
       <c r="T295" s="3" t="inlineStr"/>
@@ -22424,7 +22424,7 @@
         <v>2510</v>
       </c>
       <c r="R296" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S296" s="3" t="inlineStr"/>
       <c r="T296" s="3" t="inlineStr"/>
@@ -22498,7 +22498,7 @@
         <v>3035</v>
       </c>
       <c r="R297" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S297" s="3" t="inlineStr"/>
       <c r="T297" s="3" t="inlineStr"/>
@@ -22572,7 +22572,7 @@
         <v>2360</v>
       </c>
       <c r="R298" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S298" s="3" t="inlineStr"/>
       <c r="T298" s="3" t="inlineStr"/>
@@ -22646,7 +22646,7 @@
         <v>2380</v>
       </c>
       <c r="R299" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S299" s="3" t="inlineStr"/>
       <c r="T299" s="3" t="inlineStr"/>
@@ -22720,7 +22720,7 @@
         <v>2630</v>
       </c>
       <c r="R300" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S300" s="3" t="inlineStr"/>
       <c r="T300" s="3" t="inlineStr"/>
@@ -22794,7 +22794,7 @@
         <v>2650</v>
       </c>
       <c r="R301" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S301" s="3" t="inlineStr"/>
       <c r="T301" s="3" t="inlineStr"/>
@@ -22868,7 +22868,7 @@
         <v>1500</v>
       </c>
       <c r="R302" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S302" s="3" t="inlineStr"/>
       <c r="T302" s="3" t="inlineStr"/>
@@ -22942,7 +22942,7 @@
         <v>1495</v>
       </c>
       <c r="R303" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S303" s="3" t="inlineStr"/>
       <c r="T303" s="3" t="inlineStr"/>
@@ -23016,7 +23016,7 @@
         <v>1515</v>
       </c>
       <c r="R304" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S304" s="3" t="inlineStr"/>
       <c r="T304" s="3" t="inlineStr"/>
@@ -23090,7 +23090,7 @@
         <v>1535</v>
       </c>
       <c r="R305" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S305" s="3" t="inlineStr"/>
       <c r="T305" s="3" t="inlineStr"/>
@@ -23164,7 +23164,7 @@
         <v>670</v>
       </c>
       <c r="R306" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S306" s="3" t="inlineStr"/>
       <c r="T306" s="3" t="inlineStr"/>
@@ -23238,7 +23238,7 @@
         <v>680</v>
       </c>
       <c r="R307" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S307" s="3" t="inlineStr"/>
       <c r="T307" s="3" t="inlineStr"/>
@@ -23312,7 +23312,7 @@
         <v>670</v>
       </c>
       <c r="R308" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S308" s="3" t="inlineStr"/>
       <c r="T308" s="3" t="inlineStr"/>
@@ -23386,7 +23386,7 @@
         <v>680</v>
       </c>
       <c r="R309" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S309" s="3" t="inlineStr"/>
       <c r="T309" s="3" t="inlineStr"/>
@@ -23460,7 +23460,7 @@
         <v>1370</v>
       </c>
       <c r="R310" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S310" s="3" t="inlineStr"/>
       <c r="T310" s="3" t="inlineStr"/>
@@ -23534,7 +23534,7 @@
         <v>1390</v>
       </c>
       <c r="R311" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S311" s="3" t="inlineStr"/>
       <c r="T311" s="3" t="inlineStr"/>
@@ -23608,7 +23608,7 @@
         <v>1410</v>
       </c>
       <c r="R312" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S312" s="3" t="inlineStr"/>
       <c r="T312" s="3" t="inlineStr"/>
@@ -23682,7 +23682,7 @@
         <v>1430</v>
       </c>
       <c r="R313" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S313" s="3" t="inlineStr"/>
       <c r="T313" s="3" t="inlineStr"/>
@@ -23756,7 +23756,7 @@
         <v>1450</v>
       </c>
       <c r="R314" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S314" s="3" t="inlineStr"/>
       <c r="T314" s="3" t="inlineStr"/>
@@ -23830,7 +23830,7 @@
         <v>1470</v>
       </c>
       <c r="R315" s="3" t="n">
-        <v>9999</v>
+        <v>28</v>
       </c>
       <c r="S315" s="3" t="inlineStr"/>
       <c r="T315" s="3" t="inlineStr"/>
@@ -23904,7 +23904,7 @@
         <v>1355</v>
       </c>
       <c r="R316" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S316" s="3" t="inlineStr"/>
       <c r="T316" s="3" t="inlineStr"/>
@@ -23978,7 +23978,7 @@
         <v>1375</v>
       </c>
       <c r="R317" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S317" s="3" t="inlineStr"/>
       <c r="T317" s="3" t="inlineStr"/>
@@ -24052,7 +24052,7 @@
         <v>1395</v>
       </c>
       <c r="R318" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S318" s="3" t="inlineStr"/>
       <c r="T318" s="3" t="inlineStr"/>
@@ -24126,7 +24126,7 @@
         <v>1415</v>
       </c>
       <c r="R319" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S319" s="3" t="inlineStr"/>
       <c r="T319" s="3" t="inlineStr"/>
@@ -24200,7 +24200,7 @@
         <v>1435</v>
       </c>
       <c r="R320" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S320" s="3" t="inlineStr"/>
       <c r="T320" s="3" t="inlineStr"/>
@@ -24274,7 +24274,7 @@
         <v>1355</v>
       </c>
       <c r="R321" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S321" s="3" t="inlineStr"/>
       <c r="T321" s="3" t="inlineStr"/>
@@ -24348,7 +24348,7 @@
         <v>1375</v>
       </c>
       <c r="R322" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S322" s="3" t="inlineStr"/>
       <c r="T322" s="3" t="inlineStr"/>
@@ -24422,7 +24422,7 @@
         <v>1395</v>
       </c>
       <c r="R323" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S323" s="3" t="inlineStr"/>
       <c r="T323" s="3" t="inlineStr"/>
@@ -24496,7 +24496,7 @@
         <v>920</v>
       </c>
       <c r="R324" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S324" s="3" t="inlineStr"/>
       <c r="T324" s="3" t="inlineStr"/>
@@ -24570,7 +24570,7 @@
         <v>1335</v>
       </c>
       <c r="R325" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S325" s="3" t="inlineStr"/>
       <c r="T325" s="3" t="inlineStr"/>
@@ -24644,7 +24644,7 @@
         <v>1355</v>
       </c>
       <c r="R326" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S326" s="3" t="inlineStr"/>
       <c r="T326" s="3" t="inlineStr"/>
@@ -24718,7 +24718,7 @@
         <v>1375</v>
       </c>
       <c r="R327" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S327" s="3" t="inlineStr"/>
       <c r="T327" s="3" t="inlineStr"/>
@@ -24792,7 +24792,7 @@
         <v>1395</v>
       </c>
       <c r="R328" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S328" s="3" t="inlineStr"/>
       <c r="T328" s="3" t="inlineStr"/>
@@ -24866,7 +24866,7 @@
         <v>1415</v>
       </c>
       <c r="R329" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S329" s="3" t="inlineStr"/>
       <c r="T329" s="3" t="inlineStr"/>
@@ -24940,7 +24940,7 @@
         <v>965</v>
       </c>
       <c r="R330" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S330" s="3" t="inlineStr"/>
       <c r="T330" s="3" t="inlineStr"/>
@@ -25014,7 +25014,7 @@
         <v>975</v>
       </c>
       <c r="R331" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S331" s="3" t="inlineStr"/>
       <c r="T331" s="3" t="inlineStr"/>
@@ -25088,7 +25088,7 @@
         <v>985</v>
       </c>
       <c r="R332" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S332" s="3" t="inlineStr"/>
       <c r="T332" s="3" t="inlineStr"/>
@@ -25162,7 +25162,7 @@
         <v>905</v>
       </c>
       <c r="R333" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S333" s="3" t="inlineStr"/>
       <c r="T333" s="3" t="inlineStr"/>
@@ -25236,7 +25236,7 @@
         <v>915</v>
       </c>
       <c r="R334" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S334" s="3" t="inlineStr"/>
       <c r="T334" s="3" t="inlineStr"/>
@@ -25310,7 +25310,7 @@
         <v>925</v>
       </c>
       <c r="R335" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S335" s="3" t="inlineStr"/>
       <c r="T335" s="3" t="inlineStr"/>
@@ -25384,7 +25384,7 @@
         <v>1385</v>
       </c>
       <c r="R336" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S336" s="3" t="inlineStr"/>
       <c r="T336" s="3" t="inlineStr"/>
@@ -25458,7 +25458,7 @@
         <v>1405</v>
       </c>
       <c r="R337" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S337" s="3" t="inlineStr"/>
       <c r="T337" s="3" t="inlineStr"/>
@@ -25532,7 +25532,7 @@
         <v>905</v>
       </c>
       <c r="R338" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S338" s="3" t="inlineStr"/>
       <c r="T338" s="3" t="inlineStr"/>
@@ -25606,7 +25606,7 @@
         <v>650</v>
       </c>
       <c r="R339" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S339" s="3" t="inlineStr"/>
       <c r="T339" s="3" t="inlineStr"/>
@@ -25680,7 +25680,7 @@
         <v>660</v>
       </c>
       <c r="R340" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S340" s="3" t="inlineStr"/>
       <c r="T340" s="3" t="inlineStr"/>
@@ -25754,7 +25754,7 @@
         <v>670</v>
       </c>
       <c r="R341" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S341" s="3" t="inlineStr"/>
       <c r="T341" s="3" t="inlineStr"/>
@@ -25828,7 +25828,7 @@
         <v>600</v>
       </c>
       <c r="R342" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S342" s="3" t="inlineStr"/>
       <c r="T342" s="3" t="inlineStr"/>
@@ -25902,7 +25902,7 @@
         <v>610</v>
       </c>
       <c r="R343" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S343" s="3" t="inlineStr"/>
       <c r="T343" s="3" t="inlineStr"/>
@@ -25976,7 +25976,7 @@
         <v>620</v>
       </c>
       <c r="R344" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S344" s="3" t="inlineStr"/>
       <c r="T344" s="3" t="inlineStr"/>
@@ -26050,7 +26050,7 @@
         <v>630</v>
       </c>
       <c r="R345" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S345" s="3" t="inlineStr"/>
       <c r="T345" s="3" t="inlineStr"/>
@@ -26124,7 +26124,7 @@
         <v>640</v>
       </c>
       <c r="R346" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S346" s="3" t="inlineStr"/>
       <c r="T346" s="3" t="inlineStr"/>
@@ -26198,7 +26198,7 @@
         <v>625</v>
       </c>
       <c r="R347" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S347" s="3" t="inlineStr"/>
       <c r="T347" s="3" t="inlineStr"/>
@@ -26272,7 +26272,7 @@
         <v>635</v>
       </c>
       <c r="R348" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S348" s="3" t="inlineStr"/>
       <c r="T348" s="3" t="inlineStr"/>
@@ -26346,7 +26346,7 @@
         <v>645</v>
       </c>
       <c r="R349" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S349" s="3" t="inlineStr"/>
       <c r="T349" s="3" t="inlineStr"/>
@@ -26416,7 +26416,7 @@
       </c>
       <c r="Q350" s="3" t="inlineStr"/>
       <c r="R350" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S350" s="3" t="inlineStr">
         <is>
@@ -26490,7 +26490,7 @@
       </c>
       <c r="Q351" s="3" t="inlineStr"/>
       <c r="R351" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S351" s="3" t="inlineStr">
         <is>
@@ -26564,7 +26564,7 @@
       </c>
       <c r="Q352" s="3" t="inlineStr"/>
       <c r="R352" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S352" s="3" t="inlineStr">
         <is>
@@ -26638,7 +26638,7 @@
       </c>
       <c r="Q353" s="3" t="inlineStr"/>
       <c r="R353" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S353" s="3" t="inlineStr">
         <is>
@@ -26712,7 +26712,7 @@
       </c>
       <c r="Q354" s="3" t="inlineStr"/>
       <c r="R354" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S354" s="3" t="inlineStr">
         <is>
@@ -26786,7 +26786,7 @@
       </c>
       <c r="Q355" s="3" t="inlineStr"/>
       <c r="R355" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S355" s="3" t="inlineStr">
         <is>
@@ -26860,7 +26860,7 @@
       </c>
       <c r="Q356" s="3" t="inlineStr"/>
       <c r="R356" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S356" s="3" t="inlineStr">
         <is>
@@ -26934,7 +26934,7 @@
       </c>
       <c r="Q357" s="3" t="inlineStr"/>
       <c r="R357" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S357" s="3" t="inlineStr">
         <is>
@@ -27008,7 +27008,7 @@
       </c>
       <c r="Q358" s="3" t="inlineStr"/>
       <c r="R358" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S358" s="3" t="inlineStr">
         <is>
@@ -27082,7 +27082,7 @@
       </c>
       <c r="Q359" s="3" t="inlineStr"/>
       <c r="R359" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S359" s="3" t="inlineStr">
         <is>
@@ -27156,7 +27156,7 @@
       </c>
       <c r="Q360" s="3" t="inlineStr"/>
       <c r="R360" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S360" s="3" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
       </c>
       <c r="Q361" s="3" t="inlineStr"/>
       <c r="R361" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S361" s="3" t="inlineStr">
         <is>
@@ -27304,7 +27304,7 @@
       </c>
       <c r="Q362" s="3" t="inlineStr"/>
       <c r="R362" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S362" s="3" t="inlineStr">
         <is>
@@ -27378,7 +27378,7 @@
       </c>
       <c r="Q363" s="3" t="inlineStr"/>
       <c r="R363" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S363" s="3" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
       </c>
       <c r="Q364" s="3" t="inlineStr"/>
       <c r="R364" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S364" s="3" t="inlineStr">
         <is>
@@ -27526,7 +27526,7 @@
       </c>
       <c r="Q365" s="3" t="inlineStr"/>
       <c r="R365" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S365" s="3" t="inlineStr">
         <is>
@@ -27600,7 +27600,7 @@
       </c>
       <c r="Q366" s="3" t="inlineStr"/>
       <c r="R366" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S366" s="3" t="inlineStr">
         <is>
@@ -27674,7 +27674,7 @@
       </c>
       <c r="Q367" s="3" t="inlineStr"/>
       <c r="R367" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S367" s="3" t="inlineStr">
         <is>
@@ -27748,7 +27748,7 @@
       </c>
       <c r="Q368" s="3" t="inlineStr"/>
       <c r="R368" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S368" s="3" t="inlineStr">
         <is>
@@ -27822,7 +27822,7 @@
       </c>
       <c r="Q369" s="3" t="inlineStr"/>
       <c r="R369" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S369" s="3" t="inlineStr">
         <is>
@@ -27896,7 +27896,7 @@
       </c>
       <c r="Q370" s="3" t="inlineStr"/>
       <c r="R370" s="3" t="n">
-        <v>9999</v>
+        <v>20</v>
       </c>
       <c r="S370" s="3" t="inlineStr">
         <is>
@@ -27970,7 +27970,7 @@
       </c>
       <c r="Q371" s="3" t="inlineStr"/>
       <c r="R371" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S371" s="3" t="inlineStr">
         <is>
@@ -28044,7 +28044,7 @@
       </c>
       <c r="Q372" s="3" t="inlineStr"/>
       <c r="R372" s="3" t="n">
-        <v>9999</v>
+        <v>25</v>
       </c>
       <c r="S372" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Engine output files from background run (partial — run timed out)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -7594,7 +7594,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8778,7 +8778,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8852,7 +8852,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -9000,7 +9000,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10258,7 +10258,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10776,7 +10776,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -11072,7 +11072,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11516,7 +11516,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12108,7 +12108,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12774,7 +12774,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13144,7 +13144,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13292,7 +13292,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13366,7 +13366,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13440,7 +13440,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15808,7 +15808,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15882,7 +15882,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15956,7 +15956,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16178,7 +16178,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16252,7 +16252,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16548,7 +16548,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16844,7 +16844,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16918,7 +16918,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17362,7 +17362,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17732,7 +17732,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17880,7 +17880,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18176,7 +18176,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18250,7 +18250,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18398,7 +18398,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18990,7 +18990,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19730,7 +19730,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -20100,7 +20100,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20174,7 +20174,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20470,7 +20470,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20618,7 +20618,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20766,7 +20766,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20840,7 +20840,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21062,7 +21062,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21136,7 +21136,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21210,7 +21210,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21284,7 +21284,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21358,7 +21358,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21950,7 +21950,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22024,7 +22024,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22172,7 +22172,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22542,7 +22542,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22690,7 +22690,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22912,7 +22912,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22986,7 +22986,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23060,7 +23060,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23208,7 +23208,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23282,7 +23282,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23356,7 +23356,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23504,7 +23504,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23726,7 +23726,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23800,7 +23800,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23874,7 +23874,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23948,7 +23948,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24022,7 +24022,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24170,7 +24170,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24244,7 +24244,7 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
@@ -24392,7 +24392,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24540,7 +24540,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24614,7 +24614,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24688,7 +24688,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24762,7 +24762,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24836,7 +24836,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24910,7 +24910,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -24984,7 +24984,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr">
@@ -25280,7 +25280,7 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
@@ -25354,7 +25354,7 @@
       </c>
       <c r="I336" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J336" s="2" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J337" s="2" t="inlineStr">
@@ -25502,7 +25502,7 @@
       </c>
       <c r="I338" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J338" s="2" t="inlineStr">
@@ -25576,7 +25576,7 @@
       </c>
       <c r="I339" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J339" s="2" t="inlineStr">
@@ -25650,7 +25650,7 @@
       </c>
       <c r="I340" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J340" s="2" t="inlineStr">
@@ -25724,7 +25724,7 @@
       </c>
       <c r="I341" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J341" s="2" t="inlineStr">
@@ -25798,7 +25798,7 @@
       </c>
       <c r="I342" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J342" s="2" t="inlineStr">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J343" s="2" t="inlineStr">
@@ -25946,7 +25946,7 @@
       </c>
       <c r="I344" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J344" s="2" t="inlineStr">
@@ -26020,7 +26020,7 @@
       </c>
       <c r="I345" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J345" s="2" t="inlineStr">
@@ -26094,7 +26094,7 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
@@ -26168,7 +26168,7 @@
       </c>
       <c r="I347" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J347" s="2" t="inlineStr">
@@ -26242,7 +26242,7 @@
       </c>
       <c r="I348" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J348" s="2" t="inlineStr">
@@ -26316,7 +26316,7 @@
       </c>
       <c r="I349" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J349" s="2" t="inlineStr">
@@ -28128,16 +28128,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
@@ -28147,16 +28147,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>7</v>
-      </c>
       <c r="D4" s="3" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -28166,16 +28166,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
@@ -28185,13 +28185,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>54</v>
@@ -28204,16 +28204,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>27</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -28223,16 +28223,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>30</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -29610,7 +29610,7 @@
         <v>5</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>5</v>
@@ -29882,7 +29882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -29933,7 +29933,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -29943,12 +29943,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>130-3</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>130-5</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>132-1</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -29965,7 +29965,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -29975,12 +29975,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>130-3</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>130-5</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>132-1</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -30669,7 +30669,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -30679,7 +30679,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>310-1</t>
+          <t>310-3</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -30701,7 +30701,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -30711,7 +30711,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>310-1</t>
+          <t>310-3</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -31021,7 +31021,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -31031,12 +31031,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>710-1</t>
+          <t>710-2</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>710-2</t>
+          <t>710-3</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -31053,7 +31053,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -31063,12 +31063,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>710-1</t>
+          <t>710-2</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>710-3</t>
+          <t>751-1</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -31085,7 +31085,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -31095,12 +31095,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>710-2</t>
+          <t>710-3</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>710-3</t>
+          <t>751-1</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -31117,7 +31117,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -31127,79 +31127,15 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>710-1</t>
+          <t>710-2</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>710-2</t>
+          <t>710-3</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>NO — CONFLICT</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Saggio, Jack</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>710-1</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>710-3</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>NO — CONFLICT</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Saggio, Jack</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>710-2</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>710-3</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>NO — CONFLICT</t>
         </is>
@@ -31280,7 +31216,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -31301,7 +31237,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>145/348</t>
+          <t>149/348</t>
         </is>
       </c>
     </row>
@@ -31334,7 +31270,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13">
@@ -31344,7 +31280,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14">
@@ -31354,7 +31290,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -31374,7 +31310,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
@@ -31384,7 +31320,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update engine outputs from full run (698 conflicts, 89.3% placement)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -4930,7 +4930,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8334,7 +8334,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8482,7 +8482,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8630,7 +8630,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8778,7 +8778,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -9000,7 +9000,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9370,7 +9370,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9666,7 +9666,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10258,7 +10258,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10554,7 +10554,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11516,7 +11516,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11960,7 +11960,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12108,7 +12108,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12404,7 +12404,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12552,7 +12552,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12774,7 +12774,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13070,7 +13070,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13144,7 +13144,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13292,7 +13292,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13366,7 +13366,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13514,7 +13514,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13588,7 +13588,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13662,7 +13662,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13736,7 +13736,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14180,7 +14180,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14254,7 +14254,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14402,7 +14402,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14476,7 +14476,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15290,7 +15290,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15734,7 +15734,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15808,7 +15808,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16104,7 +16104,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16178,7 +16178,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16252,7 +16252,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16548,7 +16548,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16844,7 +16844,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16992,7 +16992,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17066,7 +17066,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17140,7 +17140,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17288,7 +17288,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17436,7 +17436,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17584,7 +17584,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17732,7 +17732,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17880,7 +17880,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -18028,7 +18028,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18176,7 +18176,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18398,7 +18398,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18472,7 +18472,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18546,7 +18546,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18620,7 +18620,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18990,7 +18990,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19286,7 +19286,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19508,7 +19508,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19656,7 +19656,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19952,7 +19952,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20026,7 +20026,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20100,7 +20100,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20174,7 +20174,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20470,7 +20470,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20618,7 +20618,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20840,7 +20840,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20988,7 +20988,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21062,7 +21062,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21136,7 +21136,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21284,7 +21284,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21358,7 +21358,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21432,7 +21432,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21506,7 +21506,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21580,7 +21580,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21802,7 +21802,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21950,7 +21950,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22024,7 +22024,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22172,7 +22172,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22246,7 +22246,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22394,7 +22394,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22542,7 +22542,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22912,7 +22912,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22986,7 +22986,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23060,7 +23060,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23134,7 +23134,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23208,7 +23208,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23282,7 +23282,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23504,7 +23504,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23726,7 +23726,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23800,7 +23800,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23874,7 +23874,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23948,7 +23948,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24022,7 +24022,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24170,7 +24170,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24244,7 +24244,7 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
@@ -24318,7 +24318,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24614,7 +24614,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24688,7 +24688,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24762,7 +24762,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24836,7 +24836,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24910,7 +24910,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -24984,7 +24984,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -25058,7 +25058,7 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr">
@@ -28045,16 +28045,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>7</v>
-      </c>
       <c r="D2" s="3" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -28064,16 +28064,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
@@ -28083,16 +28083,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -28102,16 +28102,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -28121,16 +28121,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
@@ -28143,13 +28143,13 @@
         <v>10</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>35</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">
@@ -28162,13 +28162,13 @@
         <v>13</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -28418,7 +28418,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>4</v>
@@ -28429,7 +28429,11 @@
       <c r="F9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -28496,7 +28500,7 @@
         <v>4</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>5</v>
@@ -28504,7 +28508,11 @@
       <c r="F12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -29546,7 +29554,7 @@
         <v>5</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>5</v>
@@ -29869,7 +29877,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -29901,7 +29909,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -30605,7 +30613,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -30615,7 +30623,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>310-2</t>
+          <t>310-1</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -30637,7 +30645,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -30647,7 +30655,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>310-2</t>
+          <t>310-1</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -30888,27 +30896,27 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Daniels, Torrence</t>
+          <t>Saggio, Jack</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>620-8</t>
+          <t>710-1</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>631-6</t>
+          <t>710-2</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -30920,12 +30928,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Chiaravalloti, Michael</t>
+          <t>Saggio, Jack</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -30935,12 +30943,12 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>631-1</t>
+          <t>710-1</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>631-3</t>
+          <t>710-3</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -30957,7 +30965,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -30989,22 +30997,22 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
+          <t>710-1</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
           <t>710-2</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>741-1</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -31021,22 +31029,22 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
+          <t>710-1</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>710-3</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>741-1</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -31053,7 +31061,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -31152,7 +31160,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -31162,7 +31170,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -31173,7 +31181,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>167/348</t>
+          <t>155/348</t>
         </is>
       </c>
     </row>
@@ -31196,7 +31204,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -31206,7 +31214,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13">
@@ -31216,7 +31224,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14">
@@ -31226,7 +31234,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15">
@@ -31236,7 +31244,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16">
@@ -31246,7 +31254,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -31256,7 +31264,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Engine output files: gr12 run after room double-booking fix
Results: 197 conflicts (down from 228), 87.5% placement rate
0 teacher double-bookings, 0 room double-bookings, 0 student double-bookings

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -21136,7 +21136,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -28066,10 +28066,10 @@
         <v>6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -28085,10 +28085,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -30902,7 +30902,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13">
@@ -30912,7 +30912,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Job 1 output after EC rebalance fix
Load violations reduced from 5 to 2:
- Umbrino: S1=5/5 S2=5/5 ✓ (was S1=6/5)
- Daniels: S1=5/5 S2=5/5 ✓ (was S2=6/5)
- Chiaravalloti: S1=5/5 S2=5/5 ✓ (was S1=6/5)
- Saggio: S1=5/5 S2=6/5 (was S1=7/5) — needs S2-only 6th approval
- Tuesta: S1=6/5 S2=6/5 (unchanged) — needs both-semester 6th approval

0 teacher double-bookings, 0 room double-bookings

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -2041,7 +2041,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K21" s="3" t="n">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K22" s="3" t="n">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K23" s="3" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K25" s="3" t="n">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -7742,12 +7742,12 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K98" s="3" t="n">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -8038,12 +8038,12 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K102" s="3" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8186,12 +8186,12 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K104" s="3" t="n">
@@ -8482,7 +8482,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -8630,7 +8630,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9666,7 +9666,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9888,7 +9888,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -10480,12 +10480,12 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K135" s="3" t="n">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K142" s="3" t="n">
@@ -11072,7 +11072,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11516,7 +11516,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11960,7 +11960,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12108,7 +12108,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12404,7 +12404,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12552,7 +12552,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12922,7 +12922,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13070,7 +13070,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13440,7 +13440,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13588,7 +13588,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13662,7 +13662,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13810,7 +13810,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14180,7 +14180,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14254,7 +14254,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14402,7 +14402,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14476,7 +14476,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15290,7 +15290,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15364,7 +15364,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15660,7 +15660,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15734,7 +15734,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15882,7 +15882,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15956,7 +15956,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16104,7 +16104,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16252,7 +16252,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16326,12 +16326,12 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K214" s="3" t="n">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16548,7 +16548,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16844,7 +16844,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16918,7 +16918,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16992,7 +16992,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17066,7 +17066,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17140,7 +17140,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17288,7 +17288,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17362,7 +17362,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17584,7 +17584,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17880,7 +17880,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18028,7 +18028,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18176,7 +18176,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18250,7 +18250,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18472,7 +18472,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18620,7 +18620,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18768,7 +18768,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18990,7 +18990,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19286,7 +19286,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19508,7 +19508,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19582,7 +19582,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19656,7 +19656,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19730,7 +19730,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19804,7 +19804,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -20026,7 +20026,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20174,7 +20174,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20470,7 +20470,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20618,7 +20618,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20692,7 +20692,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20766,7 +20766,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20840,7 +20840,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -21062,7 +21062,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21136,7 +21136,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21210,7 +21210,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21284,7 +21284,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21432,7 +21432,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21506,7 +21506,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21580,7 +21580,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21802,7 +21802,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21950,7 +21950,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22024,7 +22024,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22172,7 +22172,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22246,7 +22246,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22394,7 +22394,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22468,7 +22468,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22690,7 +22690,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22838,7 +22838,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22912,7 +22912,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22986,7 +22986,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23060,7 +23060,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23134,7 +23134,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23282,7 +23282,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23356,7 +23356,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23504,7 +23504,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23726,7 +23726,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23800,7 +23800,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23874,7 +23874,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23948,7 +23948,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24022,7 +24022,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24170,7 +24170,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24244,7 +24244,7 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
@@ -24318,7 +24318,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24392,7 +24392,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24540,7 +24540,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24614,7 +24614,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24762,7 +24762,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24910,7 +24910,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -24984,7 +24984,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -25058,7 +25058,7 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr">
@@ -28041,16 +28041,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -28060,16 +28060,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -28079,16 +28079,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -28098,16 +28098,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -28117,13 +28117,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>49</v>
@@ -28136,16 +28136,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -28155,16 +28155,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -28414,10 +28414,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>5</v>
@@ -28425,11 +28425,7 @@
       <c r="F9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -28493,10 +28489,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>5</v>
@@ -28504,11 +28500,7 @@
       <c r="F12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -29147,10 +29139,10 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="2" t="n">
         <v>4</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>3</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>5</v>
@@ -29222,10 +29214,10 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>6</v>
@@ -29547,10 +29539,10 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>5</v>
@@ -29705,10 +29697,10 @@
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>5</v>
@@ -29716,11 +29708,7 @@
       <c r="F60" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="G60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -30858,7 +30846,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -30892,7 +30880,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12">
@@ -30902,7 +30890,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
@@ -30912,7 +30900,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -30922,7 +30910,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15">
@@ -30942,7 +30930,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17">
@@ -30952,7 +30940,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Job 1 output: co-schedule-aware pre-flight, 2 real violations only
Pre-flight now correctly counts co-schedule groups as 1 period slot.
Dennehy (13 sections, 5 S1 period slots after co-schedule) is no
longer a false positive.

Real violations: Saggio (S2=6/5), Tuesta (S1=6/5, S2=6/5)
369/371 sections placed, 0 load violations, 0 double-bookings

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,12 +45,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FF0000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -86,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -96,7 +90,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -22394,7 +22387,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22409,19 +22402,19 @@
         <v>270</v>
       </c>
       <c r="M296" s="3" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="N296" s="3" t="n">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="O296" s="3" t="n">
         <v>30</v>
       </c>
       <c r="P296" s="3" t="n">
-        <v>720</v>
+        <v>710</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>1430</v>
+        <v>1410</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>28</v>
@@ -22542,7 +22535,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22557,10 +22550,10 @@
         <v>275</v>
       </c>
       <c r="M298" s="3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="N298" s="3" t="n">
-        <v>640</v>
+        <v>630</v>
       </c>
       <c r="O298" s="3" t="n">
         <v>0</v>
@@ -22569,7 +22562,7 @@
         <v>0</v>
       </c>
       <c r="Q298" s="3" t="n">
-        <v>935</v>
+        <v>925</v>
       </c>
       <c r="R298" s="3" t="n">
         <v>28</v>
@@ -22838,7 +22831,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22912,7 +22905,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22986,7 +22979,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23060,7 +23053,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23134,7 +23127,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23578,7 +23571,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23652,7 +23645,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23726,7 +23719,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23874,7 +23867,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23948,7 +23941,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24022,7 +24015,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24170,7 +24163,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24244,7 +24237,7 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
@@ -24540,7 +24533,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24614,7 +24607,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24688,7 +24681,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24762,7 +24755,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24836,7 +24829,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24984,7 +24977,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -25058,7 +25051,7 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr">
@@ -26773,10 +26766,10 @@
         <v>275</v>
       </c>
       <c r="M355" s="3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>640</v>
+        <v>630</v>
       </c>
       <c r="O355" s="3" t="n">
         <v>0</v>
@@ -28066,10 +28059,10 @@
         <v>4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -28085,10 +28078,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
@@ -28104,10 +28097,10 @@
         <v>11</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -28123,10 +28116,10 @@
         <v>11</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -28161,10 +28154,10 @@
         <v>7</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -29539,10 +29532,10 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" s="2" t="n">
         <v>5</v>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>6</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>5</v>
@@ -29550,11 +29543,7 @@
       <c r="F54" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="G54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -29668,10 +29657,10 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>5</v>
@@ -29679,11 +29668,7 @@
       <c r="F59" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+      <c r="G59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -30780,167 +30765,167 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Total Sections</t>
         </is>
       </c>
-      <c r="B1" s="7" t="n">
+      <c r="B1" s="6" t="n">
         <v>371</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Sections Assigned</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>371</v>
+      <c r="B2" s="6" t="n">
+        <v>369</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Sections Unassigned</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Total Courses</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Total Teachers</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Teacher Period Conflicts (non-co-sched)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Total Courses</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Total Teachers</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Teacher Period Conflicts (non-co-sched)</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Load Violations</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Load Violations</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Prior-Year Alignment</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>146/348</t>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>147/348</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="7" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Period Distribution</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr"/>
+      <c r="B10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Period A</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="6" t="n">
         <v>58</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Period B</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>49</v>
+      <c r="B12" s="6" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Period C</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="6" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Period D</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Period E</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
         <v>48</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Period D</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Period E</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>49</v>
-      </c>
-    </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Period F</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="6" t="n">
         <v>57</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Period G</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n">
-        <v>48</v>
+      <c r="B17" s="6" t="n">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Scale semester complement bonus for 6-period teachers: floor score to guarantee sharing
For teachers with max_load >= 6, sharing a period between S1/S2 sections
of the same course is a schedulability requirement, not just a preference.
Without sharing, the teacher runs out of period slots and a section becomes
unplaceable. The prior -20 bonus was negligible against Tier 2 conflict
scores (27M-62M range), so 744 Sociology S1/S2 went to separate periods
(F and A), wasting a period slot and trapping Quast's last 711 FY section.

Fix: when max_load >= 6 and a complement (opposite-semester section of the
same course) already occupies the candidate period, floor the score to 1.0
so this period wins decisively. For teachers with normal 5-period loads,
the mild -20 bonus is retained.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -2034,7 +2034,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K21" s="3" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8179,12 +8179,12 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K104" s="3" t="n">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9437,7 +9437,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9807,7 +9807,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9881,7 +9881,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10103,7 +10103,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10325,7 +10325,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10473,7 +10473,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11213,7 +11213,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11287,7 +11287,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11657,7 +11657,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11879,7 +11879,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11953,7 +11953,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12175,7 +12175,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12249,7 +12249,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12471,7 +12471,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12545,7 +12545,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12619,7 +12619,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12841,7 +12841,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12989,7 +12989,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13137,7 +13137,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13211,7 +13211,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13655,7 +13655,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -14099,7 +14099,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14173,7 +14173,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14247,7 +14247,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14543,7 +14543,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14617,7 +14617,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14691,7 +14691,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14765,7 +14765,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14839,7 +14839,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14913,7 +14913,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14987,7 +14987,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15135,7 +15135,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15209,7 +15209,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15283,7 +15283,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15653,7 +15653,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15727,7 +15727,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15949,7 +15949,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16023,7 +16023,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16097,7 +16097,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16245,7 +16245,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16319,7 +16319,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16467,7 +16467,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16541,7 +16541,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16689,7 +16689,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16911,7 +16911,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16985,7 +16985,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17133,7 +17133,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17207,7 +17207,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17281,7 +17281,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17355,7 +17355,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17577,7 +17577,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17651,7 +17651,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17725,7 +17725,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17873,7 +17873,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18095,7 +18095,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18169,7 +18169,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18243,7 +18243,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18391,7 +18391,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18539,7 +18539,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18613,7 +18613,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18761,7 +18761,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18835,7 +18835,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18909,7 +18909,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18983,7 +18983,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19057,7 +19057,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19131,7 +19131,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19205,7 +19205,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19279,7 +19279,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19353,7 +19353,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19427,7 +19427,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19501,7 +19501,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19738,19 +19738,19 @@
         <v>265</v>
       </c>
       <c r="M260" s="3" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>840</v>
+        <v>830</v>
       </c>
       <c r="O260" s="3" t="n">
         <v>35</v>
       </c>
       <c r="P260" s="3" t="n">
-        <v>1540</v>
+        <v>1530</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2665</v>
+        <v>2645</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>28</v>
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20093,7 +20093,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20241,7 +20241,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20315,7 +20315,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20463,7 +20463,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20611,7 +20611,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20685,7 +20685,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20759,7 +20759,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20833,7 +20833,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20907,7 +20907,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21055,7 +21055,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21203,7 +21203,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21277,7 +21277,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21425,7 +21425,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21573,7 +21573,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21647,7 +21647,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21721,7 +21721,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21943,7 +21943,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22091,7 +22091,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22165,7 +22165,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22313,7 +22313,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22387,7 +22387,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22402,19 +22402,19 @@
         <v>270</v>
       </c>
       <c r="M296" s="3" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="N296" s="3" t="n">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="O296" s="3" t="n">
         <v>30</v>
       </c>
       <c r="P296" s="3" t="n">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="Q296" s="3" t="n">
-        <v>1410</v>
+        <v>1430</v>
       </c>
       <c r="R296" s="3" t="n">
         <v>28</v>
@@ -22461,7 +22461,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22535,7 +22535,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22550,10 +22550,10 @@
         <v>275</v>
       </c>
       <c r="M298" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N298" s="3" t="n">
-        <v>630</v>
+        <v>640</v>
       </c>
       <c r="O298" s="3" t="n">
         <v>0</v>
@@ -22562,7 +22562,7 @@
         <v>0</v>
       </c>
       <c r="Q298" s="3" t="n">
-        <v>925</v>
+        <v>935</v>
       </c>
       <c r="R298" s="3" t="n">
         <v>28</v>
@@ -22609,7 +22609,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22757,7 +22757,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22831,7 +22831,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22905,7 +22905,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22979,7 +22979,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23053,7 +23053,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23127,7 +23127,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23275,7 +23275,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23497,7 +23497,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23571,7 +23571,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23645,7 +23645,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23719,7 +23719,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23941,7 +23941,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24015,7 +24015,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24163,7 +24163,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24237,7 +24237,7 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
@@ -24311,7 +24311,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24385,7 +24385,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24533,7 +24533,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24607,7 +24607,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24681,7 +24681,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24829,7 +24829,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24903,7 +24903,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -25051,7 +25051,7 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr">
@@ -26766,10 +26766,10 @@
         <v>275</v>
       </c>
       <c r="M355" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N355" s="3" t="n">
-        <v>630</v>
+        <v>640</v>
       </c>
       <c r="O355" s="3" t="n">
         <v>0</v>
@@ -28034,16 +28034,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>36</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -28056,13 +28056,13 @@
         <v>6</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -28072,16 +28072,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -28094,13 +28094,13 @@
         <v>13</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6">
@@ -28110,16 +28110,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>11</v>
-      </c>
       <c r="D6" s="3" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -28129,16 +28129,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>12</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
@@ -28148,13 +28148,13 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>47</v>
@@ -29457,10 +29457,10 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>6</v>
@@ -29532,16 +29532,16 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>5</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
     </row>
@@ -29657,16 +29657,16 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
     </row>
@@ -30781,7 +30781,7 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3">
@@ -30791,7 +30791,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -30842,7 +30842,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>147/348</t>
+          <t>150/348</t>
         </is>
       </c>
     </row>
@@ -30865,7 +30865,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12">
@@ -30875,7 +30875,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13">
@@ -30885,7 +30885,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -30895,7 +30895,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15">
@@ -30905,7 +30905,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
@@ -30915,7 +30915,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Job 1 output: 371/371 sections placed, 0 violations
All constraints satisfied:
- 371/371 sections assigned (100%)
- 0 teacher period conflicts
- 0 room double-bookings
- 0 load violations
- 0 consecutive-6 violations
- All 6-period teachers have interior free periods

Key placements that were previously problematic:
- Quast 744 Sociology S1/S2 share Period F (complement bonus)
- Quast 711 World History H sec1=C, sec2=G (both placed)
- Saggio 710/723/741/751 all placed within S2=6 cap
- Tuesta 310 Spanish I all 6 sections placed with FY 6th approval

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -4331,7 +4331,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7513,7 +7513,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7661,7 +7661,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9437,7 +9437,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9807,7 +9807,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9881,7 +9881,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10103,7 +10103,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11213,7 +11213,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11287,7 +11287,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11657,7 +11657,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -11879,7 +11879,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11953,7 +11953,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12101,7 +12101,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12175,7 +12175,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12471,7 +12471,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12545,7 +12545,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12619,7 +12619,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12989,7 +12989,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13137,7 +13137,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13211,7 +13211,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13581,7 +13581,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13655,7 +13655,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13951,7 +13951,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14099,7 +14099,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14247,7 +14247,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14469,7 +14469,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14543,7 +14543,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14691,7 +14691,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14839,7 +14839,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14987,7 +14987,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15283,7 +15283,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15653,7 +15653,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15949,7 +15949,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16023,7 +16023,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16097,7 +16097,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16171,7 +16171,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16245,7 +16245,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16319,7 +16319,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16467,7 +16467,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16911,7 +16911,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16985,7 +16985,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17207,7 +17207,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17281,7 +17281,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17429,7 +17429,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17577,7 +17577,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18243,7 +18243,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18317,7 +18317,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18391,7 +18391,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18465,7 +18465,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18539,7 +18539,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18761,7 +18761,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18835,7 +18835,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18909,7 +18909,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -19131,7 +19131,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19279,7 +19279,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19353,7 +19353,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19427,7 +19427,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19501,7 +19501,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19649,7 +19649,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19738,19 +19738,19 @@
         <v>265</v>
       </c>
       <c r="M260" s="3" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="N260" s="3" t="n">
-        <v>830</v>
+        <v>840</v>
       </c>
       <c r="O260" s="3" t="n">
         <v>35</v>
       </c>
       <c r="P260" s="3" t="n">
-        <v>1530</v>
+        <v>1540</v>
       </c>
       <c r="Q260" s="3" t="n">
-        <v>2645</v>
+        <v>2665</v>
       </c>
       <c r="R260" s="3" t="n">
         <v>28</v>
@@ -19871,7 +19871,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19945,7 +19945,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20241,7 +20241,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20389,7 +20389,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20463,7 +20463,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20611,7 +20611,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20685,7 +20685,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20907,7 +20907,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20981,7 +20981,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21055,7 +21055,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21203,7 +21203,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21277,7 +21277,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21425,7 +21425,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21499,7 +21499,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21573,7 +21573,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21647,7 +21647,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22165,7 +22165,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22313,7 +22313,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22535,7 +22535,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22609,7 +22609,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -23053,7 +23053,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23201,7 +23201,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23275,7 +23275,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23349,7 +23349,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23423,7 +23423,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23645,7 +23645,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -23719,7 +23719,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23867,7 +23867,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23941,7 +23941,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24089,7 +24089,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24163,7 +24163,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24237,7 +24237,7 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
@@ -24311,7 +24311,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24385,7 +24385,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24533,7 +24533,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24607,7 +24607,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24681,7 +24681,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24755,7 +24755,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24829,7 +24829,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24977,7 +24977,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -25051,7 +25051,7 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr">
@@ -28034,16 +28034,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -28053,13 +28053,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>46</v>
@@ -28075,13 +28075,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>32</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -28097,10 +28097,10 @@
         <v>12</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -28116,10 +28116,10 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -28129,16 +28129,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8">
@@ -28148,7 +28148,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>8</v>
@@ -28157,7 +28157,7 @@
         <v>30</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -29457,10 +29457,10 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>6</v>
@@ -30781,7 +30781,7 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="3">
@@ -30791,7 +30791,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -30865,7 +30865,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12">
@@ -30885,7 +30885,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
@@ -30895,7 +30895,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15">
@@ -30905,7 +30905,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
@@ -30915,7 +30915,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17">
@@ -30925,7 +30925,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Job 1 re-run: 363/367 placed after Willi room fix
Willi's 3× 410 Algebra I sections now placed in J-020.
Improvement: 360→363 sections placed (+3).

Remaining 4 unplaced (same teacher constraint issues):
- 312 Italian I (Zawiski) — consecutive_6
- 620 Driver's Ed/PE (Daniels) — S1 load cap
- 631 CPR-AED Training/PE (Chiaravalloti) — S2 load cap
- 710 World History (Saggio) — S1 load cap

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1168,16 +1168,16 @@
         <v>5100</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>5910</v>
+        <v>5895</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>6720</v>
+        <v>6690</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>13300</v>
+        <v>13255</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>28</v>
@@ -1242,16 +1242,16 @@
         <v>5110</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>5920</v>
+        <v>5905</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>6730</v>
+        <v>6700</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>13290</v>
+        <v>13245</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>28</v>
@@ -2952,16 +2952,16 @@
         <v>5120</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>5930</v>
+        <v>5915</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>6740</v>
+        <v>6710</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>13405</v>
+        <v>13360</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>28</v>
@@ -6356,16 +6356,16 @@
         <v>5130</v>
       </c>
       <c r="N79" s="3" t="n">
-        <v>5940</v>
+        <v>5925</v>
       </c>
       <c r="O79" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P79" s="3" t="n">
-        <v>6750</v>
+        <v>6720</v>
       </c>
       <c r="Q79" s="3" t="n">
-        <v>13445</v>
+        <v>13400</v>
       </c>
       <c r="R79" s="3" t="n">
         <v>28</v>
@@ -6430,16 +6430,16 @@
         <v>5140</v>
       </c>
       <c r="N80" s="3" t="n">
-        <v>5950</v>
+        <v>5935</v>
       </c>
       <c r="O80" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P80" s="3" t="n">
-        <v>6760</v>
+        <v>6730</v>
       </c>
       <c r="Q80" s="3" t="n">
-        <v>13465</v>
+        <v>13420</v>
       </c>
       <c r="R80" s="3" t="n">
         <v>28</v>
@@ -6504,16 +6504,16 @@
         <v>5150</v>
       </c>
       <c r="N81" s="3" t="n">
-        <v>5960</v>
+        <v>5945</v>
       </c>
       <c r="O81" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P81" s="3" t="n">
-        <v>6770</v>
+        <v>6740</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>13485</v>
+        <v>13440</v>
       </c>
       <c r="R81" s="3" t="n">
         <v>28</v>
@@ -8081,12 +8081,12 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>713</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>World History</t>
+          <t>AP World History</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
@@ -8099,22 +8099,22 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Saggio, Jack</t>
+          <t>Quast, Richard</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>117711</t>
+          <t>105651</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>I-117</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8123,25 +8123,25 @@
         </is>
       </c>
       <c r="K103" s="3" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="L103" s="3" t="n">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="M103" s="3" t="n">
-        <v>5160</v>
+        <v>5090</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>5970</v>
+        <v>5950</v>
       </c>
       <c r="O103" s="3" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="P103" s="3" t="n">
-        <v>6780</v>
+        <v>6810</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>13200</v>
+        <v>13275</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>28</v>
@@ -8155,12 +8155,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>713</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>World History</t>
+          <t>AP World History</t>
         </is>
       </c>
       <c r="D104" s="2" t="n">
@@ -8173,22 +8173,22 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Saggio, Jack</t>
+          <t>Quast, Richard</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>117711</t>
+          <t>105651</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>I-117</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8197,25 +8197,25 @@
         </is>
       </c>
       <c r="K104" s="3" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="L104" s="3" t="n">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="M104" s="3" t="n">
-        <v>5170</v>
+        <v>5100</v>
       </c>
       <c r="N104" s="3" t="n">
-        <v>5980</v>
+        <v>5960</v>
       </c>
       <c r="O104" s="3" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="P104" s="3" t="n">
-        <v>6790</v>
+        <v>6820</v>
       </c>
       <c r="Q104" s="3" t="n">
-        <v>13220</v>
+        <v>13295</v>
       </c>
       <c r="R104" s="3" t="n">
         <v>28</v>
@@ -8229,40 +8229,40 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>315</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>World History</t>
+          <t>Latin I H</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Saggio, Jack</t>
+          <t>Zawiski, Brian</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>117711</t>
+          <t>105729</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>S-236</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -8271,25 +8271,25 @@
         </is>
       </c>
       <c r="K105" s="3" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="L105" s="3" t="n">
-        <v>430</v>
+        <v>460</v>
       </c>
       <c r="M105" s="3" t="n">
-        <v>5170</v>
+        <v>5100</v>
       </c>
       <c r="N105" s="3" t="n">
-        <v>5980</v>
+        <v>6045</v>
       </c>
       <c r="O105" s="3" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="P105" s="3" t="n">
-        <v>6790</v>
+        <v>6990</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>13220</v>
+        <v>13540</v>
       </c>
       <c r="R105" s="3" t="n">
         <v>28</v>
@@ -8303,12 +8303,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>710</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>AP World History</t>
+          <t>World History</t>
         </is>
       </c>
       <c r="D106" s="2" t="n">
@@ -8321,22 +8321,22 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Quast, Richard</t>
+          <t>Saggio, Jack</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>105651</t>
+          <t>117711</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8345,25 +8345,25 @@
         </is>
       </c>
       <c r="K106" s="3" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="L106" s="3" t="n">
-        <v>465</v>
+        <v>430</v>
       </c>
       <c r="M106" s="3" t="n">
-        <v>5090</v>
+        <v>5160</v>
       </c>
       <c r="N106" s="3" t="n">
-        <v>5950</v>
+        <v>5955</v>
       </c>
       <c r="O106" s="3" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="P106" s="3" t="n">
-        <v>6810</v>
+        <v>6750</v>
       </c>
       <c r="Q106" s="3" t="n">
-        <v>13275</v>
+        <v>13155</v>
       </c>
       <c r="R106" s="3" t="n">
         <v>28</v>
@@ -8377,12 +8377,12 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>710</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>AP World History</t>
+          <t>World History</t>
         </is>
       </c>
       <c r="D107" s="2" t="n">
@@ -8395,22 +8395,22 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Quast, Richard</t>
+          <t>Saggio, Jack</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>105651</t>
+          <t>117711</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>I-117</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8419,25 +8419,25 @@
         </is>
       </c>
       <c r="K107" s="3" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="L107" s="3" t="n">
-        <v>465</v>
+        <v>430</v>
       </c>
       <c r="M107" s="3" t="n">
-        <v>5100</v>
+        <v>5170</v>
       </c>
       <c r="N107" s="3" t="n">
-        <v>5960</v>
+        <v>5965</v>
       </c>
       <c r="O107" s="3" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="P107" s="3" t="n">
-        <v>6820</v>
+        <v>6760</v>
       </c>
       <c r="Q107" s="3" t="n">
-        <v>13295</v>
+        <v>13175</v>
       </c>
       <c r="R107" s="3" t="n">
         <v>28</v>
@@ -8451,40 +8451,40 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>710</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Latin I H</t>
+          <t>World History</t>
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Zawiski, Brian</t>
+          <t>Saggio, Jack</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>105729</t>
+          <t>117711</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>S-236</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8493,25 +8493,25 @@
         </is>
       </c>
       <c r="K108" s="3" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="L108" s="3" t="n">
-        <v>460</v>
+        <v>430</v>
       </c>
       <c r="M108" s="3" t="n">
-        <v>5100</v>
+        <v>5170</v>
       </c>
       <c r="N108" s="3" t="n">
-        <v>6045</v>
+        <v>5965</v>
       </c>
       <c r="O108" s="3" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="P108" s="3" t="n">
-        <v>6990</v>
+        <v>6760</v>
       </c>
       <c r="Q108" s="3" t="n">
-        <v>13540</v>
+        <v>13175</v>
       </c>
       <c r="R108" s="3" t="n">
         <v>28</v>
@@ -20490,16 +20490,16 @@
         <v>60</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>580</v>
+        <v>565</v>
       </c>
       <c r="O270" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="P270" s="3" t="n">
-        <v>6790</v>
+        <v>6760</v>
       </c>
       <c r="Q270" s="3" t="n">
-        <v>7840</v>
+        <v>7795</v>
       </c>
       <c r="R270" s="3" t="n">
         <v>28</v>
@@ -20513,12 +20513,12 @@
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Algebra I H</t>
+          <t>Composition &amp; Literature</t>
         </is>
       </c>
       <c r="D271" s="2" t="n">
@@ -20526,27 +20526,27 @@
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>English</t>
         </is>
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>O'Connor, Paul</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>105617</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-101</t>
         </is>
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20555,25 +20555,25 @@
         </is>
       </c>
       <c r="K271" s="3" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="L271" s="3" t="n">
         <v>430</v>
       </c>
       <c r="M271" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="N271" s="3" t="n">
-        <v>590</v>
+        <v>1040</v>
       </c>
       <c r="O271" s="3" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="P271" s="3" t="n">
-        <v>6790</v>
+        <v>1980</v>
       </c>
       <c r="Q271" s="3" t="n">
-        <v>7855</v>
+        <v>3470</v>
       </c>
       <c r="R271" s="3" t="n">
         <v>28</v>
@@ -20587,16 +20587,16 @@
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>120</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Composition &amp; Literature</t>
+          <t>American Literature</t>
         </is>
       </c>
       <c r="D272" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E272" s="2" t="inlineStr">
         <is>
@@ -20605,22 +20605,22 @@
       </c>
       <c r="F272" s="2" t="inlineStr">
         <is>
-          <t>O'Connor, Paul</t>
+          <t>Nobilione, Lauren</t>
         </is>
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>105617</t>
+          <t>108420</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
-          <t>D-101</t>
+          <t>D-104</t>
         </is>
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20638,16 +20638,16 @@
         <v>100</v>
       </c>
       <c r="N272" s="3" t="n">
-        <v>1040</v>
+        <v>825</v>
       </c>
       <c r="O272" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P272" s="3" t="n">
-        <v>1980</v>
+        <v>1550</v>
       </c>
       <c r="Q272" s="3" t="n">
-        <v>3470</v>
+        <v>2825</v>
       </c>
       <c r="R272" s="3" t="n">
         <v>28</v>
@@ -20661,40 +20661,40 @@
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>520</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>American Literature</t>
+          <t>Chemistry</t>
         </is>
       </c>
       <c r="D273" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>Nobilione, Lauren</t>
+          <t>Doughty, Chelsea</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>108420</t>
+          <t>106757</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
-          <t>D-104</t>
+          <t>D-203</t>
         </is>
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20706,22 +20706,22 @@
         <v>20</v>
       </c>
       <c r="L273" s="3" t="n">
-        <v>430</v>
+        <v>450</v>
       </c>
       <c r="M273" s="3" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="N273" s="3" t="n">
-        <v>825</v>
+        <v>535</v>
       </c>
       <c r="O273" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P273" s="3" t="n">
-        <v>1550</v>
+        <v>1010</v>
       </c>
       <c r="Q273" s="3" t="n">
-        <v>2825</v>
+        <v>2015</v>
       </c>
       <c r="R273" s="3" t="n">
         <v>28</v>
@@ -20744,7 +20744,7 @@
         </is>
       </c>
       <c r="D274" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
@@ -20768,7 +20768,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20783,19 +20783,19 @@
         <v>450</v>
       </c>
       <c r="M274" s="3" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="N274" s="3" t="n">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="O274" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P274" s="3" t="n">
-        <v>1010</v>
+        <v>1020</v>
       </c>
       <c r="Q274" s="3" t="n">
-        <v>2015</v>
+        <v>2035</v>
       </c>
       <c r="R274" s="3" t="n">
         <v>28</v>
@@ -20818,7 +20818,7 @@
         </is>
       </c>
       <c r="D275" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20857,19 +20857,19 @@
         <v>450</v>
       </c>
       <c r="M275" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N275" s="3" t="n">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="O275" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P275" s="3" t="n">
-        <v>1020</v>
+        <v>1030</v>
       </c>
       <c r="Q275" s="3" t="n">
-        <v>2035</v>
+        <v>2055</v>
       </c>
       <c r="R275" s="3" t="n">
         <v>28</v>
@@ -20892,7 +20892,7 @@
         </is>
       </c>
       <c r="D276" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
@@ -20916,7 +20916,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20931,19 +20931,19 @@
         <v>450</v>
       </c>
       <c r="M276" s="3" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="N276" s="3" t="n">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="O276" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P276" s="3" t="n">
-        <v>1030</v>
+        <v>1040</v>
       </c>
       <c r="Q276" s="3" t="n">
-        <v>2055</v>
+        <v>2075</v>
       </c>
       <c r="R276" s="3" t="n">
         <v>28</v>
@@ -20966,7 +20966,7 @@
         </is>
       </c>
       <c r="D277" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E277" s="2" t="inlineStr">
         <is>
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21005,19 +21005,19 @@
         <v>450</v>
       </c>
       <c r="M277" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N277" s="3" t="n">
-        <v>565</v>
+        <v>575</v>
       </c>
       <c r="O277" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P277" s="3" t="n">
-        <v>1040</v>
+        <v>1050</v>
       </c>
       <c r="Q277" s="3" t="n">
-        <v>2075</v>
+        <v>2095</v>
       </c>
       <c r="R277" s="3" t="n">
         <v>28</v>
@@ -21031,40 +21031,40 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>411</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Algebra I H</t>
         </is>
       </c>
       <c r="D278" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>Doughty, Chelsea</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>106757</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>D-203</t>
+          <t>D-110</t>
         </is>
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21073,25 +21073,25 @@
         </is>
       </c>
       <c r="K278" s="3" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="L278" s="3" t="n">
-        <v>450</v>
+        <v>430</v>
       </c>
       <c r="M278" s="3" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="N278" s="3" t="n">
         <v>575</v>
       </c>
       <c r="O278" s="3" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="P278" s="3" t="n">
-        <v>1050</v>
+        <v>6760</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>2095</v>
+        <v>7810</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>28</v>
@@ -22511,40 +22511,40 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Algebra I</t>
+          <t>Composition &amp; Literature</t>
         </is>
       </c>
       <c r="D298" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>English</t>
         </is>
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Serra, Carmine</t>
         </is>
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>105803</t>
         </is>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22556,22 +22556,22 @@
         <v>20</v>
       </c>
       <c r="L298" s="3" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="M298" s="3" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="N298" s="3" t="n">
-        <v>590</v>
+        <v>515</v>
       </c>
       <c r="O298" s="3" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="P298" s="3" t="n">
-        <v>6790</v>
+        <v>970</v>
       </c>
       <c r="Q298" s="3" t="n">
-        <v>7810</v>
+        <v>1935</v>
       </c>
       <c r="R298" s="3" t="n">
         <v>28</v>
@@ -22585,40 +22585,40 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Algebra I</t>
+          <t>Composition &amp; Literature</t>
         </is>
       </c>
       <c r="D299" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>English</t>
         </is>
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Serra, Carmine</t>
         </is>
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>105803</t>
         </is>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22630,22 +22630,22 @@
         <v>20</v>
       </c>
       <c r="L299" s="3" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="M299" s="3" t="n">
         <v>70</v>
       </c>
       <c r="N299" s="3" t="n">
-        <v>590</v>
+        <v>525</v>
       </c>
       <c r="O299" s="3" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="P299" s="3" t="n">
-        <v>6790</v>
+        <v>980</v>
       </c>
       <c r="Q299" s="3" t="n">
-        <v>7810</v>
+        <v>1955</v>
       </c>
       <c r="R299" s="3" t="n">
         <v>28</v>
@@ -22659,40 +22659,40 @@
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Algebra I</t>
+          <t>Composition &amp; Literature</t>
         </is>
       </c>
       <c r="D300" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>English</t>
         </is>
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Serra, Carmine</t>
         </is>
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>105803</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-102</t>
         </is>
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22704,22 +22704,22 @@
         <v>20</v>
       </c>
       <c r="L300" s="3" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="M300" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="N300" s="3" t="n">
-        <v>590</v>
+        <v>535</v>
       </c>
       <c r="O300" s="3" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="P300" s="3" t="n">
-        <v>6790</v>
+        <v>990</v>
       </c>
       <c r="Q300" s="3" t="n">
-        <v>7810</v>
+        <v>1975</v>
       </c>
       <c r="R300" s="3" t="n">
         <v>28</v>
@@ -22742,7 +22742,7 @@
         </is>
       </c>
       <c r="D301" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
@@ -22766,7 +22766,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22781,19 +22781,19 @@
         <v>430</v>
       </c>
       <c r="M301" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="N301" s="3" t="n">
-        <v>515</v>
+        <v>545</v>
       </c>
       <c r="O301" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P301" s="3" t="n">
-        <v>970</v>
+        <v>1000</v>
       </c>
       <c r="Q301" s="3" t="n">
-        <v>1935</v>
+        <v>1995</v>
       </c>
       <c r="R301" s="3" t="n">
         <v>28</v>
@@ -22816,7 +22816,7 @@
         </is>
       </c>
       <c r="D302" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22855,19 +22855,19 @@
         <v>430</v>
       </c>
       <c r="M302" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="N302" s="3" t="n">
-        <v>525</v>
+        <v>555</v>
       </c>
       <c r="O302" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P302" s="3" t="n">
-        <v>980</v>
+        <v>1010</v>
       </c>
       <c r="Q302" s="3" t="n">
-        <v>1955</v>
+        <v>2015</v>
       </c>
       <c r="R302" s="3" t="n">
         <v>28</v>
@@ -22881,35 +22881,35 @@
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>720</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>Composition &amp; Literature</t>
+          <t>U.S. History I</t>
         </is>
       </c>
       <c r="D303" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
-          <t>Serra, Carmine</t>
+          <t>Montegari, James</t>
         </is>
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>105803</t>
+          <t>105671</t>
         </is>
       </c>
       <c r="H303" s="2" t="inlineStr">
         <is>
-          <t>D-102</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="I303" s="2" t="inlineStr">
@@ -22926,22 +22926,22 @@
         <v>20</v>
       </c>
       <c r="L303" s="3" t="n">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="M303" s="3" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="N303" s="3" t="n">
-        <v>535</v>
+        <v>510</v>
       </c>
       <c r="O303" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P303" s="3" t="n">
-        <v>990</v>
+        <v>960</v>
       </c>
       <c r="Q303" s="3" t="n">
-        <v>1975</v>
+        <v>1915</v>
       </c>
       <c r="R303" s="3" t="n">
         <v>28</v>
@@ -22955,40 +22955,40 @@
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>720</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Composition &amp; Literature</t>
+          <t>U.S. History I</t>
         </is>
       </c>
       <c r="D304" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>Serra, Carmine</t>
+          <t>Montegari, James</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t>105803</t>
+          <t>105671</t>
         </is>
       </c>
       <c r="H304" s="2" t="inlineStr">
         <is>
-          <t>D-102</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23000,22 +23000,22 @@
         <v>20</v>
       </c>
       <c r="L304" s="3" t="n">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="M304" s="3" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="N304" s="3" t="n">
-        <v>545</v>
+        <v>520</v>
       </c>
       <c r="O304" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P304" s="3" t="n">
-        <v>1000</v>
+        <v>970</v>
       </c>
       <c r="Q304" s="3" t="n">
-        <v>1995</v>
+        <v>1935</v>
       </c>
       <c r="R304" s="3" t="n">
         <v>28</v>
@@ -23029,40 +23029,40 @@
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>720</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Composition &amp; Literature</t>
+          <t>U.S. History I</t>
         </is>
       </c>
       <c r="D305" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>Serra, Carmine</t>
+          <t>Montegari, James</t>
         </is>
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t>105803</t>
+          <t>105671</t>
         </is>
       </c>
       <c r="H305" s="2" t="inlineStr">
         <is>
-          <t>D-102</t>
+          <t>I-114</t>
         </is>
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23074,22 +23074,22 @@
         <v>20</v>
       </c>
       <c r="L305" s="3" t="n">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="M305" s="3" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="N305" s="3" t="n">
-        <v>555</v>
+        <v>530</v>
       </c>
       <c r="O305" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P305" s="3" t="n">
-        <v>1010</v>
+        <v>980</v>
       </c>
       <c r="Q305" s="3" t="n">
-        <v>2015</v>
+        <v>1955</v>
       </c>
       <c r="R305" s="3" t="n">
         <v>28</v>
@@ -23112,7 +23112,7 @@
         </is>
       </c>
       <c r="D306" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
@@ -23136,7 +23136,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23151,19 +23151,19 @@
         <v>425</v>
       </c>
       <c r="M306" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="N306" s="3" t="n">
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="O306" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P306" s="3" t="n">
-        <v>960</v>
+        <v>990</v>
       </c>
       <c r="Q306" s="3" t="n">
-        <v>1915</v>
+        <v>1975</v>
       </c>
       <c r="R306" s="3" t="n">
         <v>28</v>
@@ -23186,7 +23186,7 @@
         </is>
       </c>
       <c r="D307" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
@@ -23210,7 +23210,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23225,19 +23225,19 @@
         <v>425</v>
       </c>
       <c r="M307" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="N307" s="3" t="n">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="O307" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P307" s="3" t="n">
-        <v>970</v>
+        <v>1000</v>
       </c>
       <c r="Q307" s="3" t="n">
-        <v>1935</v>
+        <v>1995</v>
       </c>
       <c r="R307" s="3" t="n">
         <v>28</v>
@@ -23251,40 +23251,40 @@
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>112</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>U.S. History I</t>
+          <t>Composition &amp; Literature</t>
         </is>
       </c>
       <c r="D308" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>English</t>
         </is>
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>Montegari, James</t>
+          <t>Judge, Michelle</t>
         </is>
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t>105671</t>
+          <t>105767</t>
         </is>
       </c>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23293,25 +23293,25 @@
         </is>
       </c>
       <c r="K308" s="3" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="L308" s="3" t="n">
-        <v>425</v>
+        <v>405</v>
       </c>
       <c r="M308" s="3" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="N308" s="3" t="n">
-        <v>530</v>
+        <v>695</v>
       </c>
       <c r="O308" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P308" s="3" t="n">
-        <v>980</v>
+        <v>0</v>
       </c>
       <c r="Q308" s="3" t="n">
-        <v>1955</v>
+        <v>1145</v>
       </c>
       <c r="R308" s="3" t="n">
         <v>28</v>
@@ -23325,40 +23325,40 @@
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>U.S. History I</t>
+          <t>American Literature</t>
         </is>
       </c>
       <c r="D309" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>English</t>
         </is>
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
-          <t>Montegari, James</t>
+          <t>Mazella, Julie</t>
         </is>
       </c>
       <c r="G309" s="2" t="inlineStr">
         <is>
-          <t>105671</t>
+          <t>105642</t>
         </is>
       </c>
       <c r="H309" s="2" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23367,25 +23367,25 @@
         </is>
       </c>
       <c r="K309" s="3" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="L309" s="3" t="n">
         <v>425</v>
       </c>
       <c r="M309" s="3" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="N309" s="3" t="n">
-        <v>540</v>
+        <v>655</v>
       </c>
       <c r="O309" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P309" s="3" t="n">
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="Q309" s="3" t="n">
-        <v>1975</v>
+        <v>1125</v>
       </c>
       <c r="R309" s="3" t="n">
         <v>28</v>
@@ -23399,40 +23399,40 @@
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>420</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>U.S. History I</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="D310" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
-          <t>Montegari, James</t>
+          <t>Hartmann, Katy</t>
         </is>
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>105671</t>
+          <t>115019</t>
         </is>
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>I-114</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23444,22 +23444,22 @@
         <v>20</v>
       </c>
       <c r="L310" s="3" t="n">
-        <v>425</v>
+        <v>450</v>
       </c>
       <c r="M310" s="3" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="N310" s="3" t="n">
-        <v>550</v>
+        <v>460</v>
       </c>
       <c r="O310" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P310" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>1995</v>
+        <v>930</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>28</v>
@@ -23473,30 +23473,30 @@
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>420</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>Composition &amp; Literature</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="D311" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
-          <t>Judge, Michelle</t>
+          <t>Hartmann, Katy</t>
         </is>
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>105767</t>
+          <t>115019</t>
         </is>
       </c>
       <c r="H311" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23515,16 +23515,16 @@
         </is>
       </c>
       <c r="K311" s="3" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="L311" s="3" t="n">
-        <v>405</v>
+        <v>450</v>
       </c>
       <c r="M311" s="3" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="N311" s="3" t="n">
-        <v>695</v>
+        <v>470</v>
       </c>
       <c r="O311" s="3" t="n">
         <v>0</v>
@@ -23533,7 +23533,7 @@
         <v>0</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>1145</v>
+        <v>940</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>28</v>
@@ -23547,30 +23547,30 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>420</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>American Literature</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="D312" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>Mazella, Julie</t>
+          <t>Oh, Burton</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>105642</t>
+          <t>122121</t>
         </is>
       </c>
       <c r="H312" s="2" t="inlineStr">
@@ -23589,16 +23589,16 @@
         </is>
       </c>
       <c r="K312" s="3" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="L312" s="3" t="n">
-        <v>425</v>
+        <v>450</v>
       </c>
       <c r="M312" s="3" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="N312" s="3" t="n">
-        <v>655</v>
+        <v>460</v>
       </c>
       <c r="O312" s="3" t="n">
         <v>0</v>
@@ -23607,7 +23607,7 @@
         <v>0</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>1125</v>
+        <v>930</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>28</v>
@@ -23630,7 +23630,7 @@
         </is>
       </c>
       <c r="D313" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
@@ -23639,12 +23639,12 @@
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>Hartmann, Katy</t>
+          <t>Oh, Burton</t>
         </is>
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>115019</t>
+          <t>122121</t>
         </is>
       </c>
       <c r="H313" s="2" t="inlineStr">
@@ -23669,10 +23669,10 @@
         <v>450</v>
       </c>
       <c r="M313" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="N313" s="3" t="n">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="O313" s="3" t="n">
         <v>0</v>
@@ -23681,7 +23681,7 @@
         <v>0</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>930</v>
+        <v>940</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>28</v>
@@ -23695,16 +23695,16 @@
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>Algebra I</t>
         </is>
       </c>
       <c r="D314" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
@@ -23713,22 +23713,22 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>Hartmann, Katy</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>115019</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H314" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23740,22 +23740,22 @@
         <v>20</v>
       </c>
       <c r="L314" s="3" t="n">
-        <v>450</v>
+        <v>410</v>
       </c>
       <c r="M314" s="3" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="N314" s="3" t="n">
-        <v>470</v>
+        <v>585</v>
       </c>
       <c r="O314" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P314" s="3" t="n">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>940</v>
+        <v>2025</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>28</v>
@@ -23769,16 +23769,16 @@
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>Algebra I</t>
         </is>
       </c>
       <c r="D315" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
@@ -23787,22 +23787,22 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>Oh, Burton</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>122121</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H315" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23814,22 +23814,22 @@
         <v>20</v>
       </c>
       <c r="L315" s="3" t="n">
-        <v>450</v>
+        <v>410</v>
       </c>
       <c r="M315" s="3" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="N315" s="3" t="n">
-        <v>460</v>
+        <v>595</v>
       </c>
       <c r="O315" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P315" s="3" t="n">
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>930</v>
+        <v>2045</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>28</v>
@@ -23843,16 +23843,16 @@
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>Algebra I</t>
         </is>
       </c>
       <c r="D316" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
@@ -23861,22 +23861,22 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>Oh, Burton</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>122121</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H316" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23888,22 +23888,22 @@
         <v>20</v>
       </c>
       <c r="L316" s="3" t="n">
-        <v>450</v>
+        <v>410</v>
       </c>
       <c r="M316" s="3" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="N316" s="3" t="n">
-        <v>470</v>
+        <v>605</v>
       </c>
       <c r="O316" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P316" s="3" t="n">
-        <v>0</v>
+        <v>1030</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>940</v>
+        <v>2065</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>28</v>
@@ -24690,7 +24690,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24764,7 +24764,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -27757,10 +27757,10 @@
         <v>8</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -27833,10 +27833,10 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
@@ -27852,10 +27852,10 @@
         <v>10</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">
@@ -30564,22 +30564,22 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>15/15</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -31649,7 +31649,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3">
@@ -31659,7 +31659,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -31689,7 +31689,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -31710,7 +31710,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>161/345</t>
+          <t>162/345</t>
         </is>
       </c>
     </row>
@@ -31733,7 +31733,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12">
@@ -31773,7 +31773,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
@@ -31783,7 +31783,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Job 1 COMPLETE: 367/367 sections placed — zero unplaced
ALL 367 sections placed. Zero conflicts. Zero violations.

Journey: 360 → 363 → 366 → 367/367
- Willi 410×3: D-110 → J-020 (room oversubscription)
- Willi 411×1: D-110 → J-020 (cascading room conflict)
- Saggio 710: S1 6th period approved
- Daniels 620: S1 6th period approved
- Chiaravalloti 631: S2 6th period approved
- Zawiski 312: consecutive-6 pre-reservation engine fix

Period distribution: A=56, B=56, C=48, D=51, E=53, F=56, G=47
Teacher conflicts: 0 | Room double-bookings: 0
Consecutive-6 violations: 0 | Load violations: 0
10 teachers with 6th-period stipends

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1168,16 +1168,16 @@
         <v>5100</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>5895</v>
+        <v>5890</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>6690</v>
+        <v>6680</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>13255</v>
+        <v>13240</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>28</v>
@@ -1242,16 +1242,16 @@
         <v>5110</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>5905</v>
+        <v>5900</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>6700</v>
+        <v>6690</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>13245</v>
+        <v>13230</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>28</v>
@@ -2952,16 +2952,16 @@
         <v>5120</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>5915</v>
+        <v>5910</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>6710</v>
+        <v>6700</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>13360</v>
+        <v>13345</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>28</v>
@@ -6800,16 +6800,16 @@
         <v>5130</v>
       </c>
       <c r="N85" s="3" t="n">
-        <v>5925</v>
+        <v>5920</v>
       </c>
       <c r="O85" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P85" s="3" t="n">
-        <v>6720</v>
+        <v>6710</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>13400</v>
+        <v>13385</v>
       </c>
       <c r="R85" s="3" t="n">
         <v>28</v>
@@ -6874,16 +6874,16 @@
         <v>5140</v>
       </c>
       <c r="N86" s="3" t="n">
-        <v>5935</v>
+        <v>5930</v>
       </c>
       <c r="O86" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P86" s="3" t="n">
-        <v>6730</v>
+        <v>6720</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>13420</v>
+        <v>13405</v>
       </c>
       <c r="R86" s="3" t="n">
         <v>28</v>
@@ -6948,16 +6948,16 @@
         <v>5150</v>
       </c>
       <c r="N87" s="3" t="n">
-        <v>5945</v>
+        <v>5940</v>
       </c>
       <c r="O87" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P87" s="3" t="n">
-        <v>6740</v>
+        <v>6730</v>
       </c>
       <c r="Q87" s="3" t="n">
-        <v>13440</v>
+        <v>13425</v>
       </c>
       <c r="R87" s="3" t="n">
         <v>28</v>
@@ -9834,16 +9834,16 @@
         <v>5160</v>
       </c>
       <c r="N126" s="3" t="n">
-        <v>5955</v>
+        <v>5950</v>
       </c>
       <c r="O126" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P126" s="3" t="n">
-        <v>6750</v>
+        <v>6740</v>
       </c>
       <c r="Q126" s="3" t="n">
-        <v>13155</v>
+        <v>13140</v>
       </c>
       <c r="R126" s="3" t="n">
         <v>28</v>
@@ -9908,16 +9908,16 @@
         <v>5170</v>
       </c>
       <c r="N127" s="3" t="n">
-        <v>5965</v>
+        <v>5960</v>
       </c>
       <c r="O127" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P127" s="3" t="n">
-        <v>6760</v>
+        <v>6750</v>
       </c>
       <c r="Q127" s="3" t="n">
-        <v>13175</v>
+        <v>13160</v>
       </c>
       <c r="R127" s="3" t="n">
         <v>28</v>
@@ -9982,16 +9982,16 @@
         <v>5180</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>5975</v>
+        <v>5970</v>
       </c>
       <c r="O128" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P128" s="3" t="n">
-        <v>6770</v>
+        <v>6760</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>13195</v>
+        <v>13180</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>28</v>
@@ -20490,16 +20490,16 @@
         <v>60</v>
       </c>
       <c r="N270" s="3" t="n">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="O270" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="P270" s="3" t="n">
-        <v>6770</v>
+        <v>6760</v>
       </c>
       <c r="Q270" s="3" t="n">
-        <v>7805</v>
+        <v>7790</v>
       </c>
       <c r="R270" s="3" t="n">
         <v>28</v>
@@ -21031,12 +21031,12 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>421</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Algebra I H</t>
+          <t>Geometry H</t>
         </is>
       </c>
       <c r="D278" s="2" t="n">
@@ -21049,22 +21049,22 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Ahn, Keun</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>105826</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>D-110</t>
+          <t>D-106</t>
         </is>
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21073,25 +21073,25 @@
         </is>
       </c>
       <c r="K278" s="3" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="L278" s="3" t="n">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="M278" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="N278" s="3" t="n">
-        <v>565</v>
+        <v>695</v>
       </c>
       <c r="O278" s="3" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="P278" s="3" t="n">
-        <v>6770</v>
+        <v>1310</v>
       </c>
       <c r="Q278" s="3" t="n">
-        <v>7810</v>
+        <v>2460</v>
       </c>
       <c r="R278" s="3" t="n">
         <v>28</v>
@@ -21114,7 +21114,7 @@
         </is>
       </c>
       <c r="D279" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
@@ -21138,7 +21138,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21153,19 +21153,19 @@
         <v>435</v>
       </c>
       <c r="M279" s="3" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="N279" s="3" t="n">
-        <v>695</v>
+        <v>705</v>
       </c>
       <c r="O279" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P279" s="3" t="n">
-        <v>1310</v>
+        <v>1320</v>
       </c>
       <c r="Q279" s="3" t="n">
-        <v>2460</v>
+        <v>2480</v>
       </c>
       <c r="R279" s="3" t="n">
         <v>28</v>
@@ -21188,7 +21188,7 @@
         </is>
       </c>
       <c r="D280" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
@@ -21212,7 +21212,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21227,19 +21227,19 @@
         <v>435</v>
       </c>
       <c r="M280" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N280" s="3" t="n">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="O280" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P280" s="3" t="n">
-        <v>1320</v>
+        <v>1330</v>
       </c>
       <c r="Q280" s="3" t="n">
-        <v>2480</v>
+        <v>2500</v>
       </c>
       <c r="R280" s="3" t="n">
         <v>28</v>
@@ -21253,40 +21253,40 @@
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>421</t>
+          <t>810</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>Geometry H</t>
+          <t>Theology 9</t>
         </is>
       </c>
       <c r="D281" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Theology</t>
         </is>
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>Ahn, Keun</t>
+          <t>TBD Theology, New</t>
         </is>
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>105826</t>
+          <t>999999</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
-          <t>D-106</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21298,22 +21298,22 @@
         <v>20</v>
       </c>
       <c r="L281" s="3" t="n">
-        <v>435</v>
+        <v>465</v>
       </c>
       <c r="M281" s="3" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="N281" s="3" t="n">
-        <v>715</v>
+        <v>560</v>
       </c>
       <c r="O281" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P281" s="3" t="n">
-        <v>1330</v>
+        <v>0</v>
       </c>
       <c r="Q281" s="3" t="n">
-        <v>2500</v>
+        <v>1045</v>
       </c>
       <c r="R281" s="3" t="n">
         <v>28</v>
@@ -21336,7 +21336,7 @@
         </is>
       </c>
       <c r="D282" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
@@ -21360,7 +21360,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21375,10 +21375,10 @@
         <v>465</v>
       </c>
       <c r="M282" s="3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="N282" s="3" t="n">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="O282" s="3" t="n">
         <v>0</v>
@@ -21387,7 +21387,7 @@
         <v>0</v>
       </c>
       <c r="Q282" s="3" t="n">
-        <v>1045</v>
+        <v>1055</v>
       </c>
       <c r="R282" s="3" t="n">
         <v>28</v>
@@ -21410,7 +21410,7 @@
         </is>
       </c>
       <c r="D283" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E283" s="2" t="inlineStr">
         <is>
@@ -21434,7 +21434,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21449,10 +21449,10 @@
         <v>465</v>
       </c>
       <c r="M283" s="3" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="N283" s="3" t="n">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="O283" s="3" t="n">
         <v>0</v>
@@ -21461,7 +21461,7 @@
         <v>0</v>
       </c>
       <c r="Q283" s="3" t="n">
-        <v>1055</v>
+        <v>1065</v>
       </c>
       <c r="R283" s="3" t="n">
         <v>28</v>
@@ -21475,40 +21475,40 @@
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>810</t>
+          <t>411</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Theology 9</t>
+          <t>Algebra I H</t>
         </is>
       </c>
       <c r="D284" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
-          <t>Theology</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>TBD Theology, New</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>999999</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21517,25 +21517,25 @@
         </is>
       </c>
       <c r="K284" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="L284" s="3" t="n">
+        <v>430</v>
+      </c>
+      <c r="M284" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="N284" s="3" t="n">
+        <v>570</v>
+      </c>
+      <c r="O284" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="L284" s="3" t="n">
-        <v>465</v>
-      </c>
-      <c r="M284" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="N284" s="3" t="n">
-        <v>580</v>
-      </c>
-      <c r="O284" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="P284" s="3" t="n">
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="Q284" s="3" t="n">
-        <v>1065</v>
+        <v>2065</v>
       </c>
       <c r="R284" s="3" t="n">
         <v>28</v>
@@ -23399,16 +23399,16 @@
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>Algebra I</t>
         </is>
       </c>
       <c r="D310" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
@@ -23417,22 +23417,22 @@
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
-          <t>Hartmann, Katy</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>115019</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23444,22 +23444,22 @@
         <v>20</v>
       </c>
       <c r="L310" s="3" t="n">
-        <v>450</v>
+        <v>410</v>
       </c>
       <c r="M310" s="3" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="N310" s="3" t="n">
-        <v>460</v>
+        <v>580</v>
       </c>
       <c r="O310" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P310" s="3" t="n">
-        <v>0</v>
+        <v>1030</v>
       </c>
       <c r="Q310" s="3" t="n">
-        <v>930</v>
+        <v>2040</v>
       </c>
       <c r="R310" s="3" t="n">
         <v>28</v>
@@ -23473,16 +23473,16 @@
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>Algebra I</t>
         </is>
       </c>
       <c r="D311" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
@@ -23491,22 +23491,22 @@
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
-          <t>Hartmann, Katy</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>115019</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H311" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23518,22 +23518,22 @@
         <v>20</v>
       </c>
       <c r="L311" s="3" t="n">
-        <v>450</v>
+        <v>410</v>
       </c>
       <c r="M311" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="N311" s="3" t="n">
+        <v>590</v>
+      </c>
+      <c r="O311" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="N311" s="3" t="n">
-        <v>470</v>
-      </c>
-      <c r="O311" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="P311" s="3" t="n">
-        <v>0</v>
+        <v>1040</v>
       </c>
       <c r="Q311" s="3" t="n">
-        <v>940</v>
+        <v>2060</v>
       </c>
       <c r="R311" s="3" t="n">
         <v>28</v>
@@ -23547,16 +23547,16 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>410</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>Algebra I</t>
         </is>
       </c>
       <c r="D312" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
@@ -23565,22 +23565,22 @@
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>Oh, Burton</t>
+          <t>Willi, Mary</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>122121</t>
+          <t>106623</t>
         </is>
       </c>
       <c r="H312" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>J-020</t>
         </is>
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23592,22 +23592,22 @@
         <v>20</v>
       </c>
       <c r="L312" s="3" t="n">
-        <v>450</v>
+        <v>410</v>
       </c>
       <c r="M312" s="3" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="N312" s="3" t="n">
-        <v>460</v>
+        <v>600</v>
       </c>
       <c r="O312" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P312" s="3" t="n">
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="Q312" s="3" t="n">
-        <v>930</v>
+        <v>2080</v>
       </c>
       <c r="R312" s="3" t="n">
         <v>28</v>
@@ -23630,7 +23630,7 @@
         </is>
       </c>
       <c r="D313" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
@@ -23639,12 +23639,12 @@
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>Oh, Burton</t>
+          <t>Hartmann, Katy</t>
         </is>
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>122121</t>
+          <t>115019</t>
         </is>
       </c>
       <c r="H313" s="2" t="inlineStr">
@@ -23669,10 +23669,10 @@
         <v>450</v>
       </c>
       <c r="M313" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N313" s="3" t="n">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="O313" s="3" t="n">
         <v>0</v>
@@ -23681,7 +23681,7 @@
         <v>0</v>
       </c>
       <c r="Q313" s="3" t="n">
-        <v>940</v>
+        <v>930</v>
       </c>
       <c r="R313" s="3" t="n">
         <v>28</v>
@@ -23695,16 +23695,16 @@
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>420</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>Algebra I</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="D314" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
@@ -23713,22 +23713,22 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Hartmann, Katy</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>115019</t>
         </is>
       </c>
       <c r="H314" s="2" t="inlineStr">
         <is>
-          <t>J-020</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23740,22 +23740,22 @@
         <v>20</v>
       </c>
       <c r="L314" s="3" t="n">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="M314" s="3" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="N314" s="3" t="n">
-        <v>575</v>
+        <v>470</v>
       </c>
       <c r="O314" s="3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P314" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="Q314" s="3" t="n">
-        <v>2005</v>
+        <v>940</v>
       </c>
       <c r="R314" s="3" t="n">
         <v>28</v>
@@ -23769,16 +23769,16 @@
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>420</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>Algebra I</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="D315" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
@@ -23787,22 +23787,22 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Oh, Burton</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>122121</t>
         </is>
       </c>
       <c r="H315" s="2" t="inlineStr">
         <is>
-          <t>J-020</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23814,22 +23814,22 @@
         <v>20</v>
       </c>
       <c r="L315" s="3" t="n">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="M315" s="3" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="N315" s="3" t="n">
-        <v>585</v>
+        <v>460</v>
       </c>
       <c r="O315" s="3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P315" s="3" t="n">
-        <v>1010</v>
+        <v>0</v>
       </c>
       <c r="Q315" s="3" t="n">
-        <v>2025</v>
+        <v>930</v>
       </c>
       <c r="R315" s="3" t="n">
         <v>28</v>
@@ -23843,16 +23843,16 @@
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>420</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>Algebra I</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="D316" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
@@ -23861,22 +23861,22 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>Willi, Mary</t>
+          <t>Oh, Burton</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>106623</t>
+          <t>122121</t>
         </is>
       </c>
       <c r="H316" s="2" t="inlineStr">
         <is>
-          <t>J-020</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23888,22 +23888,22 @@
         <v>20</v>
       </c>
       <c r="L316" s="3" t="n">
-        <v>410</v>
+        <v>450</v>
       </c>
       <c r="M316" s="3" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="N316" s="3" t="n">
-        <v>595</v>
+        <v>470</v>
       </c>
       <c r="O316" s="3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P316" s="3" t="n">
-        <v>1020</v>
+        <v>0</v>
       </c>
       <c r="Q316" s="3" t="n">
-        <v>2045</v>
+        <v>940</v>
       </c>
       <c r="R316" s="3" t="n">
         <v>28</v>
@@ -27776,10 +27776,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -30564,22 +30564,22 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>15/15</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -31649,7 +31649,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3">
@@ -31659,7 +31659,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -31743,7 +31743,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Engine run output: Job1 placements, preflight report, priority audit log (run with B1+B2+B3 fixes)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8706,7 +8706,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -9002,7 +9002,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -9979,19 +9979,19 @@
         <v>430</v>
       </c>
       <c r="M128" s="3" t="n">
-        <v>5180</v>
+        <v>5170</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>5970</v>
+        <v>5960</v>
       </c>
       <c r="O128" s="3" t="n">
         <v>50</v>
       </c>
       <c r="P128" s="3" t="n">
-        <v>6760</v>
+        <v>6750</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>13180</v>
+        <v>13160</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>28</v>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10926,7 +10926,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11148,7 +11148,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11370,7 +11370,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11666,7 +11666,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12258,7 +12258,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12776,7 +12776,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13220,7 +13220,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13442,7 +13442,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13590,7 +13590,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13738,7 +13738,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14034,7 +14034,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14404,7 +14404,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14478,7 +14478,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14552,7 +14552,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14848,7 +14848,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14922,7 +14922,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14996,7 +14996,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15514,7 +15514,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15588,7 +15588,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15810,7 +15810,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15884,7 +15884,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16106,7 +16106,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16328,7 +16328,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16550,7 +16550,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16846,7 +16846,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17068,7 +17068,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17142,7 +17142,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17216,7 +17216,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17290,7 +17290,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17660,7 +17660,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18104,7 +18104,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18400,7 +18400,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18548,7 +18548,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18696,7 +18696,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18770,7 +18770,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18844,7 +18844,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18992,7 +18992,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19214,7 +19214,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19510,7 +19510,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19658,7 +19658,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19880,7 +19880,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20324,7 +20324,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20496,10 +20496,10 @@
         <v>50</v>
       </c>
       <c r="P270" s="3" t="n">
-        <v>6760</v>
+        <v>6750</v>
       </c>
       <c r="Q270" s="3" t="n">
-        <v>7790</v>
+        <v>7780</v>
       </c>
       <c r="R270" s="3" t="n">
         <v>28</v>
@@ -20546,7 +20546,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20620,7 +20620,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20768,7 +20768,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20916,7 +20916,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21212,7 +21212,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21434,7 +21434,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21878,7 +21878,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21952,7 +21952,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22174,7 +22174,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22470,7 +22470,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22914,7 +22914,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23210,7 +23210,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23284,7 +23284,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23432,7 +23432,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23876,7 +23876,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23950,7 +23950,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24098,7 +24098,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24320,7 +24320,7 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
@@ -24394,7 +24394,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24468,7 +24468,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24542,7 +24542,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24690,7 +24690,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24838,7 +24838,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24912,7 +24912,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -24986,7 +24986,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -27751,13 +27751,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>56</v>
@@ -27770,16 +27770,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -27789,16 +27789,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
@@ -27808,16 +27808,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
@@ -27827,16 +27827,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7">
@@ -27849,13 +27849,13 @@
         <v>8</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -27865,16 +27865,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -30254,29 +30254,29 @@
           <t>117711</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>6/5</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>6/5</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>6/5</t>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>18/15</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>100% FY Stipend</t>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H54" s="3" t="n">
@@ -31649,7 +31649,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3">
@@ -31659,7 +31659,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -31710,7 +31710,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>156/345</t>
+          <t>160/345</t>
         </is>
       </c>
     </row>
@@ -31743,7 +31743,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13">
@@ -31753,7 +31753,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
@@ -31763,7 +31763,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15">
@@ -31773,7 +31773,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16">
@@ -31783,7 +31783,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">
@@ -31793,7 +31793,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Job 1 output with B9 fix — 367/367 sections placed
Saggio 710 World History #3 now placed at Period A (was UNPLACED).
Cross-course teacher consolidation pairs S1/S2 sections from different
courses into shared periods, freeing Period A for 710 #3.

Saggio schedule: A(710#3 FY), B(741#2 S1+741#3 S2), C(751#1 S1+723#1 S2),
D(710#2 FY), E(710#1 FY), F(free/C6), G(741#1 S1+744#2 S2) = 6/6 both sems.

Engine still running Phase D — Job 2 output will follow.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4340,7 +4340,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -6338,7 +6338,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -9372,7 +9372,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9446,7 +9446,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -9979,19 +9979,19 @@
         <v>430</v>
       </c>
       <c r="M128" s="3" t="n">
-        <v>5170</v>
+        <v>5180</v>
       </c>
       <c r="N128" s="3" t="n">
-        <v>5960</v>
+        <v>5970</v>
       </c>
       <c r="O128" s="3" t="n">
         <v>50</v>
       </c>
       <c r="P128" s="3" t="n">
-        <v>6750</v>
+        <v>6760</v>
       </c>
       <c r="Q128" s="3" t="n">
-        <v>13160</v>
+        <v>13180</v>
       </c>
       <c r="R128" s="3" t="n">
         <v>28</v>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11370,7 +11370,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11962,7 +11962,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12554,7 +12554,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12628,7 +12628,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12776,7 +12776,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -13220,7 +13220,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13294,7 +13294,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13442,7 +13442,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13590,7 +13590,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13738,7 +13738,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14330,7 +14330,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14404,7 +14404,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14552,7 +14552,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14848,7 +14848,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15514,7 +15514,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15588,7 +15588,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15884,7 +15884,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16106,7 +16106,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16328,7 +16328,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16550,7 +16550,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16772,7 +16772,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16846,7 +16846,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -17068,7 +17068,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17142,7 +17142,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17216,7 +17216,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17512,7 +17512,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18030,7 +18030,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18104,7 +18104,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18400,7 +18400,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18548,7 +18548,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18696,7 +18696,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19288,7 +19288,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19436,7 +19436,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19510,7 +19510,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19658,7 +19658,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19880,7 +19880,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20496,10 +20496,10 @@
         <v>50</v>
       </c>
       <c r="P270" s="3" t="n">
-        <v>6750</v>
+        <v>6760</v>
       </c>
       <c r="Q270" s="3" t="n">
-        <v>7780</v>
+        <v>7790</v>
       </c>
       <c r="R270" s="3" t="n">
         <v>28</v>
@@ -20546,7 +20546,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20768,7 +20768,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20916,7 +20916,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21212,7 +21212,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21434,7 +21434,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21656,7 +21656,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21952,7 +21952,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22026,7 +22026,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22100,7 +22100,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22248,7 +22248,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22396,7 +22396,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22766,7 +22766,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22914,7 +22914,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22988,7 +22988,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23210,7 +23210,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23432,7 +23432,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23728,7 +23728,7 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23950,7 +23950,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24098,7 +24098,7 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
@@ -24394,7 +24394,7 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
@@ -24468,7 +24468,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24690,7 +24690,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24764,7 +24764,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24838,7 +24838,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24912,7 +24912,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -24986,7 +24986,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -27751,16 +27751,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -27770,16 +27770,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -27789,16 +27789,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -27808,7 +27808,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>7</v>
@@ -27817,7 +27817,7 @@
         <v>37</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -27827,16 +27827,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -27846,16 +27846,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
@@ -27865,16 +27865,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -30254,29 +30254,29 @@
           <t>117711</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>5/5</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>5/5</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>5/5</t>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>6/5</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>6/5</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>6/5</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>15/15</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Standard</t>
+          <t>18/15</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>100% FY Stipend</t>
         </is>
       </c>
       <c r="H54" s="3" t="n">
@@ -31649,7 +31649,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3">
@@ -31659,7 +31659,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -31710,7 +31710,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>160/345</t>
+          <t>170/345</t>
         </is>
       </c>
     </row>
@@ -31733,7 +31733,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -31743,7 +31743,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13">
@@ -31753,7 +31753,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14">
@@ -31763,7 +31763,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
@@ -31773,7 +31773,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -31783,7 +31783,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
@@ -31793,7 +31793,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Engine intermediate output: Job1 placements, preflight report, priority audit (B10 run in progress)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7300,7 +7300,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -8706,7 +8706,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9446,7 +9446,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10112,7 +10112,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10408,7 +10408,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10926,7 +10926,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11370,7 +11370,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -11962,7 +11962,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12554,7 +12554,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12776,7 +12776,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13294,7 +13294,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13442,7 +13442,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13590,7 +13590,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13738,7 +13738,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14330,7 +14330,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14404,7 +14404,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14922,7 +14922,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15810,7 +15810,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15884,7 +15884,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16106,7 +16106,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16550,7 +16550,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16772,7 +16772,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -17142,7 +17142,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17290,7 +17290,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17512,7 +17512,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17660,7 +17660,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18548,7 +18548,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -19214,7 +19214,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19288,7 +19288,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19806,7 +19806,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19880,7 +19880,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20324,7 +20324,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20916,7 +20916,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21212,7 +21212,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21360,7 +21360,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21434,7 +21434,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21656,7 +21656,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21878,7 +21878,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21952,7 +21952,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22174,7 +22174,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22248,7 +22248,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22470,7 +22470,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22766,7 +22766,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22988,7 +22988,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23210,7 +23210,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23432,7 +23432,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
@@ -23876,7 +23876,7 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
@@ -23950,7 +23950,7 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
@@ -24172,7 +24172,7 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24764,7 +24764,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24986,7 +24986,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -27757,10 +27757,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -27770,16 +27770,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>9</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>10</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -27789,10 +27789,10 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>31</v>
@@ -27808,16 +27808,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -27827,16 +27827,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -27846,16 +27846,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -27865,16 +27865,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -31710,7 +31710,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>170/345</t>
+          <t>163/345</t>
         </is>
       </c>
     </row>
@@ -31733,7 +31733,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
@@ -31743,7 +31743,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -31763,7 +31763,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
@@ -31773,7 +31773,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
@@ -31783,7 +31783,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
@@ -31793,7 +31793,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Engine run in progress: Job 1 output + preflight + audit log
Engine running full mode with Phase D-2 and B17 fix.
Mid-run output — Job 2 and Phase D-2 results pending.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3245,19 +3245,19 @@
         <v>645</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>5130</v>
+        <v>5120</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>6025</v>
+        <v>6015</v>
       </c>
       <c r="O37" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>6920</v>
+        <v>6910</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>5825</v>
+        <v>5815</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>28</v>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3319,19 +3319,19 @@
         <v>645</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O38" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>5835</v>
+        <v>5815</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>28</v>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8129,19 +8129,19 @@
         <v>525</v>
       </c>
       <c r="M103" s="3" t="n">
-        <v>5220</v>
+        <v>5210</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>6230</v>
+        <v>6220</v>
       </c>
       <c r="O103" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P103" s="3" t="n">
-        <v>7240</v>
+        <v>7230</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>5830</v>
+        <v>5820</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>28</v>
@@ -8188,7 +8188,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -9372,7 +9372,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10408,7 +10408,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12554,7 +12554,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12776,7 +12776,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13294,7 +13294,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14034,7 +14034,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14478,7 +14478,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14922,7 +14922,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14996,7 +14996,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15588,7 +15588,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15810,7 +15810,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16550,7 +16550,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16846,7 +16846,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -17216,7 +17216,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17290,7 +17290,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17438,7 +17438,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -17512,7 +17512,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17660,7 +17660,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -18104,7 +18104,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18178,7 +18178,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18400,7 +18400,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18548,7 +18548,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18622,7 +18622,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18696,7 +18696,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18770,7 +18770,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18844,7 +18844,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19288,7 +19288,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19362,7 +19362,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19510,7 +19510,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19658,7 +19658,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20472,7 +20472,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20546,7 +20546,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20620,7 +20620,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20768,7 +20768,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20916,7 +20916,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21064,7 +21064,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21212,7 +21212,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21434,7 +21434,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21952,7 +21952,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22026,7 +22026,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22100,7 +22100,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22174,7 +22174,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22248,7 +22248,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22396,7 +22396,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22470,7 +22470,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22766,7 +22766,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22914,7 +22914,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -22988,7 +22988,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23210,7 +23210,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23284,7 +23284,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23358,7 +23358,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23654,7 +23654,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -24703,16 +24703,16 @@
         <v>855</v>
       </c>
       <c r="M327" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N327" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O327" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P327" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q327" s="3" t="inlineStr"/>
       <c r="R327" s="3" t="n">
@@ -24777,16 +24777,16 @@
         <v>855</v>
       </c>
       <c r="M328" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N328" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O328" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P328" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q328" s="3" t="inlineStr"/>
       <c r="R328" s="3" t="n">
@@ -24851,16 +24851,16 @@
         <v>570</v>
       </c>
       <c r="M329" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O329" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P329" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q329" s="3" t="inlineStr"/>
       <c r="R329" s="3" t="n">
@@ -27679,16 +27679,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -27698,16 +27698,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -27720,13 +27720,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -27736,16 +27736,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -27755,16 +27755,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -27774,16 +27774,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>9</v>
-      </c>
       <c r="D7" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -27793,16 +27793,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -28072,22 +28072,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>15/15</t>
+          <t>12/15</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -28610,12 +28610,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>12/15</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -31577,7 +31577,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3">
@@ -31587,7 +31587,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>159/345</t>
+          <t>156/345</t>
         </is>
       </c>
     </row>
@@ -31661,7 +31661,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12">
@@ -31671,7 +31671,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13">
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -31691,7 +31691,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15">
@@ -31701,7 +31701,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
@@ -31711,7 +31711,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
@@ -31721,7 +31721,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Engine run in progress: Job 1 output (diagnostic run with D-2 logging)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -854,7 +854,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3245,19 +3245,19 @@
         <v>645</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>5120</v>
+        <v>5130</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>6015</v>
+        <v>6025</v>
       </c>
       <c r="O37" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>6910</v>
+        <v>6920</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>5815</v>
+        <v>5825</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>28</v>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3319,19 +3319,19 @@
         <v>645</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>5120</v>
+        <v>5140</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>6015</v>
+        <v>6035</v>
       </c>
       <c r="O38" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>6910</v>
+        <v>6930</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>5815</v>
+        <v>5835</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>28</v>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7300,7 +7300,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7463,19 +7463,19 @@
         <v>670</v>
       </c>
       <c r="M94" s="3" t="n">
-        <v>5180</v>
+        <v>5170</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>6190</v>
+        <v>6180</v>
       </c>
       <c r="O94" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P94" s="3" t="n">
-        <v>7200</v>
+        <v>7190</v>
       </c>
       <c r="Q94" s="3" t="n">
-        <v>5935</v>
+        <v>5925</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>28</v>
@@ -7537,19 +7537,19 @@
         <v>670</v>
       </c>
       <c r="M95" s="3" t="n">
-        <v>5180</v>
+        <v>5170</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>6190</v>
+        <v>6180</v>
       </c>
       <c r="O95" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P95" s="3" t="n">
-        <v>7200</v>
+        <v>7190</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>5935</v>
+        <v>5925</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>28</v>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7611,19 +7611,19 @@
         <v>670</v>
       </c>
       <c r="M96" s="3" t="n">
-        <v>5190</v>
+        <v>5170</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>6200</v>
+        <v>6180</v>
       </c>
       <c r="O96" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P96" s="3" t="n">
-        <v>7210</v>
+        <v>7190</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>5945</v>
+        <v>5925</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>28</v>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8129,19 +8129,19 @@
         <v>525</v>
       </c>
       <c r="M103" s="3" t="n">
-        <v>5210</v>
+        <v>5220</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>6220</v>
+        <v>6230</v>
       </c>
       <c r="O103" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P103" s="3" t="n">
-        <v>7230</v>
+        <v>7240</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>5820</v>
+        <v>5830</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>28</v>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -9446,7 +9446,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11370,7 +11370,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12554,7 +12554,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12776,7 +12776,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14034,7 +14034,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14922,7 +14922,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14996,7 +14996,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15810,7 +15810,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16772,7 +16772,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16846,7 +16846,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17216,7 +17216,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17290,7 +17290,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17512,7 +17512,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18030,7 +18030,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18400,7 +18400,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18622,7 +18622,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -19214,7 +19214,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19362,7 +19362,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19510,7 +19510,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19806,7 +19806,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20472,7 +20472,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20546,7 +20546,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20620,7 +20620,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20768,7 +20768,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21360,7 +21360,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21878,7 +21878,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22100,7 +22100,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22174,7 +22174,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22248,7 +22248,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22470,7 +22470,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22766,7 +22766,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23284,7 +23284,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23358,7 +23358,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23432,7 +23432,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23654,7 +23654,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -24703,16 +24703,16 @@
         <v>855</v>
       </c>
       <c r="M327" s="3" t="n">
-        <v>5120</v>
+        <v>5140</v>
       </c>
       <c r="N327" s="3" t="n">
-        <v>6015</v>
+        <v>6035</v>
       </c>
       <c r="O327" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P327" s="3" t="n">
-        <v>6910</v>
+        <v>6930</v>
       </c>
       <c r="Q327" s="3" t="inlineStr"/>
       <c r="R327" s="3" t="n">
@@ -24777,16 +24777,16 @@
         <v>855</v>
       </c>
       <c r="M328" s="3" t="n">
-        <v>5120</v>
+        <v>5140</v>
       </c>
       <c r="N328" s="3" t="n">
-        <v>6015</v>
+        <v>6035</v>
       </c>
       <c r="O328" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P328" s="3" t="n">
-        <v>6910</v>
+        <v>6930</v>
       </c>
       <c r="Q328" s="3" t="inlineStr"/>
       <c r="R328" s="3" t="n">
@@ -24851,16 +24851,16 @@
         <v>570</v>
       </c>
       <c r="M329" s="3" t="n">
-        <v>5120</v>
+        <v>5140</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>6015</v>
+        <v>6035</v>
       </c>
       <c r="O329" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P329" s="3" t="n">
-        <v>6910</v>
+        <v>6930</v>
       </c>
       <c r="Q329" s="3" t="inlineStr"/>
       <c r="R329" s="3" t="n">
@@ -27679,16 +27679,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -27698,16 +27698,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -27720,13 +27720,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -27736,16 +27736,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -27755,16 +27755,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -27777,13 +27777,13 @@
         <v>9</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -28072,22 +28072,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>15/15</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -28292,27 +28292,27 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
           <t>5/5</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>5/5</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>6/5</t>
-        </is>
-      </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>16/15</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>50% FY Stipend</t>
+          <t>13/15</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H11" s="3" t="n">
@@ -28610,12 +28610,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>13/15</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -31577,7 +31577,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3">
@@ -31587,7 +31587,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -31617,7 +31617,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>156/345</t>
+          <t>157/345</t>
         </is>
       </c>
     </row>
@@ -31661,7 +31661,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -31671,7 +31671,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13">
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
@@ -31691,7 +31691,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
@@ -31701,7 +31701,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -31711,7 +31711,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Engine run in progress — partial Job 1 output (B18 verification run)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -854,7 +854,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3245,19 +3245,19 @@
         <v>645</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>5130</v>
+        <v>5120</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>6025</v>
+        <v>6015</v>
       </c>
       <c r="O37" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>6920</v>
+        <v>6910</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>5825</v>
+        <v>5815</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>28</v>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3319,19 +3319,19 @@
         <v>645</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O38" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>5835</v>
+        <v>5815</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>28</v>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7300,7 +7300,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7463,19 +7463,19 @@
         <v>670</v>
       </c>
       <c r="M94" s="3" t="n">
-        <v>5170</v>
+        <v>5180</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>6180</v>
+        <v>6190</v>
       </c>
       <c r="O94" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P94" s="3" t="n">
-        <v>7190</v>
+        <v>7200</v>
       </c>
       <c r="Q94" s="3" t="n">
-        <v>5925</v>
+        <v>5935</v>
       </c>
       <c r="R94" s="3" t="n">
         <v>28</v>
@@ -7537,19 +7537,19 @@
         <v>670</v>
       </c>
       <c r="M95" s="3" t="n">
-        <v>5170</v>
+        <v>5180</v>
       </c>
       <c r="N95" s="3" t="n">
-        <v>6180</v>
+        <v>6190</v>
       </c>
       <c r="O95" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P95" s="3" t="n">
-        <v>7190</v>
+        <v>7200</v>
       </c>
       <c r="Q95" s="3" t="n">
-        <v>5925</v>
+        <v>5935</v>
       </c>
       <c r="R95" s="3" t="n">
         <v>28</v>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7611,19 +7611,19 @@
         <v>670</v>
       </c>
       <c r="M96" s="3" t="n">
-        <v>5170</v>
+        <v>5190</v>
       </c>
       <c r="N96" s="3" t="n">
-        <v>6180</v>
+        <v>6200</v>
       </c>
       <c r="O96" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P96" s="3" t="n">
-        <v>7190</v>
+        <v>7210</v>
       </c>
       <c r="Q96" s="3" t="n">
-        <v>5925</v>
+        <v>5945</v>
       </c>
       <c r="R96" s="3" t="n">
         <v>28</v>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>UNSCHEDULED</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8129,19 +8129,19 @@
         <v>525</v>
       </c>
       <c r="M103" s="3" t="n">
-        <v>5220</v>
+        <v>5210</v>
       </c>
       <c r="N103" s="3" t="n">
-        <v>6230</v>
+        <v>6220</v>
       </c>
       <c r="O103" s="3" t="n">
         <v>45</v>
       </c>
       <c r="P103" s="3" t="n">
-        <v>7240</v>
+        <v>7230</v>
       </c>
       <c r="Q103" s="3" t="n">
-        <v>5830</v>
+        <v>5820</v>
       </c>
       <c r="R103" s="3" t="n">
         <v>28</v>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -9446,7 +9446,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11370,7 +11370,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -12554,7 +12554,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12776,7 +12776,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13960,7 +13960,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14034,7 +14034,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14922,7 +14922,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14996,7 +14996,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15810,7 +15810,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15958,7 +15958,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16772,7 +16772,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16846,7 +16846,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17216,7 +17216,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17290,7 +17290,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17364,7 +17364,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17512,7 +17512,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18030,7 +18030,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18252,7 +18252,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18400,7 +18400,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18622,7 +18622,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -19214,7 +19214,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19362,7 +19362,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19510,7 +19510,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19806,7 +19806,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20472,7 +20472,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20546,7 +20546,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20620,7 +20620,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20768,7 +20768,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21138,7 +21138,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21360,7 +21360,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21582,7 +21582,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21878,7 +21878,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22100,7 +22100,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22174,7 +22174,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22248,7 +22248,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22470,7 +22470,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22766,7 +22766,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -22840,7 +22840,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23284,7 +23284,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23358,7 +23358,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23432,7 +23432,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
@@ -23580,7 +23580,7 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
@@ -23654,7 +23654,7 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
@@ -24703,16 +24703,16 @@
         <v>855</v>
       </c>
       <c r="M327" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N327" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O327" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P327" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q327" s="3" t="inlineStr"/>
       <c r="R327" s="3" t="n">
@@ -24777,16 +24777,16 @@
         <v>855</v>
       </c>
       <c r="M328" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N328" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O328" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P328" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q328" s="3" t="inlineStr"/>
       <c r="R328" s="3" t="n">
@@ -24851,16 +24851,16 @@
         <v>570</v>
       </c>
       <c r="M329" s="3" t="n">
-        <v>5140</v>
+        <v>5120</v>
       </c>
       <c r="N329" s="3" t="n">
-        <v>6035</v>
+        <v>6015</v>
       </c>
       <c r="O329" s="3" t="n">
         <v>40</v>
       </c>
       <c r="P329" s="3" t="n">
-        <v>6930</v>
+        <v>6910</v>
       </c>
       <c r="Q329" s="3" t="inlineStr"/>
       <c r="R329" s="3" t="n">
@@ -27679,16 +27679,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -27698,16 +27698,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -27720,13 +27720,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -27736,16 +27736,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>8</v>
-      </c>
       <c r="D5" s="3" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -27755,16 +27755,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -27777,13 +27777,13 @@
         <v>9</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -28072,22 +28072,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>15/15</t>
+          <t>12/15</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -28292,27 +28292,27 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
           <t>5/5</t>
         </is>
       </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>6/5</t>
+        </is>
+      </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>13/15</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Standard</t>
+          <t>16/15</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>50% FY Stipend</t>
         </is>
       </c>
       <c r="H11" s="3" t="n">
@@ -28610,12 +28610,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>12/15</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -31577,7 +31577,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3">
@@ -31587,7 +31587,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -31617,7 +31617,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>157/345</t>
+          <t>156/345</t>
         </is>
       </c>
     </row>
@@ -31661,7 +31661,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12">
@@ -31671,7 +31671,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13">
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -31691,7 +31691,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15">
@@ -31701,7 +31701,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
@@ -31711,7 +31711,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Job 1 output: 367/367 sections placed — LEO priority + pool type changes
Results after implementing LEO I/II priority and two pool types:
- LEO I and LEO II processed first in Step 1.6
- LEO pools stored for Job 2 (student-level only), not restricting sections
- All 367 sections placed (up from 364/367)
- 3 previously unplaced 642 sections now placed
- 0 teacher conflicts, 0 room double-bookings
- 3 anchor fallbacks persist (LEO I, LEO II, Gr11) due to co-schedule required periods
- 1 consecutive-6 violation: Daniels S1 (A-F, free=G)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -4480,7 +4480,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -6049,19 +6049,19 @@
         <v>845</v>
       </c>
       <c r="M75" s="3" t="n">
-        <v>5260</v>
+        <v>5270</v>
       </c>
       <c r="N75" s="3" t="n">
-        <v>6255</v>
+        <v>6265</v>
       </c>
       <c r="O75" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P75" s="3" t="n">
-        <v>7250</v>
+        <v>7260</v>
       </c>
       <c r="Q75" s="3" t="n">
-        <v>6305</v>
+        <v>6315</v>
       </c>
       <c r="R75" s="3" t="n">
         <v>28</v>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -6123,19 +6123,19 @@
         <v>845</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>5270</v>
+        <v>5280</v>
       </c>
       <c r="N76" s="3" t="n">
-        <v>6265</v>
+        <v>6275</v>
       </c>
       <c r="O76" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P76" s="3" t="n">
-        <v>7260</v>
+        <v>7270</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>6315</v>
+        <v>6325</v>
       </c>
       <c r="R76" s="3" t="n">
         <v>28</v>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6197,19 +6197,19 @@
         <v>845</v>
       </c>
       <c r="M77" s="3" t="n">
-        <v>5270</v>
+        <v>5290</v>
       </c>
       <c r="N77" s="3" t="n">
-        <v>6265</v>
+        <v>6285</v>
       </c>
       <c r="O77" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P77" s="3" t="n">
-        <v>7260</v>
+        <v>7280</v>
       </c>
       <c r="Q77" s="3" t="n">
-        <v>6315</v>
+        <v>6335</v>
       </c>
       <c r="R77" s="3" t="n">
         <v>28</v>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -6271,19 +6271,19 @@
         <v>845</v>
       </c>
       <c r="M78" s="3" t="n">
-        <v>5270</v>
+        <v>5300</v>
       </c>
       <c r="N78" s="3" t="n">
-        <v>6265</v>
+        <v>6295</v>
       </c>
       <c r="O78" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P78" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q78" s="3" t="n">
-        <v>6315</v>
+        <v>6345</v>
       </c>
       <c r="R78" s="3" t="n">
         <v>28</v>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -6922,7 +6922,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7070,7 +7070,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7588,7 +7588,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7662,7 +7662,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -7810,7 +7810,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -9068,7 +9068,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9512,7 +9512,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10178,7 +10178,7 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -10252,7 +10252,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11288,7 +11288,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11954,7 +11954,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -12028,7 +12028,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12398,7 +12398,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12546,7 +12546,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12620,7 +12620,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12842,7 +12842,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13434,7 +13434,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13730,7 +13730,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -13878,7 +13878,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -13952,7 +13952,7 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14248,7 +14248,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14692,7 +14692,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15432,7 +15432,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15506,7 +15506,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15580,7 +15580,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16024,7 +16024,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16172,7 +16172,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16542,7 +16542,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17356,7 +17356,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17652,7 +17652,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17948,7 +17948,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18096,7 +18096,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18318,7 +18318,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18614,7 +18614,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18836,7 +18836,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18910,7 +18910,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18984,7 +18984,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19280,7 +19280,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19428,7 +19428,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19576,7 +19576,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19650,7 +19650,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20020,7 +20020,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20242,7 +20242,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20834,7 +20834,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20982,7 +20982,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21278,7 +21278,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21352,7 +21352,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21574,7 +21574,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21722,7 +21722,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22240,7 +22240,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22388,7 +22388,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22462,7 +22462,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -22610,7 +22610,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22684,7 +22684,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22832,7 +22832,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -22906,7 +22906,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -24482,7 +24482,7 @@
         <v>150</v>
       </c>
       <c r="P324" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q324" s="3" t="inlineStr"/>
       <c r="R324" s="3" t="n">
@@ -24552,7 +24552,7 @@
         <v>150</v>
       </c>
       <c r="P325" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q325" s="3" t="inlineStr"/>
       <c r="R325" s="3" t="n">
@@ -24622,7 +24622,7 @@
         <v>150</v>
       </c>
       <c r="P326" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q326" s="3" t="inlineStr"/>
       <c r="R326" s="3" t="n">
@@ -24692,7 +24692,7 @@
         <v>150</v>
       </c>
       <c r="P327" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q327" s="3" t="inlineStr"/>
       <c r="R327" s="3" t="n">
@@ -24762,7 +24762,7 @@
         <v>150</v>
       </c>
       <c r="P328" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q328" s="3" t="inlineStr"/>
       <c r="R328" s="3" t="n">
@@ -24832,7 +24832,7 @@
         <v>150</v>
       </c>
       <c r="P329" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q329" s="3" t="inlineStr"/>
       <c r="R329" s="3" t="n">
@@ -24902,7 +24902,7 @@
         <v>150</v>
       </c>
       <c r="P330" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q330" s="3" t="inlineStr"/>
       <c r="R330" s="3" t="n">
@@ -24972,7 +24972,7 @@
         <v>150</v>
       </c>
       <c r="P331" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q331" s="3" t="inlineStr"/>
       <c r="R331" s="3" t="n">
@@ -25042,7 +25042,7 @@
         <v>150</v>
       </c>
       <c r="P332" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q332" s="3" t="inlineStr"/>
       <c r="R332" s="3" t="n">
@@ -25112,7 +25112,7 @@
         <v>150</v>
       </c>
       <c r="P333" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q333" s="3" t="inlineStr"/>
       <c r="R333" s="3" t="n">
@@ -25182,7 +25182,7 @@
         <v>150</v>
       </c>
       <c r="P334" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q334" s="3" t="inlineStr"/>
       <c r="R334" s="3" t="n">
@@ -25252,7 +25252,7 @@
         <v>150</v>
       </c>
       <c r="P335" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q335" s="3" t="inlineStr"/>
       <c r="R335" s="3" t="n">
@@ -25322,7 +25322,7 @@
         <v>150</v>
       </c>
       <c r="P336" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q336" s="3" t="inlineStr"/>
       <c r="R336" s="3" t="n">
@@ -25392,7 +25392,7 @@
         <v>150</v>
       </c>
       <c r="P337" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q337" s="3" t="inlineStr"/>
       <c r="R337" s="3" t="n">
@@ -25462,7 +25462,7 @@
         <v>150</v>
       </c>
       <c r="P338" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q338" s="3" t="inlineStr"/>
       <c r="R338" s="3" t="n">
@@ -25532,7 +25532,7 @@
         <v>150</v>
       </c>
       <c r="P339" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q339" s="3" t="inlineStr"/>
       <c r="R339" s="3" t="n">
@@ -25602,7 +25602,7 @@
         <v>150</v>
       </c>
       <c r="P340" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q340" s="3" t="inlineStr"/>
       <c r="R340" s="3" t="n">
@@ -25672,7 +25672,7 @@
         <v>150</v>
       </c>
       <c r="P341" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q341" s="3" t="inlineStr"/>
       <c r="R341" s="3" t="n">
@@ -25718,7 +25718,7 @@
       </c>
       <c r="I342" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J342" s="2" t="inlineStr">
@@ -25733,16 +25733,16 @@
         <v>640</v>
       </c>
       <c r="M342" s="3" t="n">
-        <v>5270</v>
+        <v>5300</v>
       </c>
       <c r="N342" s="3" t="n">
-        <v>6265</v>
+        <v>6295</v>
       </c>
       <c r="O342" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P342" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q342" s="3" t="inlineStr"/>
       <c r="R342" s="3" t="n">
@@ -25788,7 +25788,7 @@
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J343" s="2" t="inlineStr">
@@ -25803,16 +25803,16 @@
         <v>640</v>
       </c>
       <c r="M343" s="3" t="n">
-        <v>5270</v>
+        <v>5300</v>
       </c>
       <c r="N343" s="3" t="n">
-        <v>6265</v>
+        <v>6295</v>
       </c>
       <c r="O343" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P343" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q343" s="3" t="inlineStr"/>
       <c r="R343" s="3" t="n">
@@ -25858,7 +25858,7 @@
       </c>
       <c r="I344" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J344" s="2" t="inlineStr">
@@ -25873,16 +25873,16 @@
         <v>640</v>
       </c>
       <c r="M344" s="3" t="n">
-        <v>5270</v>
+        <v>5300</v>
       </c>
       <c r="N344" s="3" t="n">
-        <v>6265</v>
+        <v>6295</v>
       </c>
       <c r="O344" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P344" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q344" s="3" t="inlineStr"/>
       <c r="R344" s="3" t="n">
@@ -25943,16 +25943,16 @@
         <v>640</v>
       </c>
       <c r="M345" s="3" t="n">
-        <v>5270</v>
+        <v>5300</v>
       </c>
       <c r="N345" s="3" t="n">
-        <v>6265</v>
+        <v>6295</v>
       </c>
       <c r="O345" s="3" t="n">
         <v>150</v>
       </c>
       <c r="P345" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q345" s="3" t="inlineStr"/>
       <c r="R345" s="3" t="n">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
@@ -26022,7 +26022,7 @@
         <v>150</v>
       </c>
       <c r="P346" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q346" s="3" t="inlineStr"/>
       <c r="R346" s="3" t="n">
@@ -26092,7 +26092,7 @@
         <v>150</v>
       </c>
       <c r="P347" s="3" t="n">
-        <v>7260</v>
+        <v>7290</v>
       </c>
       <c r="Q347" s="3" t="inlineStr"/>
       <c r="R347" s="3" t="n">
@@ -26278,7 +26278,7 @@
       </c>
       <c r="I350" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J350" s="2" t="inlineStr">
@@ -26352,7 +26352,7 @@
       </c>
       <c r="I351" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J351" s="2" t="inlineStr">
@@ -27639,16 +27639,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
@@ -27664,10 +27664,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
@@ -27677,16 +27677,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>7</v>
-      </c>
       <c r="D4" s="3" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -27696,13 +27696,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>53</v>
@@ -27715,16 +27715,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -27734,16 +27734,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>6</v>
-      </c>
       <c r="D7" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -27753,16 +27753,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>6</v>
-      </c>
       <c r="D8" s="3" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -28164,27 +28164,27 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>3/5</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
           <t>4/5</t>
         </is>
       </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>6/5</t>
+        </is>
+      </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>10/15</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Standard</t>
+          <t>14/15</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>50% FY Stipend</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
@@ -31537,7 +31537,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3">
@@ -31547,7 +31547,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -31577,7 +31577,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -31598,7 +31598,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>155/345</t>
+          <t>160/345</t>
         </is>
       </c>
     </row>
@@ -31621,7 +31621,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -31631,7 +31631,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13">
@@ -31641,7 +31641,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14">
@@ -31661,7 +31661,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -31671,7 +31671,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Job 1 output: section numbers now match T7 Column 7 (B19 fix verified)
Results:
- 367/367 sections placed (100%)
- 0 prescribed term violations (all S1/S2/FY/EC correct)
- 0 section number mismatches vs T7
- 0 teacher conflicts, 0 room double-bookings, 0 load violations
- 1 consecutive-6 violation: Daniels S1 (A-F, free=G)
- Period distribution: A=61, B=52, C=54, D=53, E=46, F=54, G=47

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -7712,7 +7712,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
@@ -7786,7 +7786,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
@@ -9932,7 +9932,7 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
@@ -10006,7 +10006,7 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
@@ -10968,7 +10968,7 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
@@ -11042,7 +11042,7 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
@@ -11116,7 +11116,7 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
@@ -11190,7 +11190,7 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
@@ -11486,7 +11486,7 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
@@ -11939,17 +11939,17 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>Gerlach, Reese</t>
+          <t>Hampson, Elizabeth</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>107125</t>
+          <t>105669</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>D-107</t>
+          <t>D-108</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr">
@@ -11972,13 +11972,13 @@
         <v>80</v>
       </c>
       <c r="N155" s="3" t="n">
-        <v>1015</v>
+        <v>920</v>
       </c>
       <c r="O155" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P155" s="3" t="n">
-        <v>1950</v>
+        <v>1760</v>
       </c>
       <c r="Q155" s="3" t="n">
         <v>785</v>
@@ -12028,7 +12028,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12043,19 +12043,19 @@
         <v>650</v>
       </c>
       <c r="M156" s="3" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="N156" s="3" t="n">
-        <v>920</v>
+        <v>930</v>
       </c>
       <c r="O156" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P156" s="3" t="n">
-        <v>1760</v>
+        <v>1770</v>
       </c>
       <c r="Q156" s="3" t="n">
-        <v>785</v>
+        <v>795</v>
       </c>
       <c r="R156" s="3" t="n">
         <v>28</v>
@@ -12102,7 +12102,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12117,19 +12117,19 @@
         <v>650</v>
       </c>
       <c r="M157" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N157" s="3" t="n">
-        <v>930</v>
+        <v>940</v>
       </c>
       <c r="O157" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P157" s="3" t="n">
-        <v>1770</v>
+        <v>1780</v>
       </c>
       <c r="Q157" s="3" t="n">
-        <v>795</v>
+        <v>805</v>
       </c>
       <c r="R157" s="3" t="n">
         <v>28</v>
@@ -12161,22 +12161,22 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>Hampson, Elizabeth</t>
+          <t>Gerlach, Reese</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>105669</t>
+          <t>107125</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>D-108</t>
+          <t>D-107</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12191,19 +12191,19 @@
         <v>650</v>
       </c>
       <c r="M158" s="3" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="N158" s="3" t="n">
-        <v>940</v>
+        <v>1015</v>
       </c>
       <c r="O158" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P158" s="3" t="n">
-        <v>1780</v>
+        <v>1950</v>
       </c>
       <c r="Q158" s="3" t="n">
-        <v>805</v>
+        <v>785</v>
       </c>
       <c r="R158" s="3" t="n">
         <v>28</v>
@@ -12670,7 +12670,7 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
@@ -12744,7 +12744,7 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
@@ -12753,17 +12753,17 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>Langan, John</t>
+          <t>Ojo, Clement</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>111895</t>
+          <t>105624</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>J-323</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="I166" s="2" t="inlineStr">
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
@@ -12827,17 +12827,17 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>Langan, John</t>
+          <t>Ojo, Clement</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>111895</t>
+          <t>105624</t>
         </is>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>J-323</t>
+          <t>J-221</t>
         </is>
       </c>
       <c r="I167" s="2" t="inlineStr">
@@ -12892,7 +12892,7 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
@@ -12916,7 +12916,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -12931,19 +12931,19 @@
         <v>640</v>
       </c>
       <c r="M168" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="N168" s="3" t="n">
-        <v>725</v>
+        <v>745</v>
       </c>
       <c r="O168" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P168" s="3" t="n">
-        <v>1390</v>
+        <v>1410</v>
       </c>
       <c r="Q168" s="3" t="n">
-        <v>755</v>
+        <v>775</v>
       </c>
       <c r="R168" s="3" t="n">
         <v>28</v>
@@ -12966,7 +12966,7 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
@@ -12990,7 +12990,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13005,19 +13005,19 @@
         <v>640</v>
       </c>
       <c r="M169" s="3" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="N169" s="3" t="n">
-        <v>735</v>
+        <v>755</v>
       </c>
       <c r="O169" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P169" s="3" t="n">
-        <v>1400</v>
+        <v>1420</v>
       </c>
       <c r="Q169" s="3" t="n">
-        <v>765</v>
+        <v>785</v>
       </c>
       <c r="R169" s="3" t="n">
         <v>28</v>
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
@@ -13064,7 +13064,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13079,19 +13079,19 @@
         <v>640</v>
       </c>
       <c r="M170" s="3" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="N170" s="3" t="n">
-        <v>745</v>
+        <v>765</v>
       </c>
       <c r="O170" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P170" s="3" t="n">
-        <v>1410</v>
+        <v>1430</v>
       </c>
       <c r="Q170" s="3" t="n">
-        <v>775</v>
+        <v>795</v>
       </c>
       <c r="R170" s="3" t="n">
         <v>28</v>
@@ -13114,7 +13114,7 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
@@ -13123,22 +13123,22 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>Ojo, Clement</t>
+          <t>Langan, John</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>105624</t>
+          <t>111895</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>J-323</t>
         </is>
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13153,19 +13153,19 @@
         <v>640</v>
       </c>
       <c r="M171" s="3" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="N171" s="3" t="n">
-        <v>755</v>
+        <v>725</v>
       </c>
       <c r="O171" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P171" s="3" t="n">
-        <v>1420</v>
+        <v>1390</v>
       </c>
       <c r="Q171" s="3" t="n">
-        <v>785</v>
+        <v>755</v>
       </c>
       <c r="R171" s="3" t="n">
         <v>28</v>
@@ -13188,7 +13188,7 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
@@ -13197,22 +13197,22 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>Ojo, Clement</t>
+          <t>Langan, John</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>105624</t>
+          <t>111895</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>J-221</t>
+          <t>J-323</t>
         </is>
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13227,19 +13227,19 @@
         <v>640</v>
       </c>
       <c r="M172" s="3" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="N172" s="3" t="n">
-        <v>765</v>
+        <v>735</v>
       </c>
       <c r="O172" s="3" t="n">
         <v>25</v>
       </c>
       <c r="P172" s="3" t="n">
-        <v>1430</v>
+        <v>1400</v>
       </c>
       <c r="Q172" s="3" t="n">
-        <v>795</v>
+        <v>765</v>
       </c>
       <c r="R172" s="3" t="n">
         <v>28</v>
@@ -13928,7 +13928,7 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
@@ -14002,7 +14002,7 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
@@ -14076,7 +14076,7 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
@@ -14742,7 +14742,7 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
@@ -14816,7 +14816,7 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
@@ -14890,7 +14890,7 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
@@ -14964,7 +14964,7 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
@@ -15778,7 +15778,7 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
@@ -16296,7 +16296,7 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
@@ -16370,7 +16370,7 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
@@ -16444,7 +16444,7 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
@@ -16740,7 +16740,7 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
@@ -16814,7 +16814,7 @@
         </is>
       </c>
       <c r="D221" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
@@ -17406,7 +17406,7 @@
         </is>
       </c>
       <c r="D229" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
@@ -17480,7 +17480,7 @@
         </is>
       </c>
       <c r="D230" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
@@ -18220,7 +18220,7 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
@@ -18368,7 +18368,7 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
@@ -18516,7 +18516,7 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
@@ -18590,7 +18590,7 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
@@ -18812,7 +18812,7 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
@@ -18886,7 +18886,7 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
@@ -19700,7 +19700,7 @@
         </is>
       </c>
       <c r="D260" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D261" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
@@ -20662,7 +20662,7 @@
         </is>
       </c>
       <c r="D273" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
@@ -20736,7 +20736,7 @@
         </is>
       </c>
       <c r="D274" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         </is>
       </c>
       <c r="D275" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
@@ -21254,7 +21254,7 @@
         </is>
       </c>
       <c r="D281" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
@@ -21328,7 +21328,7 @@
         </is>
       </c>
       <c r="D282" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
@@ -21402,7 +21402,7 @@
         </is>
       </c>
       <c r="D283" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E283" s="2" t="inlineStr">
         <is>
@@ -21476,7 +21476,7 @@
         </is>
       </c>
       <c r="D284" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
@@ -21550,7 +21550,7 @@
         </is>
       </c>
       <c r="D285" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E285" s="2" t="inlineStr">
         <is>
@@ -21624,7 +21624,7 @@
         </is>
       </c>
       <c r="D286" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
@@ -21633,12 +21633,12 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>Hartmann, Katy</t>
+          <t>Oh, Burton</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>115019</t>
+          <t>122121</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
@@ -21698,7 +21698,7 @@
         </is>
       </c>
       <c r="D287" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
@@ -21707,12 +21707,12 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>Hartmann, Katy</t>
+          <t>Oh, Burton</t>
         </is>
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>115019</t>
+          <t>122121</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr">
@@ -21772,7 +21772,7 @@
         </is>
       </c>
       <c r="D288" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
@@ -21781,12 +21781,12 @@
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>Oh, Burton</t>
+          <t>Hartmann, Katy</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>122121</t>
+          <t>115019</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
@@ -21846,7 +21846,7 @@
         </is>
       </c>
       <c r="D289" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
@@ -21855,12 +21855,12 @@
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>Oh, Burton</t>
+          <t>Hartmann, Katy</t>
         </is>
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>122121</t>
+          <t>115019</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
@@ -21920,7 +21920,7 @@
         </is>
       </c>
       <c r="D290" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
@@ -21994,7 +21994,7 @@
         </is>
       </c>
       <c r="D291" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
@@ -22068,7 +22068,7 @@
         </is>
       </c>
       <c r="D292" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
@@ -22142,7 +22142,7 @@
         </is>
       </c>
       <c r="D293" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E293" s="2" t="inlineStr">
         <is>
@@ -22216,7 +22216,7 @@
         </is>
       </c>
       <c r="D294" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
@@ -22290,7 +22290,7 @@
         </is>
       </c>
       <c r="D295" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E295" s="2" t="inlineStr">
         <is>
@@ -22364,7 +22364,7 @@
         </is>
       </c>
       <c r="D296" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
@@ -22438,7 +22438,7 @@
         </is>
       </c>
       <c r="D297" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
@@ -22512,7 +22512,7 @@
         </is>
       </c>
       <c r="D298" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
@@ -22586,7 +22586,7 @@
         </is>
       </c>
       <c r="D299" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
@@ -22610,7 +22610,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22660,7 +22660,7 @@
         </is>
       </c>
       <c r="D300" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
@@ -22684,7 +22684,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -22758,7 +22758,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -25694,7 +25694,7 @@
         </is>
       </c>
       <c r="D342" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E342" s="2" t="inlineStr">
         <is>
@@ -25764,7 +25764,7 @@
         </is>
       </c>
       <c r="D343" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E343" s="2" t="inlineStr">
         <is>
@@ -25834,7 +25834,7 @@
         </is>
       </c>
       <c r="D344" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E344" s="2" t="inlineStr">
         <is>
@@ -25904,7 +25904,7 @@
         </is>
       </c>
       <c r="D345" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E345" s="2" t="inlineStr">
         <is>
@@ -25974,7 +25974,7 @@
         </is>
       </c>
       <c r="D346" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E346" s="2" t="inlineStr">
         <is>
@@ -26044,7 +26044,7 @@
         </is>
       </c>
       <c r="D347" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E347" s="2" t="inlineStr">
         <is>
@@ -27683,10 +27683,10 @@
         <v>8</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -27740,10 +27740,10 @@
         <v>8</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -31598,7 +31598,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>160/345</t>
+          <t>161/345</t>
         </is>
       </c>
     </row>
@@ -31641,7 +31641,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14">
@@ -31671,7 +31671,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Job 1 output: 367/367 placed, 0 violations — after PE teacher 5/5 balance fix
Clean run after T7 prescribed term changes:
- 367/367 sections placed
- 0 teacher conflicts, 0 room double-bookings
- 0 load violations, 0 consecutive-6 violations
- Biggs 5/5, Chiaravalloti 5/5, Daniels 5/5 confirmed

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -5886,7 +5886,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6256,7 +6256,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -6922,7 +6922,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -9512,7 +9512,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11288,7 +11288,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12398,7 +12398,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -12546,7 +12546,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -12620,7 +12620,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12916,7 +12916,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13434,7 +13434,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -13730,7 +13730,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14692,7 +14692,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15432,7 +15432,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15580,7 +15580,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15728,7 +15728,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -16024,7 +16024,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16172,7 +16172,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16320,7 +16320,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16764,7 +16764,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17208,7 +17208,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17652,7 +17652,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18096,7 +18096,7 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18318,7 +18318,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18392,7 +18392,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18540,7 +18540,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18614,7 +18614,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18836,7 +18836,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18910,7 +18910,7 @@
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -18984,7 +18984,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19428,7 +19428,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20982,7 +20982,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21352,7 +21352,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21574,7 +21574,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21944,7 +21944,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22388,7 +22388,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22462,7 +22462,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -25863,7 +25863,7 @@
       </c>
       <c r="J344" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K344" s="3" t="n">
@@ -25928,7 +25928,7 @@
       </c>
       <c r="I345" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J345" s="2" t="inlineStr">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
@@ -26073,7 +26073,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="K347" s="3" t="n">
@@ -27639,16 +27639,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>12</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -27661,10 +27661,10 @@
         <v>10</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>52</v>
@@ -27677,16 +27677,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
@@ -27696,16 +27696,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -27715,16 +27715,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -27734,13 +27734,13 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>54</v>
@@ -27756,13 +27756,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -28164,27 +28164,27 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>6/5</t>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>14/15</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>50% FY Stipend</t>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
@@ -28296,27 +28296,27 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>6/5</t>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>14/15</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>50% FY Stipend</t>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H12" s="3" t="n">
@@ -31598,7 +31598,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>161/345</t>
+          <t>155/345</t>
         </is>
       </c>
     </row>
@@ -31621,7 +31621,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12">
@@ -31641,7 +31641,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14">
@@ -31651,7 +31651,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
@@ -31661,7 +31661,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix EC rebalance: count co-schedule groups as 1 period slot, not N raw sections
Bug: _teacher_aware_ec_rebalance() counted raw sections per semester.
McConnell's Robotics Block co-schedule (590x2 + 591x2 = 4 raw S1 sections)
occupies only 1 period. Function saw S1=8, thought it was over cap(6),
and aggressively flipped 2 EC sections to S2 — creating S2=6 with no
room for 570 Introduction to Robotics Sec#2.

Fix: Count unique period slots per semester. Co-schedule group members
sharing one period count as 1 slot. McConnell now correctly reads
S1=5 periods (1 co-sched + 4 EC), S2=4 periods — both under cap,
no flipping needed, leaving room for 570.

Same class as Bug B9 (cross-course consolidation) — co-schedule groups
must be counted as one unit wherever period occupancy matters.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1002,7 +1002,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -3222,12 +3222,12 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K37" s="3" t="n">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -4480,7 +4480,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7297,7 +7297,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K92" s="3" t="n">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7884,12 +7884,12 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K100" s="3" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>UNSCHEDULED</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -7973,19 +7973,19 @@
         <v>495</v>
       </c>
       <c r="M101" s="3" t="n">
-        <v>5210</v>
+        <v>5220</v>
       </c>
       <c r="N101" s="3" t="n">
-        <v>6015</v>
+        <v>6025</v>
       </c>
       <c r="O101" s="3" t="n">
         <v>60</v>
       </c>
       <c r="P101" s="3" t="n">
-        <v>6820</v>
+        <v>6830</v>
       </c>
       <c r="Q101" s="3" t="n">
-        <v>5775</v>
+        <v>5785</v>
       </c>
       <c r="R101" s="3" t="n">
         <v>28</v>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9068,7 +9068,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9216,7 +9216,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11584,7 +11584,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11732,7 +11732,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -12028,7 +12028,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12250,7 +12250,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12620,7 +12620,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12842,7 +12842,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13582,7 +13582,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13878,7 +13878,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14248,7 +14248,7 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15432,7 +15432,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15506,7 +15506,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16172,7 +16172,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16468,7 +16468,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16764,7 +16764,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17356,7 +17356,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17652,7 +17652,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17800,7 +17800,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -18244,7 +18244,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -18318,7 +18318,7 @@
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -18392,7 +18392,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18466,7 +18466,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18540,7 +18540,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19280,7 +19280,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19428,7 +19428,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19576,7 +19576,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19650,7 +19650,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20020,7 +20020,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20390,7 +20390,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="I272" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21574,7 +21574,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21648,7 +21648,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21944,7 +21944,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22240,7 +22240,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22388,7 +22388,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22610,7 +22610,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -23131,7 +23131,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="K306" s="3" t="n">
@@ -23881,16 +23881,16 @@
         <v>745</v>
       </c>
       <c r="M316" s="3" t="n">
-        <v>5210</v>
+        <v>5220</v>
       </c>
       <c r="N316" s="3" t="n">
-        <v>6015</v>
+        <v>6025</v>
       </c>
       <c r="O316" s="3" t="n">
         <v>60</v>
       </c>
       <c r="P316" s="3" t="n">
-        <v>6820</v>
+        <v>6830</v>
       </c>
       <c r="Q316" s="3" t="inlineStr"/>
       <c r="R316" s="3" t="n">
@@ -23955,16 +23955,16 @@
         <v>745</v>
       </c>
       <c r="M317" s="3" t="n">
-        <v>5210</v>
+        <v>5220</v>
       </c>
       <c r="N317" s="3" t="n">
-        <v>6015</v>
+        <v>6025</v>
       </c>
       <c r="O317" s="3" t="n">
         <v>60</v>
       </c>
       <c r="P317" s="3" t="n">
-        <v>6820</v>
+        <v>6830</v>
       </c>
       <c r="Q317" s="3" t="inlineStr"/>
       <c r="R317" s="3" t="n">
@@ -24029,16 +24029,16 @@
         <v>745</v>
       </c>
       <c r="M318" s="3" t="n">
-        <v>5210</v>
+        <v>5220</v>
       </c>
       <c r="N318" s="3" t="n">
-        <v>6015</v>
+        <v>6025</v>
       </c>
       <c r="O318" s="3" t="n">
         <v>60</v>
       </c>
       <c r="P318" s="3" t="n">
-        <v>6820</v>
+        <v>6830</v>
       </c>
       <c r="Q318" s="3" t="inlineStr"/>
       <c r="R318" s="3" t="n">
@@ -24103,16 +24103,16 @@
         <v>745</v>
       </c>
       <c r="M319" s="3" t="n">
-        <v>5210</v>
+        <v>5220</v>
       </c>
       <c r="N319" s="3" t="n">
-        <v>6015</v>
+        <v>6025</v>
       </c>
       <c r="O319" s="3" t="n">
         <v>60</v>
       </c>
       <c r="P319" s="3" t="n">
-        <v>6820</v>
+        <v>6830</v>
       </c>
       <c r="Q319" s="3" t="inlineStr"/>
       <c r="R319" s="3" t="n">
@@ -27623,13 +27623,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>54</v>
@@ -27645,13 +27645,13 @@
         <v>10</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -27664,13 +27664,13 @@
         <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>39</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -27680,16 +27680,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>6</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -27699,16 +27699,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -27718,16 +27718,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -27740,13 +27740,13 @@
         <v>9</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -28412,22 +28412,22 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>9/15</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -29556,22 +29556,22 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>11/15</t>
+          <t>13/15</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -30611,7 +30611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -30886,7 +30886,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -30896,12 +30896,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>253-1</t>
+          <t>242-1</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>254-1</t>
+          <t>243-1</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>255-1</t>
+          <t>254-1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -30965,7 +30965,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>764-1</t>
+          <t>255-1</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -30992,12 +30992,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>254-1</t>
+          <t>253-1</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>255-1</t>
+          <t>764-1</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -31029,7 +31029,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>764-1</t>
+          <t>255-1</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -31056,7 +31056,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>255-1</t>
+          <t>254-1</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -31083,17 +31083,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>253-1</t>
+          <t>255-1</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>254-1</t>
+          <t>764-1</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -31125,7 +31125,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>255-1</t>
+          <t>254-1</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -31157,7 +31157,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>764-1</t>
+          <t>255-1</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -31184,12 +31184,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>254-1</t>
+          <t>253-1</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>255-1</t>
+          <t>764-1</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -31221,7 +31221,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>764-1</t>
+          <t>255-1</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -31248,7 +31248,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>255-1</t>
+          <t>254-1</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -31265,27 +31265,27 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Calidas, Riddhi</t>
+          <t>Dennehy, Sheri</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>473-1</t>
+          <t>255-1</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>494-1</t>
+          <t>764-1</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -31297,12 +31297,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>McConnell, George</t>
+          <t>Calidas, Riddhi</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -31312,12 +31312,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>590-1</t>
+          <t>473-1</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>590-2</t>
+          <t>494-1</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -31349,7 +31349,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>591-1</t>
+          <t>590-2</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -31381,7 +31381,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>591-2</t>
+          <t>591-1</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -31408,12 +31408,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>590-2</t>
+          <t>590-1</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>591-1</t>
+          <t>591-2</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -31445,7 +31445,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>591-2</t>
+          <t>591-1</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -31472,15 +31472,47 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t>590-2</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>591-2</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>McConnell, George</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
           <t>591-1</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>591-2</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -31521,7 +31553,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3">
@@ -31531,7 +31563,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -31582,7 +31614,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>154/345</t>
+          <t>152/345</t>
         </is>
       </c>
     </row>
@@ -31615,7 +31647,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13">
@@ -31625,7 +31657,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14">
@@ -31635,7 +31667,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
@@ -31645,7 +31677,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -31655,7 +31687,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
@@ -31665,7 +31697,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
In-progress output from second full run (cross-run learning adaptation)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1372,7 +1372,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11288,7 +11288,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11584,7 +11584,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11732,7 +11732,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12250,7 +12250,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13582,7 +13582,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -13878,7 +13878,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -14914,7 +14914,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15506,7 +15506,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16172,7 +16172,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16468,7 +16468,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17208,7 +17208,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17356,7 +17356,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17652,7 +17652,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17948,7 +17948,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18466,7 +18466,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18540,7 +18540,7 @@
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -18614,7 +18614,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19280,7 +19280,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19576,7 +19576,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20242,7 +20242,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20390,7 +20390,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20834,7 +20834,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20982,7 +20982,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21574,7 +21574,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -21648,7 +21648,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21722,7 +21722,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21796,7 +21796,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22388,7 +22388,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -22610,7 +22610,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -27626,13 +27626,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>34</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -27645,13 +27645,13 @@
         <v>10</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -27667,10 +27667,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -27686,10 +27686,10 @@
         <v>6</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
@@ -27699,16 +27699,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>10</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -27721,13 +27721,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
@@ -27737,16 +27737,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -31614,7 +31614,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>152/345</t>
+          <t>147/345</t>
         </is>
       </c>
     </row>
@@ -31637,7 +31637,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -31647,7 +31647,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13">
@@ -31657,7 +31657,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14">
@@ -31667,7 +31667,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -31677,7 +31677,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
@@ -31687,7 +31687,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17">
@@ -31697,7 +31697,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Full run #4: 875 conflicts, 366/366 placed, 86.6% placement rate
Cross-run learning oscillating after layout change (844→857→875).
Biases may be oversteering. All 366 sections placed.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -1298,7 +1298,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9512,7 +9512,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11288,7 +11288,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14766,7 +14766,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14914,7 +14914,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15432,7 +15432,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15580,7 +15580,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -16024,7 +16024,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16172,7 +16172,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16320,7 +16320,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16542,7 +16542,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16764,7 +16764,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17356,7 +17356,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17800,7 +17800,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -17948,7 +17948,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18392,7 +18392,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18466,7 +18466,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18836,7 +18836,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19280,7 +19280,7 @@
       </c>
       <c r="I254" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I255" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19650,7 +19650,7 @@
       </c>
       <c r="I259" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20390,7 +20390,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20834,7 +20834,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21352,7 +21352,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21648,7 +21648,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21722,7 +21722,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21796,7 +21796,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -21944,7 +21944,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22240,7 +22240,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -27555,10 +27555,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
@@ -27571,13 +27571,13 @@
         <v>9</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -27593,10 +27593,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -27609,13 +27609,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
@@ -27625,16 +27625,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>12</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
@@ -27647,13 +27647,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -27663,16 +27663,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -31540,7 +31540,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>154/345</t>
+          <t>151/345</t>
         </is>
       </c>
     </row>
@@ -31563,7 +31563,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
@@ -31573,7 +31573,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -31583,7 +31583,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14">
@@ -31593,7 +31593,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -31603,7 +31603,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
@@ -31613,7 +31613,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -31623,7 +31623,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Full runs #5-8: cross-run learning oscillating 868-905 range
Clean baseline without biases: 895. With biases oscillating between
868-905. Pattern: even runs improve, odd runs regress. All 366/366
sections placed on best seeds. Cross-run learning needs investigation.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -2926,7 +2926,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -7810,7 +7810,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9512,7 +9512,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11510,7 +11510,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14766,7 +14766,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14914,7 +14914,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -15432,7 +15432,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
@@ -15580,7 +15580,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15728,7 +15728,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15802,7 +15802,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -16024,7 +16024,7 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -16320,7 +16320,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16542,7 +16542,7 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16764,7 +16764,7 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -17356,7 +17356,7 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17652,7 +17652,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17800,7 +17800,7 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18392,7 +18392,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18466,7 +18466,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18614,7 +18614,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18836,7 +18836,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18984,7 +18984,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19428,7 +19428,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -19576,7 +19576,7 @@
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -19798,7 +19798,7 @@
       </c>
       <c r="I261" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -20020,7 +20020,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20242,7 +20242,7 @@
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20390,7 +20390,7 @@
       </c>
       <c r="I269" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20834,7 +20834,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20982,7 +20982,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -21648,7 +21648,7 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -21722,7 +21722,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21796,7 +21796,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -22536,7 +22536,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -27549,16 +27549,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -27571,10 +27571,10 @@
         <v>9</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>56</v>
@@ -27593,10 +27593,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -27612,10 +27612,10 @@
         <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -27625,16 +27625,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7">
@@ -27647,13 +27647,13 @@
         <v>12</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -27669,10 +27669,10 @@
         <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -31540,7 +31540,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>151/345</t>
+          <t>152/345</t>
         </is>
       </c>
     </row>
@@ -31563,7 +31563,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -31583,7 +31583,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14">
@@ -31593,7 +31593,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15">
@@ -31603,7 +31603,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16">
@@ -31613,7 +31613,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -31623,7 +31623,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add engine output files from full run (862 conflicts, seed 1337)
- Job1_Section_Placements_2026_27.xlsx: Section placements (365 placed, 1 unplaced)
- Job2_Student_Placements_2026_27.xlsx: Student placements (86.8% rate, 862 conflicts)
- Preflight_Validation_Report.xlsx: Pre-run validation
- run_diagnostics.json: Phase A-1 analysis (for review only, biases disabled)
- priority_audit_log.json: Per-placement priority audit trail
- schedule_solution_v3.json: Full solution data

Engine ran with 3 fixes applied (commit f91790f):
1. Cross-run learning disabled (eliminated oscillation)
2. Post-greedy cleanup pass (34-46 sections moved per seed)
3. Phase D search widened (24 candidates, 12 stall, 80 iterations)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6626,7 +6626,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7070,7 +7070,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -7810,7 +7810,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11510,7 +11510,7 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -11732,7 +11732,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -12842,7 +12842,7 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -14766,7 +14766,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
@@ -14914,7 +14914,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
@@ -15580,7 +15580,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
@@ -15728,7 +15728,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -16172,7 +16172,7 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -16320,7 +16320,7 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -16468,7 +16468,7 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -17060,7 +17060,7 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr">
@@ -17208,7 +17208,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
@@ -17578,7 +17578,7 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -17652,7 +17652,7 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -18392,7 +18392,7 @@
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -18466,7 +18466,7 @@
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -18614,7 +18614,7 @@
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -18836,7 +18836,7 @@
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -18984,7 +18984,7 @@
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="I251" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="I252" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -19428,7 +19428,7 @@
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -20020,7 +20020,7 @@
       </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20834,7 +20834,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -20982,7 +20982,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21056,7 +21056,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21352,7 +21352,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -21722,7 +21722,7 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -21796,7 +21796,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -22536,7 +22536,7 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
@@ -27549,10 +27549,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>36</v>
@@ -27568,16 +27568,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>8</v>
-      </c>
       <c r="D3" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -27587,16 +27587,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -27606,16 +27606,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>58</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6">
@@ -27625,16 +27625,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
@@ -27644,7 +27644,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>9</v>
@@ -27653,7 +27653,7 @@
         <v>29</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -27663,16 +27663,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -31540,7 +31540,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>152/345</t>
+          <t>155/345</t>
         </is>
       </c>
     </row>
@@ -31573,7 +31573,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -31583,7 +31583,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
@@ -31593,7 +31593,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>58</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
@@ -31603,7 +31603,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16">
@@ -31613,7 +31613,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
@@ -31623,7 +31623,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Engine output: 833 conflicts (87.3%) — Period Rebalancing Phase reduces by 29
Results with Period Rebalancing Phase (Option B):
- Best seed: 54321, 833 conflicts (was 862, -29 = 3.4% reduction)
- Placement rate: 87.3% (was 86.8%)
- Grade breakdown: Gr9=198, Gr10=180, Gr11=179, Gr12=276
- Period rebalancing: 17-22 sections moved per seed across 11-13 courses
- 1 UNPLACED: 249 Adv Painting (Dennehy, structural)

Two seeds hit 805 (3141, 8888) but best overall was 54321 at 833.
Range: 805-920 across 16 seeds.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_2026_27.xlsx
+++ b/Job1_Section_Placements_2026_27.xlsx
@@ -9216,7 +9216,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -12546,7 +12546,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -17208,7 +17208,7 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -17948,7 +17948,7 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="I257" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr">
@@ -20464,7 +20464,7 @@
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -20760,7 +20760,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21278,7 +21278,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -21352,7 +21352,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -21574,7 +21574,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -27555,10 +27555,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -27574,10 +27574,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -27593,10 +27593,10 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
@@ -27612,10 +27612,10 @@
         <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -27631,10 +27631,10 @@
         <v>12</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -27650,10 +27650,10 @@
         <v>9</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
@@ -27669,10 +27669,10 @@
         <v>5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -31540,7 +31540,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>155/345</t>
+          <t>153/345</t>
         </is>
       </c>
     </row>
@@ -31563,7 +31563,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -31573,7 +31573,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13">
@@ -31583,7 +31583,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
@@ -31593,7 +31593,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15">
@@ -31603,7 +31603,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16">
@@ -31613,7 +31613,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17">
@@ -31623,7 +31623,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>